<commit_message>
docs(operations): link control review PR
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Items" sheetId="1" r:id="R87a2f1588dbb473b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Status" sheetId="2" r:id="R506823742c434c8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" r:id="R30ba41e25ce84092"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Work" sheetId="4" r:id="R1d0237a020fa47f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified" sheetId="5" r:id="R6b0a53eec7bd4be3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocked Deferred" sheetId="6" r:id="Rac48480db9534d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="7" r:id="R4b0143210d464e31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="8" r:id="Raa9bcbef170d4bf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="9" r:id="Re9a50618f7d94f77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="10" r:id="R833ea1d4f2b844fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Items" sheetId="1" r:id="R7f8fbb37bf4d4ffd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Status" sheetId="2" r:id="R84e9ec0666be456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" r:id="Re58125044a1e4101"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active Work" sheetId="4" r:id="Reb35f7eb20244a0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified" sheetId="5" r:id="R3970c6bec9604915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocked Deferred" sheetId="6" r:id="Rf108d14e61f54c04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="7" r:id="R85db85578ee2457a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reports" sheetId="8" r:id="R7afbfec6e021424a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Gates" sheetId="9" r:id="R033c4b77bd914d73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="10" r:id="Rf9f22c25ffb84002"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1719,8 +1719,9 @@
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="32" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="54" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2">
@@ -1731,6 +1732,7 @@
       <x:c r="C2" s="37"/>
       <x:c r="D2" s="37"/>
       <x:c r="E2" s="37"/>
+      <x:c r="F2" s="37"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="39" t="str">
@@ -1743,9 +1745,12 @@
         <x:v>الفرع</x:v>
       </x:c>
       <x:c r="D4" s="39" t="str">
+        <x:v>PR</x:v>
+      </x:c>
+      <x:c r="E4" s="39" t="str">
         <x:v>البنود</x:v>
       </x:c>
-      <x:c r="E4" s="39" t="str">
+      <x:c r="F4" s="39" t="str">
         <x:v>الخطوة التالية</x:v>
       </x:c>
     </x:row>
@@ -1759,10 +1764,13 @@
       <x:c r="C5" s="30" t="str">
         <x:v>docs/operations-control-v2</x:v>
       </x:c>
-      <x:c r="D5" s="30" t="str">
+      <x:c r="D5" s="30" t="n">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="E5" s="30" t="str">
         <x:v>CTRL-001</x:v>
       </x:c>
-      <x:c r="E5" s="30" t="str">
+      <x:c r="F5" s="30" t="str">
         <x:v>مراجعة المالك وAgent مستقل؛ لا دمج قبل قبول الملاحظات.</x:v>
       </x:c>
     </x:row>
@@ -1776,10 +1784,13 @@
       <x:c r="C6" s="31" t="str">
         <x:v>legacy-pr-141</x:v>
       </x:c>
-      <x:c r="D6" s="31" t="str">
+      <x:c r="D6" s="31" t="n">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="E6" s="31" t="str">
         <x:v>CLEAN-001</x:v>
       </x:c>
-      <x:c r="E6" s="31" t="str">
+      <x:c r="F6" s="31" t="str">
         <x:v>قارن مع main الحالي ثم قرر الإغلاق أو الاستخراج؛ لا تدمج كما هي.</x:v>
       </x:c>
     </x:row>
@@ -1793,16 +1804,19 @@
       <x:c r="C7" s="44" t="str">
         <x:v>report/deep-system-audit-20260916</x:v>
       </x:c>
-      <x:c r="D7" s="44" t="str">
+      <x:c r="D7" s="44" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="E7" s="44" t="str">
         <x:v>AUDIT-001</x:v>
       </x:c>
-      <x:c r="E7" s="44" t="str">
+      <x:c r="F7" s="44" t="str">
         <x:v>احفظ قيمة التقرير التاريخية أو أغلق PR بعد مراجعة المالك؛ لا تعتبره تدقيق main الحالي.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A2:F2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: close superseded legacy workstreams
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -6652,7 +6652,7 @@
       </c>
       <c r="B6" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="C6" s="54" t="inlineStr">
@@ -6670,7 +6670,7 @@
       </c>
       <c r="F6" s="54" t="inlineStr">
         <is>
-          <t>قارن مع main الحالي ثم قرر الإغلاق أو الاستخراج؛ لا تدمج كما هي.</t>
+          <t>لا إجراء؛ PR #141 مغلق موثقًا. احتفظ بالرابط كسجل تاريخي ولا تعاود المطالبة به.</t>
         </is>
       </c>
     </row>
@@ -6682,7 +6682,7 @@
       </c>
       <c r="B7" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="C7" s="54" t="inlineStr">
@@ -6700,7 +6700,7 @@
       </c>
       <c r="F7" s="54" t="inlineStr">
         <is>
-          <t>احفظ قيمة التقرير التاريخية أو أغلق PR بعد مراجعة المالك؛ لا تعتبره تدقيق main الحالي.</t>
+          <t>لا إجراء؛ PR #161 مغلق موثقًا. احتفظ بالرابط كسجل تاريخي ولا تعاود المطالبة به.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: close operations control review
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1214,68 +1214,72 @@
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="54" t="inlineStr">
         <is>
+          <t>FIN-001</t>
+        </is>
+      </c>
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>تسجيل اقتراض داخل المشروع</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>FEATURE</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="E12" s="54" t="inlineStr">
+        <is>
+          <t>FIX_BEFORE_PILOT</t>
+        </is>
+      </c>
+      <c r="F12" s="54" t="inlineStr">
+        <is>
+          <t>NOT_APPLICABLE</t>
+        </is>
+      </c>
+      <c r="G12" s="54" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H12" s="54" t="inlineStr">
+        <is>
+          <t>stage-3</t>
+        </is>
+      </c>
+      <c r="I12" s="54" t="inlineStr">
+        <is>
+          <t>Product owner / Manus coordination</t>
+        </is>
+      </c>
+      <c r="J12" s="54" t="inlineStr">
+        <is>
+          <t>Layer 3, domain, application, presentation</t>
+        </is>
+      </c>
+      <c r="K12" s="54" t="inlineStr">
+        <is>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L12" s="54" t="inlineStr">
+        <is>
           <t>CTRL-001</t>
         </is>
       </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>اعتماد Operations Control v2</t>
-        </is>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
-        <is>
-          <t>GOVERNANCE</t>
-        </is>
-      </c>
-      <c r="D12" s="54" t="inlineStr">
-        <is>
-          <t>IN_REVIEW</t>
-        </is>
-      </c>
-      <c r="E12" s="54" t="inlineStr">
-        <is>
-          <t>GOVERNANCE</t>
-        </is>
-      </c>
-      <c r="F12" s="54" t="inlineStr">
-        <is>
-          <t>NOT_APPLICABLE</t>
-        </is>
-      </c>
-      <c r="G12" s="54" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="H12" s="54" t="inlineStr">
-        <is>
-          <t>stage-0</t>
-        </is>
-      </c>
-      <c r="I12" s="54" t="inlineStr">
-        <is>
-          <t>Product owner / Manus coordination</t>
-        </is>
-      </c>
-      <c r="J12" s="54" t="inlineStr">
-        <is>
-          <t>governance, documentation</t>
-        </is>
-      </c>
-      <c r="K12" s="54" t="inlineStr">
-        <is>
-          <t>Validator/schema test | Generated-view freshness check | Owner review evidence</t>
-        </is>
-      </c>
-      <c r="L12" s="54" t="inlineStr"/>
       <c r="M12" s="54" t="inlineStr">
         <is>
-          <t>اعتماد النظام بعد مراجعة المالك وAgent مستقل.</t>
+          <t>اعتماد سياسة القرض المأخوذ: الكاش والالتزام والمحفظة والسداد وفصل الأصل عن الرسوم/الفوائد.</t>
         </is>
       </c>
       <c r="N12" s="54" t="inlineStr">
         <is>
-          <t>استكمل مراجعة المالك والمراجع المستقل ثم حدّث الحالة في PR نفسه.</t>
+          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O12" s="54" t="inlineStr"/>
@@ -1293,32 +1297,32 @@
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="54" t="inlineStr">
         <is>
-          <t>CTRL-002</t>
+          <t>FIN-003</t>
         </is>
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
+          <t>مقارنة الفترات وجسر الربح إلى الكاش</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">
         <is>
-          <t>GOVERNANCE</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D13" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="E13" s="54" t="inlineStr">
         <is>
-          <t>GOVERNANCE</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F13" s="54" t="inlineStr">
         <is>
-          <t>EVIDENCE_RECONCILIATION_REQUIRED</t>
+          <t>NOT_APPLICABLE</t>
         </is>
       </c>
       <c r="G13" s="54" t="inlineStr">
@@ -1328,7 +1332,7 @@
       </c>
       <c r="H13" s="54" t="inlineStr">
         <is>
-          <t>stage-0</t>
+          <t>stage-3</t>
         </is>
       </c>
       <c r="I13" s="54" t="inlineStr">
@@ -1338,23 +1342,23 @@
       </c>
       <c r="J13" s="54" t="inlineStr">
         <is>
-          <t>governance, documentation</t>
+          <t>Layer 3, domain, application, presentation</t>
         </is>
       </c>
       <c r="K13" s="54" t="inlineStr">
         <is>
-          <t>Validator/schema test | Generated-view freshness check | Owner review evidence</t>
-        </is>
-      </c>
-      <c r="L13" s="54" t="inlineStr"/>
-      <c r="M13" s="54" t="inlineStr">
-        <is>
-          <t>تسجيل تعريف العد ومراجعة الأدلة؛ لا يجوز حسم فرق 49/46 بقرار وصفي بلا مصفوفة مصادر.</t>
-        </is>
-      </c>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L13" s="54" t="inlineStr">
+        <is>
+          <t>FIN-001</t>
+        </is>
+      </c>
+      <c r="M13" s="54" t="inlineStr"/>
       <c r="N13" s="54" t="inlineStr">
         <is>
-          <t>أرفق مصفوفة الأدلة التي تحسم تعريف 49/46 ومسارات القدرة، ثم اطلب مراجعة المالك قبل فتح أي Claim كودي.</t>
+          <t>تحقق من الاعتماديات (FIN-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O13" s="54" t="inlineStr"/>
@@ -1372,12 +1376,12 @@
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="54" t="inlineStr">
         <is>
-          <t>FIN-001</t>
+          <t>FIN-004</t>
         </is>
       </c>
       <c r="B14" s="54" t="inlineStr">
         <is>
-          <t>تسجيل اقتراض داخل المشروع</t>
+          <t>حد السحب الآمن للمالك</t>
         </is>
       </c>
       <c r="C14" s="54" t="inlineStr">
@@ -1427,17 +1431,13 @@
       </c>
       <c r="L14" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
-        </is>
-      </c>
-      <c r="M14" s="54" t="inlineStr">
-        <is>
-          <t>اعتماد سياسة القرض المأخوذ: الكاش والالتزام والمحفظة والسداد وفصل الأصل عن الرسوم/الفوائد.</t>
-        </is>
-      </c>
+          <t>FIN-003, FIN-005</t>
+        </is>
+      </c>
+      <c r="M14" s="54" t="inlineStr"/>
       <c r="N14" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (FIN-003, FIN-005) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O14" s="54" t="inlineStr"/>
@@ -1455,12 +1455,12 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="54" t="inlineStr">
         <is>
-          <t>FIN-003</t>
+          <t>FIN-005</t>
         </is>
       </c>
       <c r="B15" s="54" t="inlineStr">
         <is>
-          <t>مقارنة الفترات وجسر الربح إلى الكاش</t>
+          <t>توقع الكاش والتصريحات المتوقعة</t>
         </is>
       </c>
       <c r="C15" s="54" t="inlineStr">
@@ -1510,13 +1510,13 @@
       </c>
       <c r="L15" s="54" t="inlineStr">
         <is>
-          <t>FIN-001</t>
+          <t>OPS-001</t>
         </is>
       </c>
       <c r="M15" s="54" t="inlineStr"/>
       <c r="N15" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (FIN-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (OPS-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O15" s="54" t="inlineStr"/>
@@ -1534,12 +1534,12 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="54" t="inlineStr">
         <is>
-          <t>FIN-004</t>
+          <t>OPS-001</t>
         </is>
       </c>
       <c r="B16" s="54" t="inlineStr">
         <is>
-          <t>حد السحب الآمن للمالك</t>
+          <t>المواعيد والاستحقاقات وتقادم الذمم الأساسي</t>
         </is>
       </c>
       <c r="C16" s="54" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H16" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I16" s="54" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="J16" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K16" s="54" t="inlineStr">
@@ -1589,13 +1589,13 @@
       </c>
       <c r="L16" s="54" t="inlineStr">
         <is>
-          <t>FIN-003, FIN-005</t>
+          <t>CTRL-001</t>
         </is>
       </c>
       <c r="M16" s="54" t="inlineStr"/>
       <c r="N16" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (FIN-003, FIN-005) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O16" s="54" t="inlineStr"/>
@@ -1613,12 +1613,12 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="54" t="inlineStr">
         <is>
-          <t>FIN-005</t>
+          <t>OPS-005</t>
         </is>
       </c>
       <c r="B17" s="54" t="inlineStr">
         <is>
-          <t>توقع الكاش والتصريحات المتوقعة</t>
+          <t>سطح قادم موحد للدفعات والتحصيلات والطلبات والالتزامات</t>
         </is>
       </c>
       <c r="C17" s="54" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="H17" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I17" s="54" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="J17" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K17" s="54" t="inlineStr">
@@ -1668,19 +1668,19 @@
       </c>
       <c r="L17" s="54" t="inlineStr">
         <is>
-          <t>OPS-001</t>
+          <t>CTRL-001, OPS-001</t>
         </is>
       </c>
       <c r="M17" s="54" t="inlineStr"/>
       <c r="N17" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (OPS-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
         </is>
       </c>
       <c r="O17" s="54" t="inlineStr"/>
       <c r="P17" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q17" s="54" t="inlineStr">
@@ -1692,17 +1692,17 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="54" t="inlineStr">
         <is>
-          <t>OPS-001</t>
+          <t>OPS-009</t>
         </is>
       </c>
       <c r="B18" s="54" t="inlineStr">
         <is>
-          <t>المواعيد والاستحقاقات وتقادم الذمم الأساسي</t>
+          <t>حماية Cost Snapshot وإعلان النتيجة النهائية أو التقديرية</t>
         </is>
       </c>
       <c r="C18" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D18" s="54" t="inlineStr">
@@ -1742,24 +1742,24 @@
       </c>
       <c r="K18" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
         </is>
       </c>
       <c r="L18" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
+          <t>CTRL-001, OPS-007</t>
         </is>
       </c>
       <c r="M18" s="54" t="inlineStr"/>
       <c r="N18" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
         </is>
       </c>
       <c r="O18" s="54" t="inlineStr"/>
       <c r="P18" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q18" s="54" t="inlineStr">
@@ -1771,17 +1771,17 @@
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="54" t="inlineStr">
         <is>
-          <t>OPS-005</t>
+          <t>REL-001</t>
         </is>
       </c>
       <c r="B19" s="54" t="inlineStr">
         <is>
-          <t>سطح قادم موحد للدفعات والتحصيلات والطلبات والالتزامات</t>
+          <t>اختبارات الصمود والفشل</t>
         </is>
       </c>
       <c r="C19" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D19" s="54" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="H19" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>stage-6</t>
         </is>
       </c>
       <c r="I19" s="54" t="inlineStr">
@@ -1816,29 +1816,29 @@
       </c>
       <c r="J19" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>storage, transfer, resilience</t>
         </is>
       </c>
       <c r="K19" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
         </is>
       </c>
       <c r="L19" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-001</t>
+          <t>CLEAN-001</t>
         </is>
       </c>
       <c r="M19" s="54" t="inlineStr"/>
       <c r="N19" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>تحقق من الاعتماديات (CLEAN-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O19" s="54" t="inlineStr"/>
       <c r="P19" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q19" s="54" t="inlineStr">
@@ -1850,12 +1850,12 @@
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="54" t="inlineStr">
         <is>
-          <t>OPS-009</t>
+          <t>CLEAN-001</t>
         </is>
       </c>
       <c r="B20" s="54" t="inlineStr">
         <is>
-          <t>حماية Cost Snapshot وإعلان النتيجة النهائية أو التقديرية</t>
+          <t>تنظيف الأسطح الجزئية والميتة</t>
         </is>
       </c>
       <c r="C20" s="54" t="inlineStr">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="G20" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H20" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>stage-4</t>
         </is>
       </c>
       <c r="I20" s="54" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="J20" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>cross-layer, presentation</t>
         </is>
       </c>
       <c r="K20" s="54" t="inlineStr">
@@ -1905,19 +1905,19 @@
       </c>
       <c r="L20" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-007</t>
+          <t>FIN-007, OPS-004</t>
         </is>
       </c>
       <c r="M20" s="54" t="inlineStr"/>
       <c r="N20" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>تحقق من الاعتماديات (FIN-007, OPS-004) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O20" s="54" t="inlineStr"/>
       <c r="P20" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q20" s="54" t="inlineStr">
@@ -1929,17 +1929,17 @@
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="54" t="inlineStr">
         <is>
-          <t>REL-001</t>
+          <t>FIN-007</t>
         </is>
       </c>
       <c r="B21" s="54" t="inlineStr">
         <is>
-          <t>اختبارات الصمود والفشل</t>
+          <t>مراجعة فترة مرنة</t>
         </is>
       </c>
       <c r="C21" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D21" s="54" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="G21" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H21" s="54" t="inlineStr">
         <is>
-          <t>stage-6</t>
+          <t>stage-3</t>
         </is>
       </c>
       <c r="I21" s="54" t="inlineStr">
@@ -1974,23 +1974,23 @@
       </c>
       <c r="J21" s="54" t="inlineStr">
         <is>
-          <t>storage, transfer, resilience</t>
+          <t>Layer 3, domain, application, presentation</t>
         </is>
       </c>
       <c r="K21" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
       <c r="L21" s="54" t="inlineStr">
         <is>
-          <t>CLEAN-001</t>
+          <t>FIN-003</t>
         </is>
       </c>
       <c r="M21" s="54" t="inlineStr"/>
       <c r="N21" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CLEAN-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (FIN-003) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O21" s="54" t="inlineStr"/>
@@ -2008,17 +2008,17 @@
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="54" t="inlineStr">
         <is>
-          <t>CLEAN-001</t>
+          <t>OPS-002</t>
         </is>
       </c>
       <c r="B22" s="54" t="inlineStr">
         <is>
-          <t>تنظيف الأسطح الجزئية والميتة</t>
+          <t>تنبيهات انخفاض المخزون</t>
         </is>
       </c>
       <c r="C22" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D22" s="54" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="H22" s="54" t="inlineStr">
         <is>
-          <t>stage-4</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I22" s="54" t="inlineStr">
@@ -2053,23 +2053,23 @@
       </c>
       <c r="J22" s="54" t="inlineStr">
         <is>
-          <t>cross-layer, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K22" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
       <c r="L22" s="54" t="inlineStr">
         <is>
-          <t>FIN-007, OPS-004</t>
+          <t>CTRL-001</t>
         </is>
       </c>
       <c r="M22" s="54" t="inlineStr"/>
       <c r="N22" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (FIN-007, OPS-004) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O22" s="54" t="inlineStr"/>
@@ -2087,12 +2087,12 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="54" t="inlineStr">
         <is>
-          <t>FIN-007</t>
+          <t>OPS-004</t>
         </is>
       </c>
       <c r="B23" s="54" t="inlineStr">
         <is>
-          <t>مراجعة فترة مرنة</t>
+          <t>ربط القوالب بالتكلفة المخططة دون استهلاك فعلي</t>
         </is>
       </c>
       <c r="C23" s="54" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="H23" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I23" s="54" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="J23" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K23" s="54" t="inlineStr">
@@ -2142,13 +2142,13 @@
       </c>
       <c r="L23" s="54" t="inlineStr">
         <is>
-          <t>FIN-003</t>
+          <t>CTRL-001</t>
         </is>
       </c>
       <c r="M23" s="54" t="inlineStr"/>
       <c r="N23" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (FIN-003) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O23" s="54" t="inlineStr"/>
@@ -2166,12 +2166,12 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="54" t="inlineStr">
         <is>
-          <t>OPS-002</t>
+          <t>OPS-006</t>
         </is>
       </c>
       <c r="B24" s="54" t="inlineStr">
         <is>
-          <t>تنبيهات انخفاض المخزون</t>
+          <t>تقادم ديون مبسط قبل الشرائح المتقدمة</t>
         </is>
       </c>
       <c r="C24" s="54" t="inlineStr">
@@ -2221,19 +2221,19 @@
       </c>
       <c r="L24" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
+          <t>CTRL-001, OPS-001</t>
         </is>
       </c>
       <c r="M24" s="54" t="inlineStr"/>
       <c r="N24" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
         </is>
       </c>
       <c r="O24" s="54" t="inlineStr"/>
       <c r="P24" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q24" s="54" t="inlineStr">
@@ -2245,12 +2245,12 @@
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="54" t="inlineStr">
         <is>
-          <t>OPS-004</t>
+          <t>OPS-007</t>
         </is>
       </c>
       <c r="B25" s="54" t="inlineStr">
         <is>
-          <t>ربط القوالب بالتكلفة المخططة دون استهلاك فعلي</t>
+          <t>مقارنة التكلفة المخططة بالمستهلكة والفرق</t>
         </is>
       </c>
       <c r="C25" s="54" t="inlineStr">
@@ -2300,19 +2300,19 @@
       </c>
       <c r="L25" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
+          <t>CTRL-001, OPS-004</t>
         </is>
       </c>
       <c r="M25" s="54" t="inlineStr"/>
       <c r="N25" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
         </is>
       </c>
       <c r="O25" s="54" t="inlineStr"/>
       <c r="P25" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q25" s="54" t="inlineStr">
@@ -2324,12 +2324,12 @@
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="54" t="inlineStr">
         <is>
-          <t>OPS-006</t>
+          <t>OPS-008</t>
         </is>
       </c>
       <c r="B26" s="54" t="inlineStr">
         <is>
-          <t>تقادم ديون مبسط قبل الشرائح المتقدمة</t>
+          <t>الوقت الفعلي مقابل المخطط</t>
         </is>
       </c>
       <c r="C26" s="54" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="L26" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-001</t>
+          <t>CTRL-001, OPS-004</t>
         </is>
       </c>
       <c r="M26" s="54" t="inlineStr"/>
@@ -2403,27 +2403,27 @@
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="54" t="inlineStr">
         <is>
-          <t>OPS-007</t>
+          <t>AUDIT-001</t>
         </is>
       </c>
       <c r="B27" s="54" t="inlineStr">
         <is>
-          <t>مقارنة التكلفة المخططة بالمستهلكة والفرق</t>
+          <t>تدقيق مستقل نهائي قبل الـPilot</t>
         </is>
       </c>
       <c r="C27" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D27" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E27" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>RELEASE_GATE</t>
         </is>
       </c>
       <c r="F27" s="54" t="inlineStr">
@@ -2433,12 +2433,12 @@
       </c>
       <c r="G27" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H27" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>stage-9</t>
         </is>
       </c>
       <c r="I27" s="54" t="inlineStr">
@@ -2448,29 +2448,29 @@
       </c>
       <c r="J27" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>uat, audit, cross-layer</t>
         </is>
       </c>
       <c r="K27" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
         </is>
       </c>
       <c r="L27" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-004</t>
+          <t>UAT-001</t>
         </is>
       </c>
       <c r="M27" s="54" t="inlineStr"/>
       <c r="N27" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>حوّل البند إلى READY بعد تحقق الاعتماديات (UAT-001) ومعيار القبول.</t>
         </is>
       </c>
       <c r="O27" s="54" t="inlineStr"/>
       <c r="P27" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q27" s="54" t="inlineStr">
@@ -2482,27 +2482,27 @@
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="54" t="inlineStr">
         <is>
-          <t>OPS-008</t>
+          <t>UAT-001</t>
         </is>
       </c>
       <c r="B28" s="54" t="inlineStr">
         <is>
-          <t>الوقت الفعلي مقابل المخطط</t>
+          <t>قبول داخلي ببيانات Demo كاملة</t>
         </is>
       </c>
       <c r="C28" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D28" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E28" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>RELEASE_GATE</t>
         </is>
       </c>
       <c r="F28" s="54" t="inlineStr">
@@ -2512,12 +2512,12 @@
       </c>
       <c r="G28" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H28" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>stage-9</t>
         </is>
       </c>
       <c r="I28" s="54" t="inlineStr">
@@ -2527,29 +2527,29 @@
       </c>
       <c r="J28" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>uat, audit, cross-layer</t>
         </is>
       </c>
       <c r="K28" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
         </is>
       </c>
       <c r="L28" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-004</t>
+          <t>DEVICE-001, LEGAL-001</t>
         </is>
       </c>
       <c r="M28" s="54" t="inlineStr"/>
       <c r="N28" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>حوّل البند إلى READY بعد تحقق الاعتماديات (DEVICE-001, LEGAL-001) ومعيار القبول.</t>
         </is>
       </c>
       <c r="O28" s="54" t="inlineStr"/>
       <c r="P28" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q28" s="54" t="inlineStr">
@@ -2561,27 +2561,27 @@
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="54" t="inlineStr">
         <is>
-          <t>AUDIT-001</t>
+          <t>G-001</t>
         </is>
       </c>
       <c r="B29" s="54" t="inlineStr">
         <is>
-          <t>تدقيق مستقل نهائي قبل الـPilot</t>
+          <t>فخ الاستهلاك المزدوج عند التسليم</t>
         </is>
       </c>
       <c r="C29" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>DEFECT</t>
         </is>
       </c>
       <c r="D29" s="54" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="E29" s="54" t="inlineStr">
         <is>
-          <t>RELEASE_GATE</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F29" s="54" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="H29" s="54" t="inlineStr">
         <is>
-          <t>stage-9</t>
+          <t>audit-2026-09-19</t>
         </is>
       </c>
       <c r="I29" s="54" t="inlineStr">
@@ -2606,29 +2606,25 @@
       </c>
       <c r="J29" s="54" t="inlineStr">
         <is>
-          <t>uat, audit, cross-layer</t>
+          <t>cross-layer</t>
         </is>
       </c>
       <c r="K29" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
-        </is>
-      </c>
-      <c r="L29" s="54" t="inlineStr">
-        <is>
-          <t>UAT-001</t>
-        </is>
-      </c>
+          <t>Domain/Service tests where the invariant is owned | DOM/Integration test for the affected journey | Live scenario with before/after evidence | Retry, partial failure, concurrency, or stale-read test as applicable | No regression in existing financial calculations | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L29" s="54" t="inlineStr"/>
       <c r="M29" s="54" t="inlineStr"/>
       <c r="N29" s="54" t="inlineStr">
         <is>
-          <t>حوّل البند إلى READY بعد تحقق الاعتماديات (UAT-001) ومعيار القبول.</t>
+          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
         </is>
       </c>
       <c r="O29" s="54" t="inlineStr"/>
       <c r="P29" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q29" s="54" t="inlineStr">
@@ -2640,27 +2636,27 @@
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="54" t="inlineStr">
         <is>
-          <t>UAT-001</t>
+          <t>GOV-001</t>
         </is>
       </c>
       <c r="B30" s="54" t="inlineStr">
         <is>
-          <t>قبول داخلي ببيانات Demo كاملة</t>
+          <t>مصالحة G10-A مع تعارض عقد C1</t>
         </is>
       </c>
       <c r="C30" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>DECISION</t>
         </is>
       </c>
       <c r="D30" s="54" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="E30" s="54" t="inlineStr">
         <is>
-          <t>RELEASE_GATE</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="F30" s="54" t="inlineStr">
@@ -2675,7 +2671,7 @@
       </c>
       <c r="H30" s="54" t="inlineStr">
         <is>
-          <t>stage-9</t>
+          <t>governance</t>
         </is>
       </c>
       <c r="I30" s="54" t="inlineStr">
@@ -2685,29 +2681,29 @@
       </c>
       <c r="J30" s="54" t="inlineStr">
         <is>
-          <t>uat, audit, cross-layer</t>
+          <t>governance, contracts</t>
         </is>
       </c>
       <c r="K30" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
-        </is>
-      </c>
-      <c r="L30" s="54" t="inlineStr">
-        <is>
-          <t>DEVICE-001, LEGAL-001</t>
-        </is>
-      </c>
-      <c r="M30" s="54" t="inlineStr"/>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L30" s="54" t="inlineStr"/>
+      <c r="M30" s="54" t="inlineStr">
+        <is>
+          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
+        </is>
+      </c>
       <c r="N30" s="54" t="inlineStr">
         <is>
-          <t>حوّل البند إلى READY بعد تحقق الاعتماديات (DEVICE-001, LEGAL-001) ومعيار القبول.</t>
+          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
         </is>
       </c>
       <c r="O30" s="54" t="inlineStr"/>
       <c r="P30" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q30" s="54" t="inlineStr">
@@ -2719,12 +2715,12 @@
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="54" t="inlineStr">
         <is>
-          <t>G-001</t>
+          <t>G-002</t>
         </is>
       </c>
       <c r="B31" s="54" t="inlineStr">
         <is>
-          <t>فخ الاستهلاك المزدوج عند التسليم</t>
+          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
         </is>
       </c>
       <c r="C31" s="54" t="inlineStr">
@@ -2749,7 +2745,7 @@
       </c>
       <c r="G31" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H31" s="54" t="inlineStr">
@@ -2776,7 +2772,7 @@
       <c r="M31" s="54" t="inlineStr"/>
       <c r="N31" s="54" t="inlineStr">
         <is>
-          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
+          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
         </is>
       </c>
       <c r="O31" s="54" t="inlineStr"/>
@@ -2794,17 +2790,17 @@
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="54" t="inlineStr">
         <is>
-          <t>GOV-001</t>
+          <t>G-003</t>
         </is>
       </c>
       <c r="B32" s="54" t="inlineStr">
         <is>
-          <t>مصالحة G10-A مع تعارض عقد C1</t>
+          <t>حرس القراءة القديمة عند حفظ الطلب</t>
         </is>
       </c>
       <c r="C32" s="54" t="inlineStr">
         <is>
-          <t>DECISION</t>
+          <t>DEFECT</t>
         </is>
       </c>
       <c r="D32" s="54" t="inlineStr">
@@ -2814,7 +2810,7 @@
       </c>
       <c r="E32" s="54" t="inlineStr">
         <is>
-          <t>GOVERNANCE</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F32" s="54" t="inlineStr">
@@ -2824,12 +2820,12 @@
       </c>
       <c r="G32" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H32" s="54" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>audit-2026-09-19</t>
         </is>
       </c>
       <c r="I32" s="54" t="inlineStr">
@@ -2839,23 +2835,19 @@
       </c>
       <c r="J32" s="54" t="inlineStr">
         <is>
-          <t>governance, contracts</t>
+          <t>cross-layer</t>
         </is>
       </c>
       <c r="K32" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Domain/Service tests where the invariant is owned | DOM/Integration test for the affected journey | Live scenario with before/after evidence | Retry, partial failure, concurrency, or stale-read test as applicable | No regression in existing financial calculations | Merge and verification evidence on main</t>
         </is>
       </c>
       <c r="L32" s="54" t="inlineStr"/>
-      <c r="M32" s="54" t="inlineStr">
-        <is>
-          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
-        </is>
-      </c>
+      <c r="M32" s="54" t="inlineStr"/>
       <c r="N32" s="54" t="inlineStr">
         <is>
-          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
+          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
         </is>
       </c>
       <c r="O32" s="54" t="inlineStr"/>
@@ -2873,12 +2865,12 @@
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="54" t="inlineStr">
         <is>
-          <t>G-002</t>
+          <t>G-004</t>
         </is>
       </c>
       <c r="B33" s="54" t="inlineStr">
         <is>
-          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
+          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
         </is>
       </c>
       <c r="C33" s="54" t="inlineStr">
@@ -2930,7 +2922,7 @@
       <c r="M33" s="54" t="inlineStr"/>
       <c r="N33" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
+          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
         </is>
       </c>
       <c r="O33" s="54" t="inlineStr"/>
@@ -2948,12 +2940,12 @@
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="54" t="inlineStr">
         <is>
-          <t>G-003</t>
+          <t>G-005</t>
         </is>
       </c>
       <c r="B34" s="54" t="inlineStr">
         <is>
-          <t>حرس القراءة القديمة عند حفظ الطلب</t>
+          <t>عزل فشل قراءات صفحة المالية</t>
         </is>
       </c>
       <c r="C34" s="54" t="inlineStr">
@@ -3005,7 +2997,7 @@
       <c r="M34" s="54" t="inlineStr"/>
       <c r="N34" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
+          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
         </is>
       </c>
       <c r="O34" s="54" t="inlineStr"/>
@@ -3023,12 +3015,12 @@
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="54" t="inlineStr">
         <is>
-          <t>G-004</t>
+          <t>G-006</t>
         </is>
       </c>
       <c r="B35" s="54" t="inlineStr">
         <is>
-          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
+          <t>توحيد حرس السحب بين مساري مال المالك</t>
         </is>
       </c>
       <c r="C35" s="54" t="inlineStr">
@@ -3053,7 +3045,7 @@
       </c>
       <c r="G35" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H35" s="54" t="inlineStr">
@@ -3080,7 +3072,7 @@
       <c r="M35" s="54" t="inlineStr"/>
       <c r="N35" s="54" t="inlineStr">
         <is>
-          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
+          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
         </is>
       </c>
       <c r="O35" s="54" t="inlineStr"/>
@@ -3098,42 +3090,42 @@
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="54" t="inlineStr">
         <is>
-          <t>G-005</t>
+          <t>SCOPE-001</t>
         </is>
       </c>
       <c r="B36" s="54" t="inlineStr">
         <is>
-          <t>عزل فشل قراءات صفحة المالية</t>
+          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
         </is>
       </c>
       <c r="C36" s="54" t="inlineStr">
         <is>
-          <t>DEFECT</t>
+          <t>DECISION</t>
         </is>
       </c>
       <c r="D36" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="E36" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>FUTURE_SCOPE</t>
         </is>
       </c>
       <c r="F36" s="54" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE</t>
+          <t>OUT_OF_SCOPE</t>
         </is>
       </c>
       <c r="G36" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H36" s="54" t="inlineStr">
         <is>
-          <t>audit-2026-09-19</t>
+          <t>future-scope</t>
         </is>
       </c>
       <c r="I36" s="54" t="inlineStr">
@@ -3143,22 +3135,30 @@
       </c>
       <c r="J36" s="54" t="inlineStr">
         <is>
-          <t>cross-layer</t>
+          <t>future-scope</t>
         </is>
       </c>
       <c r="K36" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests where the invariant is owned | DOM/Integration test for the affected journey | Live scenario with before/after evidence | Retry, partial failure, concurrency, or stale-read test as applicable | No regression in existing financial calculations | Merge and verification evidence on main</t>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
       <c r="L36" s="54" t="inlineStr"/>
-      <c r="M36" s="54" t="inlineStr"/>
+      <c r="M36" s="54" t="inlineStr">
+        <is>
+          <t>تحديد بوابة مستقلة لكل توسع مستقبلًا.</t>
+        </is>
+      </c>
       <c r="N36" s="54" t="inlineStr">
         <is>
-          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
-        </is>
-      </c>
-      <c r="O36" s="54" t="inlineStr"/>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+        </is>
+      </c>
+      <c r="O36" s="54" t="inlineStr">
+        <is>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+        </is>
+      </c>
       <c r="P36" s="54" t="inlineStr">
         <is>
           <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
@@ -3173,22 +3173,22 @@
     <row r="37">
       <c r="A37" s="54" t="inlineStr">
         <is>
-          <t>G-006</t>
+          <t>UX-001</t>
         </is>
       </c>
       <c r="B37" s="54" t="inlineStr">
         <is>
-          <t>توحيد حرس السحب بين مساري مال المالك</t>
+          <t>إعادة تصميم UI وUX جذرية</t>
         </is>
       </c>
       <c r="C37" s="54" t="inlineStr">
         <is>
-          <t>DEFECT</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D37" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="E37" s="54" t="inlineStr">
@@ -3198,17 +3198,17 @@
       </c>
       <c r="F37" s="54" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE</t>
+          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="G37" s="54" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H37" s="54" t="inlineStr">
         <is>
-          <t>audit-2026-09-19</t>
+          <t>stage-5</t>
         </is>
       </c>
       <c r="I37" s="54" t="inlineStr">
@@ -3218,25 +3218,37 @@
       </c>
       <c r="J37" s="54" t="inlineStr">
         <is>
-          <t>cross-layer</t>
+          <t>ui/ux, presentation</t>
         </is>
       </c>
       <c r="K37" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests where the invariant is owned | DOM/Integration test for the affected journey | Live scenario with before/after evidence | Retry, partial failure, concurrency, or stale-read test as applicable | No regression in existing financial calculations | Merge and verification evidence on main</t>
-        </is>
-      </c>
-      <c r="L37" s="54" t="inlineStr"/>
-      <c r="M37" s="54" t="inlineStr"/>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L37" s="54" t="inlineStr">
+        <is>
+          <t>CLEAN-001</t>
+        </is>
+      </c>
+      <c r="M37" s="54" t="inlineStr">
+        <is>
+          <t>اعتماد الاتجاه البصري النهائي ونتائج Benchmark قبل التنفيذ.</t>
+        </is>
+      </c>
       <c r="N37" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
-        </is>
-      </c>
-      <c r="O37" s="54" t="inlineStr"/>
+          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
+        </is>
+      </c>
+      <c r="O37" s="54" t="inlineStr">
+        <is>
+          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+        </is>
+      </c>
       <c r="P37" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
         </is>
       </c>
       <c r="Q37" s="54" t="inlineStr">
@@ -3248,17 +3260,17 @@
     <row r="38">
       <c r="A38" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-001</t>
+          <t>BE-001</t>
         </is>
       </c>
       <c r="B38" s="54" t="inlineStr">
         <is>
-          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
+          <t>مصاريف متكررة محلية</t>
         </is>
       </c>
       <c r="C38" s="54" t="inlineStr">
         <is>
-          <t>DECISION</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D38" s="54" t="inlineStr">
@@ -3268,22 +3280,22 @@
       </c>
       <c r="E38" s="54" t="inlineStr">
         <is>
-          <t>FUTURE_SCOPE</t>
+          <t>HISTORICAL</t>
         </is>
       </c>
       <c r="F38" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE</t>
+          <t>DUPLICATE_HISTORICAL</t>
         </is>
       </c>
       <c r="G38" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H38" s="54" t="inlineStr">
         <is>
-          <t>future-scope</t>
+          <t>build-after-evidence</t>
         </is>
       </c>
       <c r="I38" s="54" t="inlineStr">
@@ -3293,7 +3305,7 @@
       </c>
       <c r="J38" s="54" t="inlineStr">
         <is>
-          <t>future-scope</t>
+          <t>future-capability</t>
         </is>
       </c>
       <c r="K38" s="54" t="inlineStr">
@@ -3302,19 +3314,15 @@
         </is>
       </c>
       <c r="L38" s="54" t="inlineStr"/>
-      <c r="M38" s="54" t="inlineStr">
-        <is>
-          <t>تحديد بوابة مستقلة لكل توسع مستقبلًا.</t>
-        </is>
-      </c>
+      <c r="M38" s="54" t="inlineStr"/>
       <c r="N38" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
       <c r="O38" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
         </is>
       </c>
       <c r="P38" s="54" t="inlineStr">
@@ -3331,12 +3339,12 @@
     <row r="39">
       <c r="A39" s="54" t="inlineStr">
         <is>
-          <t>UX-001</t>
+          <t>BE-002</t>
         </is>
       </c>
       <c r="B39" s="54" t="inlineStr">
         <is>
-          <t>إعادة تصميم UI وUX جذرية</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="C39" s="54" t="inlineStr">
@@ -3351,22 +3359,22 @@
       </c>
       <c r="E39" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>HISTORICAL</t>
         </is>
       </c>
       <c r="F39" s="54" t="inlineStr">
         <is>
-          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
+          <t>DUPLICATE_HISTORICAL</t>
         </is>
       </c>
       <c r="G39" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H39" s="54" t="inlineStr">
         <is>
-          <t>stage-5</t>
+          <t>build-after-evidence</t>
         </is>
       </c>
       <c r="I39" s="54" t="inlineStr">
@@ -3376,7 +3384,7 @@
       </c>
       <c r="J39" s="54" t="inlineStr">
         <is>
-          <t>ui/ux, presentation</t>
+          <t>future-capability</t>
         </is>
       </c>
       <c r="K39" s="54" t="inlineStr">
@@ -3384,29 +3392,21 @@
           <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
-      <c r="L39" s="54" t="inlineStr">
-        <is>
-          <t>CLEAN-001</t>
-        </is>
-      </c>
-      <c r="M39" s="54" t="inlineStr">
-        <is>
-          <t>اعتماد الاتجاه البصري النهائي ونتائج Benchmark قبل التنفيذ.</t>
-        </is>
-      </c>
+      <c r="L39" s="54" t="inlineStr"/>
+      <c r="M39" s="54" t="inlineStr"/>
       <c r="N39" s="54" t="inlineStr">
         <is>
-          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
       <c r="O39" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
         </is>
       </c>
       <c r="P39" s="54" t="inlineStr">
         <is>
-          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q39" s="54" t="inlineStr">
@@ -3418,12 +3418,12 @@
     <row r="40">
       <c r="A40" s="54" t="inlineStr">
         <is>
-          <t>BE-001</t>
+          <t>BE-003</t>
         </is>
       </c>
       <c r="B40" s="54" t="inlineStr">
         <is>
-          <t>مصاريف متكررة محلية</t>
+          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="C40" s="54" t="inlineStr">
@@ -3475,7 +3475,7 @@
       <c r="M40" s="54" t="inlineStr"/>
       <c r="N40" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
       <c r="O40" s="54" t="inlineStr">
@@ -3497,12 +3497,12 @@
     <row r="41">
       <c r="A41" s="54" t="inlineStr">
         <is>
-          <t>BE-002</t>
+          <t>BE-004</t>
         </is>
       </c>
       <c r="B41" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>إغلاق فترة رسمي</t>
         </is>
       </c>
       <c r="C41" s="54" t="inlineStr">
@@ -3517,12 +3517,12 @@
       </c>
       <c r="E41" s="54" t="inlineStr">
         <is>
-          <t>HISTORICAL</t>
+          <t>PILOT_VALIDATION</t>
         </is>
       </c>
       <c r="F41" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL</t>
+          <t>PILOT_EVIDENCE_REQUIRED</t>
         </is>
       </c>
       <c r="G41" s="54" t="inlineStr">
@@ -3554,12 +3554,12 @@
       <c r="M41" s="54" t="inlineStr"/>
       <c r="N41" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
       <c r="O41" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="P41" s="54" t="inlineStr">
@@ -3576,12 +3576,12 @@
     <row r="42">
       <c r="A42" s="54" t="inlineStr">
         <is>
-          <t>BE-003</t>
+          <t>BE-005</t>
         </is>
       </c>
       <c r="B42" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
+          <t>تقادم الديون بشرائح 30/60/90</t>
         </is>
       </c>
       <c r="C42" s="54" t="inlineStr">
@@ -3596,12 +3596,12 @@
       </c>
       <c r="E42" s="54" t="inlineStr">
         <is>
-          <t>HISTORICAL</t>
+          <t>PILOT_VALIDATION</t>
         </is>
       </c>
       <c r="F42" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL</t>
+          <t>PILOT_EVIDENCE_REQUIRED</t>
         </is>
       </c>
       <c r="G42" s="54" t="inlineStr">
@@ -3633,12 +3633,12 @@
       <c r="M42" s="54" t="inlineStr"/>
       <c r="N42" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
       <c r="O42" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="P42" s="54" t="inlineStr">
@@ -3655,12 +3655,12 @@
     <row r="43">
       <c r="A43" s="54" t="inlineStr">
         <is>
-          <t>BE-004</t>
+          <t>FIN-002</t>
         </is>
       </c>
       <c r="B43" s="54" t="inlineStr">
         <is>
-          <t>إغلاق فترة رسمي</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="C43" s="54" t="inlineStr">
@@ -3675,12 +3675,12 @@
       </c>
       <c r="E43" s="54" t="inlineStr">
         <is>
-          <t>PILOT_VALIDATION</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F43" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED</t>
+          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="G43" s="54" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="H43" s="54" t="inlineStr">
         <is>
-          <t>build-after-evidence</t>
+          <t>stage-3</t>
         </is>
       </c>
       <c r="I43" s="54" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="J43" s="54" t="inlineStr">
         <is>
-          <t>future-capability</t>
+          <t>Layer 3, domain, application, presentation</t>
         </is>
       </c>
       <c r="K43" s="54" t="inlineStr">
@@ -3708,21 +3708,25 @@
           <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
-      <c r="L43" s="54" t="inlineStr"/>
+      <c r="L43" s="54" t="inlineStr">
+        <is>
+          <t>CTRL-001</t>
+        </is>
+      </c>
       <c r="M43" s="54" t="inlineStr"/>
       <c r="N43" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
         </is>
       </c>
       <c r="O43" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="P43" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q43" s="54" t="inlineStr">
@@ -3734,12 +3738,12 @@
     <row r="44">
       <c r="A44" s="54" t="inlineStr">
         <is>
-          <t>BE-005</t>
+          <t>FIN-006</t>
         </is>
       </c>
       <c r="B44" s="54" t="inlineStr">
         <is>
-          <t>تقادم الديون بشرائح 30/60/90</t>
+          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="C44" s="54" t="inlineStr">
@@ -3754,12 +3758,12 @@
       </c>
       <c r="E44" s="54" t="inlineStr">
         <is>
-          <t>PILOT_VALIDATION</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F44" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED</t>
+          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="G44" s="54" t="inlineStr">
@@ -3769,7 +3773,7 @@
       </c>
       <c r="H44" s="54" t="inlineStr">
         <is>
-          <t>build-after-evidence</t>
+          <t>stage-3</t>
         </is>
       </c>
       <c r="I44" s="54" t="inlineStr">
@@ -3779,7 +3783,7 @@
       </c>
       <c r="J44" s="54" t="inlineStr">
         <is>
-          <t>future-capability</t>
+          <t>Layer 3, domain, application, presentation</t>
         </is>
       </c>
       <c r="K44" s="54" t="inlineStr">
@@ -3787,21 +3791,25 @@
           <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
-      <c r="L44" s="54" t="inlineStr"/>
+      <c r="L44" s="54" t="inlineStr">
+        <is>
+          <t>OPS-004</t>
+        </is>
+      </c>
       <c r="M44" s="54" t="inlineStr"/>
       <c r="N44" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
         </is>
       </c>
       <c r="O44" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="P44" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q44" s="54" t="inlineStr">
@@ -3813,17 +3821,17 @@
     <row r="45">
       <c r="A45" s="54" t="inlineStr">
         <is>
-          <t>FIN-002</t>
+          <t>FIN-008</t>
         </is>
       </c>
       <c r="B45" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>تحقق الإهلاك بعد مرور الزمن</t>
         </is>
       </c>
       <c r="C45" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D45" s="54" t="inlineStr">
@@ -3863,23 +3871,23 @@
       </c>
       <c r="K45" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
-        </is>
-      </c>
-      <c r="L45" s="54" t="inlineStr">
-        <is>
-          <t>CTRL-001</t>
-        </is>
-      </c>
-      <c r="M45" s="54" t="inlineStr"/>
+          <t>اختبار Domain/Service مع Clock قابل للحقن يثبت تاريخ الاستحقاق قبل/بعد نقطة زمنية اصطناعية | اختبار idempotency يمنع تسجيل الإهلاك نفسه مرتين عند إعادة تشغيل الساعة/الفعل | اختبار DOM يثبت أن الإهلاك غير النقدي لا يخصم من الكاش ويعرض الحالة الصادقة | اختبار export/import يحافظ على أصل الإهلاك وتاريخه إن دخلت البيانات الدائمة | دليل CI وMerge SHA وverified_on_main_sha قبل VERIFIED</t>
+        </is>
+      </c>
+      <c r="L45" s="54" t="inlineStr"/>
+      <c r="M45" s="54" t="inlineStr">
+        <is>
+          <t>تحديد نافذة اختبار الإهلاك أو آلية ساعة اختبار معتمدة قبل فتح Claim.</t>
+        </is>
+      </c>
       <c r="N45" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
+          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
         </is>
       </c>
       <c r="O45" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
         </is>
       </c>
       <c r="P45" s="54" t="inlineStr">
@@ -3896,12 +3904,12 @@
     <row r="46">
       <c r="A46" s="54" t="inlineStr">
         <is>
-          <t>FIN-006</t>
+          <t>OPS-003</t>
         </is>
       </c>
       <c r="B46" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
+          <t>المصروفات المتكررة المحلية</t>
         </is>
       </c>
       <c r="C46" s="54" t="inlineStr">
@@ -3931,7 +3939,7 @@
       </c>
       <c r="H46" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I46" s="54" t="inlineStr">
@@ -3941,7 +3949,7 @@
       </c>
       <c r="J46" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K46" s="54" t="inlineStr">
@@ -3951,18 +3959,22 @@
       </c>
       <c r="L46" s="54" t="inlineStr">
         <is>
-          <t>OPS-004</t>
-        </is>
-      </c>
-      <c r="M46" s="54" t="inlineStr"/>
+          <t>CTRL-001</t>
+        </is>
+      </c>
+      <c r="M46" s="54" t="inlineStr">
+        <is>
+          <t>اعتماد أن المصروف المتكرر تذكير يحتاج تأكيدًا ولا ينشئ حدثًا ماليًا تلقائيًا.</t>
+        </is>
+      </c>
       <c r="N46" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
         </is>
       </c>
       <c r="O46" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
         </is>
       </c>
       <c r="P46" s="54" t="inlineStr">
@@ -3979,17 +3991,17 @@
     <row r="47">
       <c r="A47" s="54" t="inlineStr">
         <is>
-          <t>FIN-008</t>
+          <t>SCOPE-002</t>
         </is>
       </c>
       <c r="B47" s="54" t="inlineStr">
         <is>
-          <t>تحقق الإهلاك بعد مرور الزمن</t>
+          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
         </is>
       </c>
       <c r="C47" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>RESEARCH</t>
         </is>
       </c>
       <c r="D47" s="54" t="inlineStr">
@@ -3999,12 +4011,12 @@
       </c>
       <c r="E47" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>FUTURE_SCOPE</t>
         </is>
       </c>
       <c r="F47" s="54" t="inlineStr">
         <is>
-          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
+          <t>OUT_OF_SCOPE</t>
         </is>
       </c>
       <c r="G47" s="54" t="inlineStr">
@@ -4014,7 +4026,7 @@
       </c>
       <c r="H47" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>future-scope</t>
         </is>
       </c>
       <c r="I47" s="54" t="inlineStr">
@@ -4024,33 +4036,29 @@
       </c>
       <c r="J47" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>future-scope</t>
         </is>
       </c>
       <c r="K47" s="54" t="inlineStr">
         <is>
-          <t>اختبار Domain/Service مع Clock قابل للحقن يثبت تاريخ الاستحقاق قبل/بعد نقطة زمنية اصطناعية | اختبار idempotency يمنع تسجيل الإهلاك نفسه مرتين عند إعادة تشغيل الساعة/الفعل | اختبار DOM يثبت أن الإهلاك غير النقدي لا يخصم من الكاش ويعرض الحالة الصادقة | اختبار export/import يحافظ على أصل الإهلاك وتاريخه إن دخلت البيانات الدائمة | دليل CI وMerge SHA وverified_on_main_sha قبل VERIFIED</t>
+          <t>Source/report comparison | Explicit unknowns and limits | Owner decision or pilot evidence</t>
         </is>
       </c>
       <c r="L47" s="54" t="inlineStr"/>
-      <c r="M47" s="54" t="inlineStr">
-        <is>
-          <t>تحديد نافذة اختبار الإهلاك أو آلية ساعة اختبار معتمدة قبل فتح Claim.</t>
-        </is>
-      </c>
+      <c r="M47" s="54" t="inlineStr"/>
       <c r="N47" s="54" t="inlineStr">
         <is>
-          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
       <c r="O47" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="P47" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q47" s="54" t="inlineStr">
@@ -4062,17 +4070,17 @@
     <row r="48">
       <c r="A48" s="54" t="inlineStr">
         <is>
-          <t>OPS-003</t>
+          <t>UX-002</t>
         </is>
       </c>
       <c r="B48" s="54" t="inlineStr">
         <is>
-          <t>المصروفات المتكررة المحلية</t>
+          <t>Backlog الموجة الرابعة في عقد الملكية</t>
         </is>
       </c>
       <c r="C48" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D48" s="54" t="inlineStr">
@@ -4082,12 +4090,12 @@
       </c>
       <c r="E48" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>FUTURE_SCOPE</t>
         </is>
       </c>
       <c r="F48" s="54" t="inlineStr">
         <is>
-          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
+          <t>OUT_OF_SCOPE</t>
         </is>
       </c>
       <c r="G48" s="54" t="inlineStr">
@@ -4097,7 +4105,7 @@
       </c>
       <c r="H48" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>post-pilot-gate</t>
         </is>
       </c>
       <c r="I48" s="54" t="inlineStr">
@@ -4107,37 +4115,29 @@
       </c>
       <c r="J48" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>post-pilot</t>
         </is>
       </c>
       <c r="K48" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
-        </is>
-      </c>
-      <c r="L48" s="54" t="inlineStr">
-        <is>
-          <t>CTRL-001</t>
-        </is>
-      </c>
-      <c r="M48" s="54" t="inlineStr">
-        <is>
-          <t>اعتماد أن المصروف المتكرر تذكير يحتاج تأكيدًا ولا ينشئ حدثًا ماليًا تلقائيًا.</t>
-        </is>
-      </c>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
+        </is>
+      </c>
+      <c r="L48" s="54" t="inlineStr"/>
+      <c r="M48" s="54" t="inlineStr"/>
       <c r="N48" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
       <c r="O48" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="P48" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q48" s="54" t="inlineStr">
@@ -4149,12 +4149,12 @@
     <row r="49">
       <c r="A49" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-002</t>
+          <t>V-001</t>
         </is>
       </c>
       <c r="B49" s="54" t="inlineStr">
         <is>
-          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
+          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
         </is>
       </c>
       <c r="C49" s="54" t="inlineStr">
@@ -4169,12 +4169,12 @@
       </c>
       <c r="E49" s="54" t="inlineStr">
         <is>
-          <t>FUTURE_SCOPE</t>
+          <t>PILOT_VALIDATION</t>
         </is>
       </c>
       <c r="F49" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE</t>
+          <t>PILOT_EVIDENCE_REQUIRED</t>
         </is>
       </c>
       <c r="G49" s="54" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="H49" s="54" t="inlineStr">
         <is>
-          <t>future-scope</t>
+          <t>pilot-validation</t>
         </is>
       </c>
       <c r="I49" s="54" t="inlineStr">
@@ -4194,24 +4194,24 @@
       </c>
       <c r="J49" s="54" t="inlineStr">
         <is>
-          <t>future-scope</t>
+          <t>pilot-validation</t>
         </is>
       </c>
       <c r="K49" s="54" t="inlineStr">
         <is>
-          <t>Source/report comparison | Explicit unknowns and limits | Owner decision or pilot evidence</t>
+          <t>Pilot observation protocol | Evidence log with denominator and outcome | Owner decision before any Feature claim</t>
         </is>
       </c>
       <c r="L49" s="54" t="inlineStr"/>
       <c r="M49" s="54" t="inlineStr"/>
       <c r="N49" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
       <c r="O49" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="P49" s="54" t="inlineStr">
@@ -4228,17 +4228,17 @@
     <row r="50">
       <c r="A50" s="54" t="inlineStr">
         <is>
-          <t>UX-002</t>
+          <t>V-002</t>
         </is>
       </c>
       <c r="B50" s="54" t="inlineStr">
         <is>
-          <t>Backlog الموجة الرابعة في عقد الملكية</t>
+          <t>V-02 — متوقعات الكاش القصيرة</t>
         </is>
       </c>
       <c r="C50" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>RESEARCH</t>
         </is>
       </c>
       <c r="D50" s="54" t="inlineStr">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="E50" s="54" t="inlineStr">
         <is>
-          <t>FUTURE_SCOPE</t>
+          <t>PILOT_VALIDATION</t>
         </is>
       </c>
       <c r="F50" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE</t>
+          <t>PILOT_EVIDENCE_REQUIRED</t>
         </is>
       </c>
       <c r="G50" s="54" t="inlineStr">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="H50" s="54" t="inlineStr">
         <is>
-          <t>post-pilot-gate</t>
+          <t>pilot-validation</t>
         </is>
       </c>
       <c r="I50" s="54" t="inlineStr">
@@ -4273,24 +4273,24 @@
       </c>
       <c r="J50" s="54" t="inlineStr">
         <is>
-          <t>post-pilot</t>
+          <t>pilot-validation</t>
         </is>
       </c>
       <c r="K50" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
+          <t>Pilot observation protocol | Evidence log with denominator and outcome | Owner decision before any Feature claim</t>
         </is>
       </c>
       <c r="L50" s="54" t="inlineStr"/>
       <c r="M50" s="54" t="inlineStr"/>
       <c r="N50" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
       <c r="O50" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="P50" s="54" t="inlineStr">
@@ -4307,12 +4307,12 @@
     <row r="51">
       <c r="A51" s="54" t="inlineStr">
         <is>
-          <t>V-001</t>
+          <t>V-003</t>
         </is>
       </c>
       <c r="B51" s="54" t="inlineStr">
         <is>
-          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
+          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
         </is>
       </c>
       <c r="C51" s="54" t="inlineStr">
@@ -4386,12 +4386,12 @@
     <row r="52">
       <c r="A52" s="54" t="inlineStr">
         <is>
-          <t>V-002</t>
+          <t>V-004</t>
         </is>
       </c>
       <c r="B52" s="54" t="inlineStr">
         <is>
-          <t>V-02 — متوقعات الكاش القصيرة</t>
+          <t>V-04 — عرض التغطية عند قرار السحب</t>
         </is>
       </c>
       <c r="C52" s="54" t="inlineStr">
@@ -4465,12 +4465,12 @@
     <row r="53">
       <c r="A53" s="54" t="inlineStr">
         <is>
-          <t>V-003</t>
+          <t>V-005</t>
         </is>
       </c>
       <c r="B53" s="54" t="inlineStr">
         <is>
-          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
+          <t>V-05 — مقارنة فترتين بسيطة</t>
         </is>
       </c>
       <c r="C53" s="54" t="inlineStr">
@@ -4544,12 +4544,12 @@
     <row r="54">
       <c r="A54" s="54" t="inlineStr">
         <is>
-          <t>V-004</t>
+          <t>V-006</t>
         </is>
       </c>
       <c r="B54" s="54" t="inlineStr">
         <is>
-          <t>V-04 — عرض التغطية عند قرار السحب</t>
+          <t>V-06 — جسر ربح إلى كاش رقمي</t>
         </is>
       </c>
       <c r="C54" s="54" t="inlineStr">
@@ -4623,12 +4623,12 @@
     <row r="55">
       <c r="A55" s="54" t="inlineStr">
         <is>
-          <t>V-005</t>
+          <t>V-007</t>
         </is>
       </c>
       <c r="B55" s="54" t="inlineStr">
         <is>
-          <t>V-05 — مقارنة فترتين بسيطة</t>
+          <t>V-07 — تنبيه انخفاض المواد</t>
         </is>
       </c>
       <c r="C55" s="54" t="inlineStr">
@@ -4702,12 +4702,12 @@
     <row r="56">
       <c r="A56" s="54" t="inlineStr">
         <is>
-          <t>V-006</t>
+          <t>V-008</t>
         </is>
       </c>
       <c r="B56" s="54" t="inlineStr">
         <is>
-          <t>V-06 — جسر ربح إلى كاش رقمي</t>
+          <t>V-08 — مصروف اليوم على الرئيسية</t>
         </is>
       </c>
       <c r="C56" s="54" t="inlineStr">
@@ -4781,12 +4781,12 @@
     <row r="57">
       <c r="A57" s="54" t="inlineStr">
         <is>
-          <t>V-007</t>
+          <t>V-009</t>
         </is>
       </c>
       <c r="B57" s="54" t="inlineStr">
         <is>
-          <t>V-07 — تنبيه انخفاض المواد</t>
+          <t>V-09 — رقم السحب الآمن الموحد</t>
         </is>
       </c>
       <c r="C57" s="54" t="inlineStr">
@@ -4860,12 +4860,12 @@
     <row r="58">
       <c r="A58" s="54" t="inlineStr">
         <is>
-          <t>V-008</t>
+          <t>V-010</t>
         </is>
       </c>
       <c r="B58" s="54" t="inlineStr">
         <is>
-          <t>V-08 — مصروف اليوم على الرئيسية</t>
+          <t>V-10 — كثافة صفحة المالية</t>
         </is>
       </c>
       <c r="C58" s="54" t="inlineStr">
@@ -4939,12 +4939,12 @@
     <row r="59">
       <c r="A59" s="54" t="inlineStr">
         <is>
-          <t>V-009</t>
+          <t>V-011</t>
         </is>
       </c>
       <c r="B59" s="54" t="inlineStr">
         <is>
-          <t>V-09 — رقم السحب الآمن الموحد</t>
+          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
         </is>
       </c>
       <c r="C59" s="54" t="inlineStr">
@@ -5018,12 +5018,12 @@
     <row r="60">
       <c r="A60" s="54" t="inlineStr">
         <is>
-          <t>V-010</t>
+          <t>V-012</t>
         </is>
       </c>
       <c r="B60" s="54" t="inlineStr">
         <is>
-          <t>V-10 — كثافة صفحة المالية</t>
+          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
         </is>
       </c>
       <c r="C60" s="54" t="inlineStr">
@@ -5097,42 +5097,42 @@
     <row r="61">
       <c r="A61" s="54" t="inlineStr">
         <is>
-          <t>V-011</t>
+          <t>CTRL-001</t>
         </is>
       </c>
       <c r="B61" s="54" t="inlineStr">
         <is>
-          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
+          <t>اعتماد Operations Control v2</t>
         </is>
       </c>
       <c r="C61" s="54" t="inlineStr">
         <is>
-          <t>RESEARCH</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="D61" s="54" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E61" s="54" t="inlineStr">
         <is>
-          <t>PILOT_VALIDATION</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="F61" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED</t>
+          <t>NOT_APPLICABLE</t>
         </is>
       </c>
       <c r="G61" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H61" s="54" t="inlineStr">
         <is>
-          <t>pilot-validation</t>
+          <t>stage-0</t>
         </is>
       </c>
       <c r="I61" s="54" t="inlineStr">
@@ -5142,29 +5142,29 @@
       </c>
       <c r="J61" s="54" t="inlineStr">
         <is>
-          <t>pilot-validation</t>
+          <t>governance, documentation</t>
         </is>
       </c>
       <c r="K61" s="54" t="inlineStr">
         <is>
-          <t>Pilot observation protocol | Evidence log with denominator and outcome | Owner decision before any Feature claim</t>
+          <t>Validator/schema test | Generated-view freshness check | Owner review evidence</t>
         </is>
       </c>
       <c r="L61" s="54" t="inlineStr"/>
-      <c r="M61" s="54" t="inlineStr"/>
+      <c r="M61" s="54" t="inlineStr">
+        <is>
+          <t>تم اعتماد الإغلاق بعد دمج PR #188 والتحقق من main؛ لا يفتح Claim كودي بهذا السجل.</t>
+        </is>
+      </c>
       <c r="N61" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-      <c r="O61" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
+          <t>لا إجراء؛ سجل Operations Control v2 مدموج ومثبت على main. التنفيذ التالي يبدأ من G-001..G-006 في Claim مستقل.</t>
+        </is>
+      </c>
+      <c r="O61" s="54" t="inlineStr"/>
       <c r="P61" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q61" s="54" t="inlineStr">
@@ -5176,42 +5176,42 @@
     <row r="62">
       <c r="A62" s="54" t="inlineStr">
         <is>
-          <t>V-012</t>
+          <t>CTRL-002</t>
         </is>
       </c>
       <c r="B62" s="54" t="inlineStr">
         <is>
-          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
+          <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
         </is>
       </c>
       <c r="C62" s="54" t="inlineStr">
         <is>
-          <t>RESEARCH</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="D62" s="54" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E62" s="54" t="inlineStr">
         <is>
-          <t>PILOT_VALIDATION</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="F62" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED</t>
+          <t>EVIDENCE_RECONCILIATION_REQUIRED</t>
         </is>
       </c>
       <c r="G62" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H62" s="54" t="inlineStr">
         <is>
-          <t>pilot-validation</t>
+          <t>stage-0</t>
         </is>
       </c>
       <c r="I62" s="54" t="inlineStr">
@@ -5221,29 +5221,29 @@
       </c>
       <c r="J62" s="54" t="inlineStr">
         <is>
-          <t>pilot-validation</t>
+          <t>governance, documentation</t>
         </is>
       </c>
       <c r="K62" s="54" t="inlineStr">
         <is>
-          <t>Pilot observation protocol | Evidence log with denominator and outcome | Owner decision before any Feature claim</t>
+          <t>Validator/schema test | Generated-view freshness check | Owner review evidence</t>
         </is>
       </c>
       <c r="L62" s="54" t="inlineStr"/>
-      <c r="M62" s="54" t="inlineStr"/>
+      <c r="M62" s="54" t="inlineStr">
+        <is>
+          <t>تم اعتماد الإغلاق بعد دمج PR #188 والتحقق من main؛ لا يفتح Claim كودي بهذا السجل.</t>
+        </is>
+      </c>
       <c r="N62" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-      <c r="O62" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
+          <t>لا إجراء؛ المصالحة والبوابات مدموجة ومثبتة. لا تبدأ معالجة 49/46 أو Claim كودي جديد دون دليل جديد.</t>
+        </is>
+      </c>
+      <c r="O62" s="54" t="inlineStr"/>
       <c r="P62" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q62" s="54" t="inlineStr">
@@ -6217,7 +6217,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6232,7 +6232,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="B5" s="53" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C5" s="53" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="F5" s="53" t="inlineStr">
         <is>
-          <t>مراجعة المالك وAgent مستقل؛ لا دمج قبل قبول الملاحظات.</t>
+          <t>لا إجراء؛ Workstream التوثيقي مغلق. يبدأ أي تنفيذ لاحق في Workstream مستقل من G-001..G-006.</t>
         </is>
       </c>
     </row>
@@ -6718,7 +6718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6774,221 +6774,271 @@
     <row r="5">
       <c r="A5" s="53" t="inlineStr">
         <is>
+          <t>CTRL-001</t>
+        </is>
+      </c>
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t>اعتماد Operations Control v2</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="inlineStr">
+        <is>
+          <t>e75419504d61a60141c1776a5bfa69ed1faeb529</t>
+        </is>
+      </c>
+      <c r="D5" s="53" t="inlineStr">
+        <is>
+          <t>docs/operations/control/README.md
+https://github.com/Qays7753/Micro/pull/188
+docs/operations/control/generated/MASTER-TRACKER.md
+docs/operations/control/generated/MASTER-TRACKER.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t>CTRL-002</t>
+        </is>
+      </c>
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>e75419504d61a60141c1776a5bfa69ed1faeb529</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="inlineStr">
+        <is>
+          <t>docs/operations/control/migration-map.md
+docs/operations/control/evidence/capability-reconciliation.md
+https://github.com/Qays7753/Micro/pull/188
+docs/operations/control/releases/pre-pilot.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="54" t="inlineStr">
+        <is>
           <t>HARD-009</t>
         </is>
       </c>
-      <c r="B5" s="53" t="inlineStr">
+      <c r="B7" s="54" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 9</t>
         </is>
       </c>
-      <c r="C5" s="53" t="inlineStr">
+      <c r="C7" s="54" t="inlineStr">
         <is>
           <t>255974a8cf66674e0a3dba477da9d9400cb28306</t>
         </is>
       </c>
-      <c r="D5" s="53" t="inlineStr">
+      <c r="D7" s="54" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="54" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="53" t="inlineStr">
         <is>
           <t>HARD-010</t>
         </is>
       </c>
-      <c r="B6" s="54" t="inlineStr">
+      <c r="B8" s="53" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 10</t>
         </is>
       </c>
-      <c r="C6" s="54" t="inlineStr">
+      <c r="C8" s="53" t="inlineStr">
         <is>
           <t>dcf60dbed79c09a06a46fcbad07e104277cb17de</t>
         </is>
       </c>
-      <c r="D6" s="54" t="inlineStr">
+      <c r="D8" s="53" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="54" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="54" t="inlineStr">
         <is>
           <t>HARD-011</t>
         </is>
       </c>
-      <c r="B7" s="54" t="inlineStr">
+      <c r="B9" s="54" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 11</t>
         </is>
       </c>
-      <c r="C7" s="54" t="inlineStr">
+      <c r="C9" s="54" t="inlineStr">
         <is>
           <t>79dac8e726b3cf5e682cb912b90d7c3757636f71</t>
         </is>
       </c>
-      <c r="D7" s="54" t="inlineStr">
+      <c r="D9" s="54" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="53" t="inlineStr">
-        <is>
-          <t>HIST-001</t>
-        </is>
-      </c>
-      <c r="B8" s="53" t="inlineStr">
-        <is>
-          <t>الموجة الأولى: إصلاحات حرجة محددة</t>
-        </is>
-      </c>
-      <c r="C8" s="53" t="inlineStr">
-        <is>
-          <t>5c54d8a</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="inlineStr">
-        <is>
-          <t>docs/operations/current-state.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
-        <is>
-          <t>HIST-002</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>الموجة الثانية: الأساسات المالية والبيانية</t>
-        </is>
-      </c>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>81d8d253984dee410c7fd6c3e461fcd0e76f327e</t>
-        </is>
-      </c>
-      <c r="D9" s="54" t="inlineStr">
-        <is>
-          <t>reports/agent-report/2026-09-17_wave-2-financial-data-foundations/report.md</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>HIST-007</t>
+          <t>HIST-001</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>الموجة 4.4: الجودة النظامية والقبول المحلي</t>
+          <t>الموجة الأولى: إصلاحات حرجة محددة</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>87ebcf2ffa74752bf385eff3a10962454b45d33e</t>
+          <t>5c54d8a</t>
         </is>
       </c>
       <c r="D10" s="54" t="inlineStr">
         <is>
-          <t>reports/agent-report/2026-09-18_wave-4-4-system-quality-final-qa/report.md</t>
+          <t>docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>HIST-003</t>
+          <t>HIST-002</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>الموجة الثالثة: العقود والملكية التقنية</t>
+          <t>الموجة الثانية: الأساسات المالية والبيانية</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t>f8b37062c14aecf85abf5f64e11a191b00eb3c0d</t>
+          <t>81d8d253984dee410c7fd6c3e461fcd0e76f327e</t>
         </is>
       </c>
       <c r="D11" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/current-state.md</t>
+          <t>reports/agent-report/2026-09-17_wave-2-financial-data-foundations/report.md</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="54" t="inlineStr">
         <is>
-          <t>HIST-004</t>
+          <t>HIST-007</t>
         </is>
       </c>
       <c r="B12" s="54" t="inlineStr">
         <is>
-          <t>الموجة 4.1: مخطط تجربة المنتج</t>
+          <t>الموجة 4.4: الجودة النظامية والقبول المحلي</t>
         </is>
       </c>
       <c r="C12" s="54" t="inlineStr">
         <is>
-          <t>281a2878b61870792f76d651d0d822c7f0a5c0e1</t>
+          <t>87ebcf2ffa74752bf385eff3a10962454b45d33e</t>
         </is>
       </c>
       <c r="D12" s="54" t="inlineStr">
         <is>
-          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
+          <t>reports/agent-report/2026-09-18_wave-4-4-system-quality-final-qa/report.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="54" t="inlineStr">
         <is>
-          <t>HIST-005</t>
+          <t>HIST-003</t>
         </is>
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>الموجة 4.2: الهيكل والتنقل والتسمية</t>
+          <t>الموجة الثالثة: العقود والملكية التقنية</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">
         <is>
-          <t>9179ea785d7c35790c422a997fa210aaf7e875a6</t>
+          <t>f8b37062c14aecf85abf5f64e11a191b00eb3c0d</t>
         </is>
       </c>
       <c r="D13" s="54" t="inlineStr">
         <is>
-          <t>reports/agent-report/2026-09-17_wave-4-2-structure-navigation-naming/report.md</t>
+          <t>docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="54" t="inlineStr">
         <is>
+          <t>HIST-004</t>
+        </is>
+      </c>
+      <c r="B14" s="54" t="inlineStr">
+        <is>
+          <t>الموجة 4.1: مخطط تجربة المنتج</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>281a2878b61870792f76d651d0d822c7f0a5c0e1</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="54" t="inlineStr">
+        <is>
+          <t>HIST-005</t>
+        </is>
+      </c>
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>الموجة 4.2: الهيكل والتنقل والتسمية</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>9179ea785d7c35790c422a997fa210aaf7e875a6</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-17_wave-4-2-structure-navigation-naming/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="54" t="inlineStr">
+        <is>
           <t>HIST-006</t>
         </is>
       </c>
-      <c r="B14" s="54" t="inlineStr">
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>الموجة 4.3: إعادة بناء أسطح المنتج</t>
         </is>
       </c>
-      <c r="C14" s="54" t="inlineStr">
+      <c r="C16" s="54" t="inlineStr">
         <is>
           <t>e8a7b5a5f6678a4a93e3ab4c21814764f5895335</t>
         </is>
       </c>
-      <c r="D14" s="54" t="inlineStr">
+      <c r="D16" s="54" t="inlineStr">
         <is>
           <t>docs/operations/current-state.md</t>
         </is>
@@ -7008,7 +7058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7154,61 +7204,57 @@
     <row r="8">
       <c r="A8" s="53" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
+          <t>G-001</t>
         </is>
       </c>
       <c r="B8" s="53" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="C8" s="53" t="inlineStr">
         <is>
-          <t>اعتماد Operations Control v2</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="inlineStr">
-        <is>
-          <t>اعتماد النظام بعد مراجعة المالك وAgent مستقل.</t>
-        </is>
-      </c>
+          <t>فخ الاستهلاك المزدوج عند التسليم</t>
+        </is>
+      </c>
+      <c r="D8" s="53" t="inlineStr"/>
       <c r="E8" s="53" t="inlineStr">
         <is>
-          <t>استكمل مراجعة المالك والمراجع المستقل ثم حدّث الحالة في PR نفسه.</t>
+          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="54" t="inlineStr">
         <is>
-          <t>CTRL-002</t>
+          <t>GOV-001</t>
         </is>
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
         <is>
-          <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
+          <t>مصالحة G10-A مع تعارض عقد C1</t>
         </is>
       </c>
       <c r="D9" s="54" t="inlineStr">
         <is>
-          <t>تسجيل تعريف العد ومراجعة الأدلة؛ لا يجوز حسم فرق 49/46 بقرار وصفي بلا مصفوفة مصادر.</t>
+          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
         </is>
       </c>
       <c r="E9" s="54" t="inlineStr">
         <is>
-          <t>أرفق مصفوفة الأدلة التي تحسم تعريف 49/46 ومسارات القدرة، ثم اطلب مراجعة المالك قبل فتح أي Claim كودي.</t>
+          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>G-001</t>
+          <t>G-002</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
@@ -7218,20 +7264,20 @@
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>فخ الاستهلاك المزدوج عند التسليم</t>
+          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
         </is>
       </c>
       <c r="D10" s="54" t="inlineStr"/>
       <c r="E10" s="54" t="inlineStr">
         <is>
-          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
+          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>GOV-001</t>
+          <t>G-003</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
@@ -7241,24 +7287,20 @@
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t>مصالحة G10-A مع تعارض عقد C1</t>
-        </is>
-      </c>
-      <c r="D11" s="54" t="inlineStr">
-        <is>
-          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
-        </is>
-      </c>
+          <t>حرس القراءة القديمة عند حفظ الطلب</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="inlineStr"/>
       <c r="E11" s="54" t="inlineStr">
         <is>
-          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
+          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="54" t="inlineStr">
         <is>
-          <t>G-002</t>
+          <t>G-004</t>
         </is>
       </c>
       <c r="B12" s="54" t="inlineStr">
@@ -7268,20 +7310,20 @@
       </c>
       <c r="C12" s="54" t="inlineStr">
         <is>
-          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
+          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
         </is>
       </c>
       <c r="D12" s="54" t="inlineStr"/>
       <c r="E12" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
+          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="54" t="inlineStr">
         <is>
-          <t>G-003</t>
+          <t>G-005</t>
         </is>
       </c>
       <c r="B13" s="54" t="inlineStr">
@@ -7291,20 +7333,20 @@
       </c>
       <c r="C13" s="54" t="inlineStr">
         <is>
-          <t>حرس القراءة القديمة عند حفظ الطلب</t>
+          <t>عزل فشل قراءات صفحة المالية</t>
         </is>
       </c>
       <c r="D13" s="54" t="inlineStr"/>
       <c r="E13" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
+          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="54" t="inlineStr">
         <is>
-          <t>G-004</t>
+          <t>G-006</t>
         </is>
       </c>
       <c r="B14" s="54" t="inlineStr">
@@ -7314,66 +7356,74 @@
       </c>
       <c r="C14" s="54" t="inlineStr">
         <is>
-          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
+          <t>توحيد حرس السحب بين مساري مال المالك</t>
         </is>
       </c>
       <c r="D14" s="54" t="inlineStr"/>
       <c r="E14" s="54" t="inlineStr">
         <is>
-          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
+          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="54" t="inlineStr">
         <is>
-          <t>G-005</t>
+          <t>SCOPE-001</t>
         </is>
       </c>
       <c r="B15" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C15" s="54" t="inlineStr">
         <is>
-          <t>عزل فشل قراءات صفحة المالية</t>
-        </is>
-      </c>
-      <c r="D15" s="54" t="inlineStr"/>
+          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+        </is>
+      </c>
       <c r="E15" s="54" t="inlineStr">
         <is>
-          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="54" t="inlineStr">
         <is>
-          <t>G-006</t>
+          <t>UX-001</t>
         </is>
       </c>
       <c r="B16" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C16" s="54" t="inlineStr">
         <is>
-          <t>توحيد حرس السحب بين مساري مال المالك</t>
-        </is>
-      </c>
-      <c r="D16" s="54" t="inlineStr"/>
+          <t>إعادة تصميم UI وUX جذرية</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="inlineStr">
+        <is>
+          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+        </is>
+      </c>
       <c r="E16" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
+          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-001</t>
+          <t>BE-001</t>
         </is>
       </c>
       <c r="B17" s="54" t="inlineStr">
@@ -7383,24 +7433,24 @@
       </c>
       <c r="C17" s="54" t="inlineStr">
         <is>
-          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
+          <t>مصاريف متكررة محلية</t>
         </is>
       </c>
       <c r="D17" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
         </is>
       </c>
       <c r="E17" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="54" t="inlineStr">
         <is>
-          <t>UX-001</t>
+          <t>BE-002</t>
         </is>
       </c>
       <c r="B18" s="54" t="inlineStr">
@@ -7410,24 +7460,24 @@
       </c>
       <c r="C18" s="54" t="inlineStr">
         <is>
-          <t>إعادة تصميم UI وUX جذرية</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="D18" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
         </is>
       </c>
       <c r="E18" s="54" t="inlineStr">
         <is>
-          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="54" t="inlineStr">
         <is>
-          <t>BE-001</t>
+          <t>BE-003</t>
         </is>
       </c>
       <c r="B19" s="54" t="inlineStr">
@@ -7437,7 +7487,7 @@
       </c>
       <c r="C19" s="54" t="inlineStr">
         <is>
-          <t>مصاريف متكررة محلية</t>
+          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="D19" s="54" t="inlineStr">
@@ -7447,14 +7497,14 @@
       </c>
       <c r="E19" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="54" t="inlineStr">
         <is>
-          <t>BE-002</t>
+          <t>BE-004</t>
         </is>
       </c>
       <c r="B20" s="54" t="inlineStr">
@@ -7464,24 +7514,24 @@
       </c>
       <c r="C20" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>إغلاق فترة رسمي</t>
         </is>
       </c>
       <c r="D20" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="E20" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="54" t="inlineStr">
         <is>
-          <t>BE-003</t>
+          <t>BE-005</t>
         </is>
       </c>
       <c r="B21" s="54" t="inlineStr">
@@ -7491,24 +7541,24 @@
       </c>
       <c r="C21" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
+          <t>تقادم الديون بشرائح 30/60/90</t>
         </is>
       </c>
       <c r="D21" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="E21" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="54" t="inlineStr">
         <is>
-          <t>BE-004</t>
+          <t>FIN-002</t>
         </is>
       </c>
       <c r="B22" s="54" t="inlineStr">
@@ -7518,24 +7568,24 @@
       </c>
       <c r="C22" s="54" t="inlineStr">
         <is>
-          <t>إغلاق فترة رسمي</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="D22" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="E22" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="54" t="inlineStr">
         <is>
-          <t>BE-005</t>
+          <t>FIN-006</t>
         </is>
       </c>
       <c r="B23" s="54" t="inlineStr">
@@ -7545,24 +7595,24 @@
       </c>
       <c r="C23" s="54" t="inlineStr">
         <is>
-          <t>تقادم الديون بشرائح 30/60/90</t>
+          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="D23" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="E23" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="54" t="inlineStr">
         <is>
-          <t>FIN-002</t>
+          <t>FIN-008</t>
         </is>
       </c>
       <c r="B24" s="54" t="inlineStr">
@@ -7572,24 +7622,24 @@
       </c>
       <c r="C24" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>تحقق الإهلاك بعد مرور الزمن</t>
         </is>
       </c>
       <c r="D24" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
         </is>
       </c>
       <c r="E24" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
+          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="54" t="inlineStr">
         <is>
-          <t>FIN-006</t>
+          <t>OPS-003</t>
         </is>
       </c>
       <c r="B25" s="54" t="inlineStr">
@@ -7599,24 +7649,24 @@
       </c>
       <c r="C25" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
+          <t>المصروفات المتكررة المحلية</t>
         </is>
       </c>
       <c r="D25" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
         </is>
       </c>
       <c r="E25" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="54" t="inlineStr">
         <is>
-          <t>FIN-008</t>
+          <t>SCOPE-002</t>
         </is>
       </c>
       <c r="B26" s="54" t="inlineStr">
@@ -7626,24 +7676,24 @@
       </c>
       <c r="C26" s="54" t="inlineStr">
         <is>
-          <t>تحقق الإهلاك بعد مرور الزمن</t>
+          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
         </is>
       </c>
       <c r="D26" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="E26" s="54" t="inlineStr">
         <is>
-          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="54" t="inlineStr">
         <is>
-          <t>OPS-003</t>
+          <t>UX-002</t>
         </is>
       </c>
       <c r="B27" s="54" t="inlineStr">
@@ -7653,24 +7703,24 @@
       </c>
       <c r="C27" s="54" t="inlineStr">
         <is>
-          <t>المصروفات المتكررة المحلية</t>
+          <t>Backlog الموجة الرابعة في عقد الملكية</t>
         </is>
       </c>
       <c r="D27" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="E27" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-002</t>
+          <t>V-001</t>
         </is>
       </c>
       <c r="B28" s="54" t="inlineStr">
@@ -7680,24 +7730,24 @@
       </c>
       <c r="C28" s="54" t="inlineStr">
         <is>
-          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
+          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
         </is>
       </c>
       <c r="D28" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E28" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="54" t="inlineStr">
         <is>
-          <t>UX-002</t>
+          <t>V-002</t>
         </is>
       </c>
       <c r="B29" s="54" t="inlineStr">
@@ -7707,24 +7757,24 @@
       </c>
       <c r="C29" s="54" t="inlineStr">
         <is>
-          <t>Backlog الموجة الرابعة في عقد الملكية</t>
+          <t>V-02 — متوقعات الكاش القصيرة</t>
         </is>
       </c>
       <c r="D29" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E29" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="54" t="inlineStr">
         <is>
-          <t>V-001</t>
+          <t>V-003</t>
         </is>
       </c>
       <c r="B30" s="54" t="inlineStr">
@@ -7734,7 +7784,7 @@
       </c>
       <c r="C30" s="54" t="inlineStr">
         <is>
-          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
+          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
         </is>
       </c>
       <c r="D30" s="54" t="inlineStr">
@@ -7751,7 +7801,7 @@
     <row r="31">
       <c r="A31" s="54" t="inlineStr">
         <is>
-          <t>V-002</t>
+          <t>V-004</t>
         </is>
       </c>
       <c r="B31" s="54" t="inlineStr">
@@ -7761,7 +7811,7 @@
       </c>
       <c r="C31" s="54" t="inlineStr">
         <is>
-          <t>V-02 — متوقعات الكاش القصيرة</t>
+          <t>V-04 — عرض التغطية عند قرار السحب</t>
         </is>
       </c>
       <c r="D31" s="54" t="inlineStr">
@@ -7778,7 +7828,7 @@
     <row r="32">
       <c r="A32" s="54" t="inlineStr">
         <is>
-          <t>V-003</t>
+          <t>V-005</t>
         </is>
       </c>
       <c r="B32" s="54" t="inlineStr">
@@ -7788,7 +7838,7 @@
       </c>
       <c r="C32" s="54" t="inlineStr">
         <is>
-          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
+          <t>V-05 — مقارنة فترتين بسيطة</t>
         </is>
       </c>
       <c r="D32" s="54" t="inlineStr">
@@ -7805,7 +7855,7 @@
     <row r="33">
       <c r="A33" s="54" t="inlineStr">
         <is>
-          <t>V-004</t>
+          <t>V-006</t>
         </is>
       </c>
       <c r="B33" s="54" t="inlineStr">
@@ -7815,7 +7865,7 @@
       </c>
       <c r="C33" s="54" t="inlineStr">
         <is>
-          <t>V-04 — عرض التغطية عند قرار السحب</t>
+          <t>V-06 — جسر ربح إلى كاش رقمي</t>
         </is>
       </c>
       <c r="D33" s="54" t="inlineStr">
@@ -7832,7 +7882,7 @@
     <row r="34">
       <c r="A34" s="54" t="inlineStr">
         <is>
-          <t>V-005</t>
+          <t>V-007</t>
         </is>
       </c>
       <c r="B34" s="54" t="inlineStr">
@@ -7842,7 +7892,7 @@
       </c>
       <c r="C34" s="54" t="inlineStr">
         <is>
-          <t>V-05 — مقارنة فترتين بسيطة</t>
+          <t>V-07 — تنبيه انخفاض المواد</t>
         </is>
       </c>
       <c r="D34" s="54" t="inlineStr">
@@ -7859,7 +7909,7 @@
     <row r="35">
       <c r="A35" s="54" t="inlineStr">
         <is>
-          <t>V-006</t>
+          <t>V-008</t>
         </is>
       </c>
       <c r="B35" s="54" t="inlineStr">
@@ -7869,7 +7919,7 @@
       </c>
       <c r="C35" s="54" t="inlineStr">
         <is>
-          <t>V-06 — جسر ربح إلى كاش رقمي</t>
+          <t>V-08 — مصروف اليوم على الرئيسية</t>
         </is>
       </c>
       <c r="D35" s="54" t="inlineStr">
@@ -7886,7 +7936,7 @@
     <row r="36">
       <c r="A36" s="54" t="inlineStr">
         <is>
-          <t>V-007</t>
+          <t>V-009</t>
         </is>
       </c>
       <c r="B36" s="54" t="inlineStr">
@@ -7896,7 +7946,7 @@
       </c>
       <c r="C36" s="54" t="inlineStr">
         <is>
-          <t>V-07 — تنبيه انخفاض المواد</t>
+          <t>V-09 — رقم السحب الآمن الموحد</t>
         </is>
       </c>
       <c r="D36" s="54" t="inlineStr">
@@ -7913,7 +7963,7 @@
     <row r="37">
       <c r="A37" s="54" t="inlineStr">
         <is>
-          <t>V-008</t>
+          <t>V-010</t>
         </is>
       </c>
       <c r="B37" s="54" t="inlineStr">
@@ -7923,7 +7973,7 @@
       </c>
       <c r="C37" s="54" t="inlineStr">
         <is>
-          <t>V-08 — مصروف اليوم على الرئيسية</t>
+          <t>V-10 — كثافة صفحة المالية</t>
         </is>
       </c>
       <c r="D37" s="54" t="inlineStr">
@@ -7940,7 +7990,7 @@
     <row r="38">
       <c r="A38" s="54" t="inlineStr">
         <is>
-          <t>V-009</t>
+          <t>V-011</t>
         </is>
       </c>
       <c r="B38" s="54" t="inlineStr">
@@ -7950,7 +8000,7 @@
       </c>
       <c r="C38" s="54" t="inlineStr">
         <is>
-          <t>V-09 — رقم السحب الآمن الموحد</t>
+          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
         </is>
       </c>
       <c r="D38" s="54" t="inlineStr">
@@ -7967,7 +8017,7 @@
     <row r="39">
       <c r="A39" s="54" t="inlineStr">
         <is>
-          <t>V-010</t>
+          <t>V-012</t>
         </is>
       </c>
       <c r="B39" s="54" t="inlineStr">
@@ -7977,7 +8027,7 @@
       </c>
       <c r="C39" s="54" t="inlineStr">
         <is>
-          <t>V-10 — كثافة صفحة المالية</t>
+          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
         </is>
       </c>
       <c r="D39" s="54" t="inlineStr">
@@ -7986,60 +8036,6 @@
         </is>
       </c>
       <c r="E39" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="54" t="inlineStr">
-        <is>
-          <t>V-011</t>
-        </is>
-      </c>
-      <c r="B40" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C40" s="54" t="inlineStr">
-        <is>
-          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
-        </is>
-      </c>
-      <c r="D40" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E40" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="54" t="inlineStr">
-        <is>
-          <t>V-012</t>
-        </is>
-      </c>
-      <c r="B41" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C41" s="54" t="inlineStr">
-        <is>
-          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
-        </is>
-      </c>
-      <c r="D41" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E41" s="54" t="inlineStr">
         <is>
           <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
@@ -8606,7 +8602,7 @@
       </c>
       <c r="B5" s="53" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C5" s="53" t="inlineStr">
@@ -8638,7 +8634,7 @@
       </c>
       <c r="B6" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C6" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs: close operations control review (#189)
Co-authored-by: Qays7753 <2.14180459e+08+Qays7753@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1214,68 +1214,72 @@
     <row r="12" ht="24" customHeight="1">
       <c r="A12" s="54" t="inlineStr">
         <is>
+          <t>FIN-001</t>
+        </is>
+      </c>
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>تسجيل اقتراض داخل المشروع</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>FEATURE</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="E12" s="54" t="inlineStr">
+        <is>
+          <t>FIX_BEFORE_PILOT</t>
+        </is>
+      </c>
+      <c r="F12" s="54" t="inlineStr">
+        <is>
+          <t>NOT_APPLICABLE</t>
+        </is>
+      </c>
+      <c r="G12" s="54" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H12" s="54" t="inlineStr">
+        <is>
+          <t>stage-3</t>
+        </is>
+      </c>
+      <c r="I12" s="54" t="inlineStr">
+        <is>
+          <t>Product owner / Manus coordination</t>
+        </is>
+      </c>
+      <c r="J12" s="54" t="inlineStr">
+        <is>
+          <t>Layer 3, domain, application, presentation</t>
+        </is>
+      </c>
+      <c r="K12" s="54" t="inlineStr">
+        <is>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L12" s="54" t="inlineStr">
+        <is>
           <t>CTRL-001</t>
         </is>
       </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>اعتماد Operations Control v2</t>
-        </is>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
-        <is>
-          <t>GOVERNANCE</t>
-        </is>
-      </c>
-      <c r="D12" s="54" t="inlineStr">
-        <is>
-          <t>IN_REVIEW</t>
-        </is>
-      </c>
-      <c r="E12" s="54" t="inlineStr">
-        <is>
-          <t>GOVERNANCE</t>
-        </is>
-      </c>
-      <c r="F12" s="54" t="inlineStr">
-        <is>
-          <t>NOT_APPLICABLE</t>
-        </is>
-      </c>
-      <c r="G12" s="54" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="H12" s="54" t="inlineStr">
-        <is>
-          <t>stage-0</t>
-        </is>
-      </c>
-      <c r="I12" s="54" t="inlineStr">
-        <is>
-          <t>Product owner / Manus coordination</t>
-        </is>
-      </c>
-      <c r="J12" s="54" t="inlineStr">
-        <is>
-          <t>governance, documentation</t>
-        </is>
-      </c>
-      <c r="K12" s="54" t="inlineStr">
-        <is>
-          <t>Validator/schema test | Generated-view freshness check | Owner review evidence</t>
-        </is>
-      </c>
-      <c r="L12" s="54" t="inlineStr"/>
       <c r="M12" s="54" t="inlineStr">
         <is>
-          <t>اعتماد النظام بعد مراجعة المالك وAgent مستقل.</t>
+          <t>اعتماد سياسة القرض المأخوذ: الكاش والالتزام والمحفظة والسداد وفصل الأصل عن الرسوم/الفوائد.</t>
         </is>
       </c>
       <c r="N12" s="54" t="inlineStr">
         <is>
-          <t>استكمل مراجعة المالك والمراجع المستقل ثم حدّث الحالة في PR نفسه.</t>
+          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O12" s="54" t="inlineStr"/>
@@ -1293,32 +1297,32 @@
     <row r="13" ht="24" customHeight="1">
       <c r="A13" s="54" t="inlineStr">
         <is>
-          <t>CTRL-002</t>
+          <t>FIN-003</t>
         </is>
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
+          <t>مقارنة الفترات وجسر الربح إلى الكاش</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">
         <is>
-          <t>GOVERNANCE</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D13" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="E13" s="54" t="inlineStr">
         <is>
-          <t>GOVERNANCE</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F13" s="54" t="inlineStr">
         <is>
-          <t>EVIDENCE_RECONCILIATION_REQUIRED</t>
+          <t>NOT_APPLICABLE</t>
         </is>
       </c>
       <c r="G13" s="54" t="inlineStr">
@@ -1328,7 +1332,7 @@
       </c>
       <c r="H13" s="54" t="inlineStr">
         <is>
-          <t>stage-0</t>
+          <t>stage-3</t>
         </is>
       </c>
       <c r="I13" s="54" t="inlineStr">
@@ -1338,23 +1342,23 @@
       </c>
       <c r="J13" s="54" t="inlineStr">
         <is>
-          <t>governance, documentation</t>
+          <t>Layer 3, domain, application, presentation</t>
         </is>
       </c>
       <c r="K13" s="54" t="inlineStr">
         <is>
-          <t>Validator/schema test | Generated-view freshness check | Owner review evidence</t>
-        </is>
-      </c>
-      <c r="L13" s="54" t="inlineStr"/>
-      <c r="M13" s="54" t="inlineStr">
-        <is>
-          <t>تسجيل تعريف العد ومراجعة الأدلة؛ لا يجوز حسم فرق 49/46 بقرار وصفي بلا مصفوفة مصادر.</t>
-        </is>
-      </c>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L13" s="54" t="inlineStr">
+        <is>
+          <t>FIN-001</t>
+        </is>
+      </c>
+      <c r="M13" s="54" t="inlineStr"/>
       <c r="N13" s="54" t="inlineStr">
         <is>
-          <t>أرفق مصفوفة الأدلة التي تحسم تعريف 49/46 ومسارات القدرة، ثم اطلب مراجعة المالك قبل فتح أي Claim كودي.</t>
+          <t>تحقق من الاعتماديات (FIN-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O13" s="54" t="inlineStr"/>
@@ -1372,12 +1376,12 @@
     <row r="14" ht="24" customHeight="1">
       <c r="A14" s="54" t="inlineStr">
         <is>
-          <t>FIN-001</t>
+          <t>FIN-004</t>
         </is>
       </c>
       <c r="B14" s="54" t="inlineStr">
         <is>
-          <t>تسجيل اقتراض داخل المشروع</t>
+          <t>حد السحب الآمن للمالك</t>
         </is>
       </c>
       <c r="C14" s="54" t="inlineStr">
@@ -1427,17 +1431,13 @@
       </c>
       <c r="L14" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
-        </is>
-      </c>
-      <c r="M14" s="54" t="inlineStr">
-        <is>
-          <t>اعتماد سياسة القرض المأخوذ: الكاش والالتزام والمحفظة والسداد وفصل الأصل عن الرسوم/الفوائد.</t>
-        </is>
-      </c>
+          <t>FIN-003, FIN-005</t>
+        </is>
+      </c>
+      <c r="M14" s="54" t="inlineStr"/>
       <c r="N14" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (FIN-003, FIN-005) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O14" s="54" t="inlineStr"/>
@@ -1455,12 +1455,12 @@
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="54" t="inlineStr">
         <is>
-          <t>FIN-003</t>
+          <t>FIN-005</t>
         </is>
       </c>
       <c r="B15" s="54" t="inlineStr">
         <is>
-          <t>مقارنة الفترات وجسر الربح إلى الكاش</t>
+          <t>توقع الكاش والتصريحات المتوقعة</t>
         </is>
       </c>
       <c r="C15" s="54" t="inlineStr">
@@ -1510,13 +1510,13 @@
       </c>
       <c r="L15" s="54" t="inlineStr">
         <is>
-          <t>FIN-001</t>
+          <t>OPS-001</t>
         </is>
       </c>
       <c r="M15" s="54" t="inlineStr"/>
       <c r="N15" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (FIN-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (OPS-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O15" s="54" t="inlineStr"/>
@@ -1534,12 +1534,12 @@
     <row r="16" ht="24" customHeight="1">
       <c r="A16" s="54" t="inlineStr">
         <is>
-          <t>FIN-004</t>
+          <t>OPS-001</t>
         </is>
       </c>
       <c r="B16" s="54" t="inlineStr">
         <is>
-          <t>حد السحب الآمن للمالك</t>
+          <t>المواعيد والاستحقاقات وتقادم الذمم الأساسي</t>
         </is>
       </c>
       <c r="C16" s="54" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H16" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I16" s="54" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="J16" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K16" s="54" t="inlineStr">
@@ -1589,13 +1589,13 @@
       </c>
       <c r="L16" s="54" t="inlineStr">
         <is>
-          <t>FIN-003, FIN-005</t>
+          <t>CTRL-001</t>
         </is>
       </c>
       <c r="M16" s="54" t="inlineStr"/>
       <c r="N16" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (FIN-003, FIN-005) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O16" s="54" t="inlineStr"/>
@@ -1613,12 +1613,12 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="54" t="inlineStr">
         <is>
-          <t>FIN-005</t>
+          <t>OPS-005</t>
         </is>
       </c>
       <c r="B17" s="54" t="inlineStr">
         <is>
-          <t>توقع الكاش والتصريحات المتوقعة</t>
+          <t>سطح قادم موحد للدفعات والتحصيلات والطلبات والالتزامات</t>
         </is>
       </c>
       <c r="C17" s="54" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="H17" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I17" s="54" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="J17" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K17" s="54" t="inlineStr">
@@ -1668,19 +1668,19 @@
       </c>
       <c r="L17" s="54" t="inlineStr">
         <is>
-          <t>OPS-001</t>
+          <t>CTRL-001, OPS-001</t>
         </is>
       </c>
       <c r="M17" s="54" t="inlineStr"/>
       <c r="N17" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (OPS-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
         </is>
       </c>
       <c r="O17" s="54" t="inlineStr"/>
       <c r="P17" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q17" s="54" t="inlineStr">
@@ -1692,17 +1692,17 @@
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="54" t="inlineStr">
         <is>
-          <t>OPS-001</t>
+          <t>OPS-009</t>
         </is>
       </c>
       <c r="B18" s="54" t="inlineStr">
         <is>
-          <t>المواعيد والاستحقاقات وتقادم الذمم الأساسي</t>
+          <t>حماية Cost Snapshot وإعلان النتيجة النهائية أو التقديرية</t>
         </is>
       </c>
       <c r="C18" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D18" s="54" t="inlineStr">
@@ -1742,24 +1742,24 @@
       </c>
       <c r="K18" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
         </is>
       </c>
       <c r="L18" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
+          <t>CTRL-001, OPS-007</t>
         </is>
       </c>
       <c r="M18" s="54" t="inlineStr"/>
       <c r="N18" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
         </is>
       </c>
       <c r="O18" s="54" t="inlineStr"/>
       <c r="P18" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q18" s="54" t="inlineStr">
@@ -1771,17 +1771,17 @@
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="54" t="inlineStr">
         <is>
-          <t>OPS-005</t>
+          <t>REL-001</t>
         </is>
       </c>
       <c r="B19" s="54" t="inlineStr">
         <is>
-          <t>سطح قادم موحد للدفعات والتحصيلات والطلبات والالتزامات</t>
+          <t>اختبارات الصمود والفشل</t>
         </is>
       </c>
       <c r="C19" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D19" s="54" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="H19" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>stage-6</t>
         </is>
       </c>
       <c r="I19" s="54" t="inlineStr">
@@ -1816,29 +1816,29 @@
       </c>
       <c r="J19" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>storage, transfer, resilience</t>
         </is>
       </c>
       <c r="K19" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
         </is>
       </c>
       <c r="L19" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-001</t>
+          <t>CLEAN-001</t>
         </is>
       </c>
       <c r="M19" s="54" t="inlineStr"/>
       <c r="N19" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>تحقق من الاعتماديات (CLEAN-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O19" s="54" t="inlineStr"/>
       <c r="P19" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q19" s="54" t="inlineStr">
@@ -1850,12 +1850,12 @@
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="54" t="inlineStr">
         <is>
-          <t>OPS-009</t>
+          <t>CLEAN-001</t>
         </is>
       </c>
       <c r="B20" s="54" t="inlineStr">
         <is>
-          <t>حماية Cost Snapshot وإعلان النتيجة النهائية أو التقديرية</t>
+          <t>تنظيف الأسطح الجزئية والميتة</t>
         </is>
       </c>
       <c r="C20" s="54" t="inlineStr">
@@ -1880,12 +1880,12 @@
       </c>
       <c r="G20" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H20" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>stage-4</t>
         </is>
       </c>
       <c r="I20" s="54" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="J20" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>cross-layer, presentation</t>
         </is>
       </c>
       <c r="K20" s="54" t="inlineStr">
@@ -1905,19 +1905,19 @@
       </c>
       <c r="L20" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-007</t>
+          <t>FIN-007, OPS-004</t>
         </is>
       </c>
       <c r="M20" s="54" t="inlineStr"/>
       <c r="N20" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>تحقق من الاعتماديات (FIN-007, OPS-004) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O20" s="54" t="inlineStr"/>
       <c r="P20" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q20" s="54" t="inlineStr">
@@ -1929,17 +1929,17 @@
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="54" t="inlineStr">
         <is>
-          <t>REL-001</t>
+          <t>FIN-007</t>
         </is>
       </c>
       <c r="B21" s="54" t="inlineStr">
         <is>
-          <t>اختبارات الصمود والفشل</t>
+          <t>مراجعة فترة مرنة</t>
         </is>
       </c>
       <c r="C21" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D21" s="54" t="inlineStr">
@@ -1959,12 +1959,12 @@
       </c>
       <c r="G21" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H21" s="54" t="inlineStr">
         <is>
-          <t>stage-6</t>
+          <t>stage-3</t>
         </is>
       </c>
       <c r="I21" s="54" t="inlineStr">
@@ -1974,23 +1974,23 @@
       </c>
       <c r="J21" s="54" t="inlineStr">
         <is>
-          <t>storage, transfer, resilience</t>
+          <t>Layer 3, domain, application, presentation</t>
         </is>
       </c>
       <c r="K21" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
       <c r="L21" s="54" t="inlineStr">
         <is>
-          <t>CLEAN-001</t>
+          <t>FIN-003</t>
         </is>
       </c>
       <c r="M21" s="54" t="inlineStr"/>
       <c r="N21" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CLEAN-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (FIN-003) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O21" s="54" t="inlineStr"/>
@@ -2008,17 +2008,17 @@
     <row r="22" ht="24" customHeight="1">
       <c r="A22" s="54" t="inlineStr">
         <is>
-          <t>CLEAN-001</t>
+          <t>OPS-002</t>
         </is>
       </c>
       <c r="B22" s="54" t="inlineStr">
         <is>
-          <t>تنظيف الأسطح الجزئية والميتة</t>
+          <t>تنبيهات انخفاض المخزون</t>
         </is>
       </c>
       <c r="C22" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D22" s="54" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="H22" s="54" t="inlineStr">
         <is>
-          <t>stage-4</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I22" s="54" t="inlineStr">
@@ -2053,23 +2053,23 @@
       </c>
       <c r="J22" s="54" t="inlineStr">
         <is>
-          <t>cross-layer, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K22" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
       <c r="L22" s="54" t="inlineStr">
         <is>
-          <t>FIN-007, OPS-004</t>
+          <t>CTRL-001</t>
         </is>
       </c>
       <c r="M22" s="54" t="inlineStr"/>
       <c r="N22" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (FIN-007, OPS-004) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O22" s="54" t="inlineStr"/>
@@ -2087,12 +2087,12 @@
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="54" t="inlineStr">
         <is>
-          <t>FIN-007</t>
+          <t>OPS-004</t>
         </is>
       </c>
       <c r="B23" s="54" t="inlineStr">
         <is>
-          <t>مراجعة فترة مرنة</t>
+          <t>ربط القوالب بالتكلفة المخططة دون استهلاك فعلي</t>
         </is>
       </c>
       <c r="C23" s="54" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="H23" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I23" s="54" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="J23" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K23" s="54" t="inlineStr">
@@ -2142,13 +2142,13 @@
       </c>
       <c r="L23" s="54" t="inlineStr">
         <is>
-          <t>FIN-003</t>
+          <t>CTRL-001</t>
         </is>
       </c>
       <c r="M23" s="54" t="inlineStr"/>
       <c r="N23" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (FIN-003) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
         </is>
       </c>
       <c r="O23" s="54" t="inlineStr"/>
@@ -2166,12 +2166,12 @@
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="54" t="inlineStr">
         <is>
-          <t>OPS-002</t>
+          <t>OPS-006</t>
         </is>
       </c>
       <c r="B24" s="54" t="inlineStr">
         <is>
-          <t>تنبيهات انخفاض المخزون</t>
+          <t>تقادم ديون مبسط قبل الشرائح المتقدمة</t>
         </is>
       </c>
       <c r="C24" s="54" t="inlineStr">
@@ -2221,19 +2221,19 @@
       </c>
       <c r="L24" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
+          <t>CTRL-001, OPS-001</t>
         </is>
       </c>
       <c r="M24" s="54" t="inlineStr"/>
       <c r="N24" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
         </is>
       </c>
       <c r="O24" s="54" t="inlineStr"/>
       <c r="P24" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q24" s="54" t="inlineStr">
@@ -2245,12 +2245,12 @@
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="54" t="inlineStr">
         <is>
-          <t>OPS-004</t>
+          <t>OPS-007</t>
         </is>
       </c>
       <c r="B25" s="54" t="inlineStr">
         <is>
-          <t>ربط القوالب بالتكلفة المخططة دون استهلاك فعلي</t>
+          <t>مقارنة التكلفة المخططة بالمستهلكة والفرق</t>
         </is>
       </c>
       <c r="C25" s="54" t="inlineStr">
@@ -2300,19 +2300,19 @@
       </c>
       <c r="L25" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
+          <t>CTRL-001, OPS-004</t>
         </is>
       </c>
       <c r="M25" s="54" t="inlineStr"/>
       <c r="N25" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
         </is>
       </c>
       <c r="O25" s="54" t="inlineStr"/>
       <c r="P25" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q25" s="54" t="inlineStr">
@@ -2324,12 +2324,12 @@
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="54" t="inlineStr">
         <is>
-          <t>OPS-006</t>
+          <t>OPS-008</t>
         </is>
       </c>
       <c r="B26" s="54" t="inlineStr">
         <is>
-          <t>تقادم ديون مبسط قبل الشرائح المتقدمة</t>
+          <t>الوقت الفعلي مقابل المخطط</t>
         </is>
       </c>
       <c r="C26" s="54" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="L26" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-001</t>
+          <t>CTRL-001, OPS-004</t>
         </is>
       </c>
       <c r="M26" s="54" t="inlineStr"/>
@@ -2403,27 +2403,27 @@
     <row r="27" ht="24" customHeight="1">
       <c r="A27" s="54" t="inlineStr">
         <is>
-          <t>OPS-007</t>
+          <t>AUDIT-001</t>
         </is>
       </c>
       <c r="B27" s="54" t="inlineStr">
         <is>
-          <t>مقارنة التكلفة المخططة بالمستهلكة والفرق</t>
+          <t>تدقيق مستقل نهائي قبل الـPilot</t>
         </is>
       </c>
       <c r="C27" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D27" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E27" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>RELEASE_GATE</t>
         </is>
       </c>
       <c r="F27" s="54" t="inlineStr">
@@ -2433,12 +2433,12 @@
       </c>
       <c r="G27" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H27" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>stage-9</t>
         </is>
       </c>
       <c r="I27" s="54" t="inlineStr">
@@ -2448,29 +2448,29 @@
       </c>
       <c r="J27" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>uat, audit, cross-layer</t>
         </is>
       </c>
       <c r="K27" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
         </is>
       </c>
       <c r="L27" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-004</t>
+          <t>UAT-001</t>
         </is>
       </c>
       <c r="M27" s="54" t="inlineStr"/>
       <c r="N27" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>حوّل البند إلى READY بعد تحقق الاعتماديات (UAT-001) ومعيار القبول.</t>
         </is>
       </c>
       <c r="O27" s="54" t="inlineStr"/>
       <c r="P27" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q27" s="54" t="inlineStr">
@@ -2482,27 +2482,27 @@
     <row r="28" ht="24" customHeight="1">
       <c r="A28" s="54" t="inlineStr">
         <is>
-          <t>OPS-008</t>
+          <t>UAT-001</t>
         </is>
       </c>
       <c r="B28" s="54" t="inlineStr">
         <is>
-          <t>الوقت الفعلي مقابل المخطط</t>
+          <t>قبول داخلي ببيانات Demo كاملة</t>
         </is>
       </c>
       <c r="C28" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D28" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E28" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>RELEASE_GATE</t>
         </is>
       </c>
       <c r="F28" s="54" t="inlineStr">
@@ -2512,12 +2512,12 @@
       </c>
       <c r="G28" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H28" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>stage-9</t>
         </is>
       </c>
       <c r="I28" s="54" t="inlineStr">
@@ -2527,29 +2527,29 @@
       </c>
       <c r="J28" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>uat, audit, cross-layer</t>
         </is>
       </c>
       <c r="K28" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
         </is>
       </c>
       <c r="L28" s="54" t="inlineStr">
         <is>
-          <t>CTRL-001, OPS-004</t>
+          <t>DEVICE-001, LEGAL-001</t>
         </is>
       </c>
       <c r="M28" s="54" t="inlineStr"/>
       <c r="N28" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>حوّل البند إلى READY بعد تحقق الاعتماديات (DEVICE-001, LEGAL-001) ومعيار القبول.</t>
         </is>
       </c>
       <c r="O28" s="54" t="inlineStr"/>
       <c r="P28" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q28" s="54" t="inlineStr">
@@ -2561,27 +2561,27 @@
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="54" t="inlineStr">
         <is>
-          <t>AUDIT-001</t>
+          <t>G-001</t>
         </is>
       </c>
       <c r="B29" s="54" t="inlineStr">
         <is>
-          <t>تدقيق مستقل نهائي قبل الـPilot</t>
+          <t>فخ الاستهلاك المزدوج عند التسليم</t>
         </is>
       </c>
       <c r="C29" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>DEFECT</t>
         </is>
       </c>
       <c r="D29" s="54" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="E29" s="54" t="inlineStr">
         <is>
-          <t>RELEASE_GATE</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F29" s="54" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="H29" s="54" t="inlineStr">
         <is>
-          <t>stage-9</t>
+          <t>audit-2026-09-19</t>
         </is>
       </c>
       <c r="I29" s="54" t="inlineStr">
@@ -2606,29 +2606,25 @@
       </c>
       <c r="J29" s="54" t="inlineStr">
         <is>
-          <t>uat, audit, cross-layer</t>
+          <t>cross-layer</t>
         </is>
       </c>
       <c r="K29" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
-        </is>
-      </c>
-      <c r="L29" s="54" t="inlineStr">
-        <is>
-          <t>UAT-001</t>
-        </is>
-      </c>
+          <t>Domain/Service tests where the invariant is owned | DOM/Integration test for the affected journey | Live scenario with before/after evidence | Retry, partial failure, concurrency, or stale-read test as applicable | No regression in existing financial calculations | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L29" s="54" t="inlineStr"/>
       <c r="M29" s="54" t="inlineStr"/>
       <c r="N29" s="54" t="inlineStr">
         <is>
-          <t>حوّل البند إلى READY بعد تحقق الاعتماديات (UAT-001) ومعيار القبول.</t>
+          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
         </is>
       </c>
       <c r="O29" s="54" t="inlineStr"/>
       <c r="P29" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q29" s="54" t="inlineStr">
@@ -2640,27 +2636,27 @@
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="54" t="inlineStr">
         <is>
-          <t>UAT-001</t>
+          <t>GOV-001</t>
         </is>
       </c>
       <c r="B30" s="54" t="inlineStr">
         <is>
-          <t>قبول داخلي ببيانات Demo كاملة</t>
+          <t>مصالحة G10-A مع تعارض عقد C1</t>
         </is>
       </c>
       <c r="C30" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>DECISION</t>
         </is>
       </c>
       <c r="D30" s="54" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="E30" s="54" t="inlineStr">
         <is>
-          <t>RELEASE_GATE</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="F30" s="54" t="inlineStr">
@@ -2675,7 +2671,7 @@
       </c>
       <c r="H30" s="54" t="inlineStr">
         <is>
-          <t>stage-9</t>
+          <t>governance</t>
         </is>
       </c>
       <c r="I30" s="54" t="inlineStr">
@@ -2685,29 +2681,29 @@
       </c>
       <c r="J30" s="54" t="inlineStr">
         <is>
-          <t>uat, audit, cross-layer</t>
+          <t>governance, contracts</t>
         </is>
       </c>
       <c r="K30" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
-        </is>
-      </c>
-      <c r="L30" s="54" t="inlineStr">
-        <is>
-          <t>DEVICE-001, LEGAL-001</t>
-        </is>
-      </c>
-      <c r="M30" s="54" t="inlineStr"/>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L30" s="54" t="inlineStr"/>
+      <c r="M30" s="54" t="inlineStr">
+        <is>
+          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
+        </is>
+      </c>
       <c r="N30" s="54" t="inlineStr">
         <is>
-          <t>حوّل البند إلى READY بعد تحقق الاعتماديات (DEVICE-001, LEGAL-001) ومعيار القبول.</t>
+          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
         </is>
       </c>
       <c r="O30" s="54" t="inlineStr"/>
       <c r="P30" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q30" s="54" t="inlineStr">
@@ -2719,12 +2715,12 @@
     <row r="31" ht="24" customHeight="1">
       <c r="A31" s="54" t="inlineStr">
         <is>
-          <t>G-001</t>
+          <t>G-002</t>
         </is>
       </c>
       <c r="B31" s="54" t="inlineStr">
         <is>
-          <t>فخ الاستهلاك المزدوج عند التسليم</t>
+          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
         </is>
       </c>
       <c r="C31" s="54" t="inlineStr">
@@ -2749,7 +2745,7 @@
       </c>
       <c r="G31" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H31" s="54" t="inlineStr">
@@ -2776,7 +2772,7 @@
       <c r="M31" s="54" t="inlineStr"/>
       <c r="N31" s="54" t="inlineStr">
         <is>
-          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
+          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
         </is>
       </c>
       <c r="O31" s="54" t="inlineStr"/>
@@ -2794,17 +2790,17 @@
     <row r="32" ht="24" customHeight="1">
       <c r="A32" s="54" t="inlineStr">
         <is>
-          <t>GOV-001</t>
+          <t>G-003</t>
         </is>
       </c>
       <c r="B32" s="54" t="inlineStr">
         <is>
-          <t>مصالحة G10-A مع تعارض عقد C1</t>
+          <t>حرس القراءة القديمة عند حفظ الطلب</t>
         </is>
       </c>
       <c r="C32" s="54" t="inlineStr">
         <is>
-          <t>DECISION</t>
+          <t>DEFECT</t>
         </is>
       </c>
       <c r="D32" s="54" t="inlineStr">
@@ -2814,7 +2810,7 @@
       </c>
       <c r="E32" s="54" t="inlineStr">
         <is>
-          <t>GOVERNANCE</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F32" s="54" t="inlineStr">
@@ -2824,12 +2820,12 @@
       </c>
       <c r="G32" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H32" s="54" t="inlineStr">
         <is>
-          <t>governance</t>
+          <t>audit-2026-09-19</t>
         </is>
       </c>
       <c r="I32" s="54" t="inlineStr">
@@ -2839,23 +2835,19 @@
       </c>
       <c r="J32" s="54" t="inlineStr">
         <is>
-          <t>governance, contracts</t>
+          <t>cross-layer</t>
         </is>
       </c>
       <c r="K32" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+          <t>Domain/Service tests where the invariant is owned | DOM/Integration test for the affected journey | Live scenario with before/after evidence | Retry, partial failure, concurrency, or stale-read test as applicable | No regression in existing financial calculations | Merge and verification evidence on main</t>
         </is>
       </c>
       <c r="L32" s="54" t="inlineStr"/>
-      <c r="M32" s="54" t="inlineStr">
-        <is>
-          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
-        </is>
-      </c>
+      <c r="M32" s="54" t="inlineStr"/>
       <c r="N32" s="54" t="inlineStr">
         <is>
-          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
+          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
         </is>
       </c>
       <c r="O32" s="54" t="inlineStr"/>
@@ -2873,12 +2865,12 @@
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="54" t="inlineStr">
         <is>
-          <t>G-002</t>
+          <t>G-004</t>
         </is>
       </c>
       <c r="B33" s="54" t="inlineStr">
         <is>
-          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
+          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
         </is>
       </c>
       <c r="C33" s="54" t="inlineStr">
@@ -2930,7 +2922,7 @@
       <c r="M33" s="54" t="inlineStr"/>
       <c r="N33" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
+          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
         </is>
       </c>
       <c r="O33" s="54" t="inlineStr"/>
@@ -2948,12 +2940,12 @@
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="54" t="inlineStr">
         <is>
-          <t>G-003</t>
+          <t>G-005</t>
         </is>
       </c>
       <c r="B34" s="54" t="inlineStr">
         <is>
-          <t>حرس القراءة القديمة عند حفظ الطلب</t>
+          <t>عزل فشل قراءات صفحة المالية</t>
         </is>
       </c>
       <c r="C34" s="54" t="inlineStr">
@@ -3005,7 +2997,7 @@
       <c r="M34" s="54" t="inlineStr"/>
       <c r="N34" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
+          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
         </is>
       </c>
       <c r="O34" s="54" t="inlineStr"/>
@@ -3023,12 +3015,12 @@
     <row r="35" ht="24" customHeight="1">
       <c r="A35" s="54" t="inlineStr">
         <is>
-          <t>G-004</t>
+          <t>G-006</t>
         </is>
       </c>
       <c r="B35" s="54" t="inlineStr">
         <is>
-          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
+          <t>توحيد حرس السحب بين مساري مال المالك</t>
         </is>
       </c>
       <c r="C35" s="54" t="inlineStr">
@@ -3053,7 +3045,7 @@
       </c>
       <c r="G35" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H35" s="54" t="inlineStr">
@@ -3080,7 +3072,7 @@
       <c r="M35" s="54" t="inlineStr"/>
       <c r="N35" s="54" t="inlineStr">
         <is>
-          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
+          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
         </is>
       </c>
       <c r="O35" s="54" t="inlineStr"/>
@@ -3098,42 +3090,42 @@
     <row r="36" ht="24" customHeight="1">
       <c r="A36" s="54" t="inlineStr">
         <is>
-          <t>G-005</t>
+          <t>SCOPE-001</t>
         </is>
       </c>
       <c r="B36" s="54" t="inlineStr">
         <is>
-          <t>عزل فشل قراءات صفحة المالية</t>
+          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
         </is>
       </c>
       <c r="C36" s="54" t="inlineStr">
         <is>
-          <t>DEFECT</t>
+          <t>DECISION</t>
         </is>
       </c>
       <c r="D36" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="E36" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>FUTURE_SCOPE</t>
         </is>
       </c>
       <c r="F36" s="54" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE</t>
+          <t>OUT_OF_SCOPE</t>
         </is>
       </c>
       <c r="G36" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H36" s="54" t="inlineStr">
         <is>
-          <t>audit-2026-09-19</t>
+          <t>future-scope</t>
         </is>
       </c>
       <c r="I36" s="54" t="inlineStr">
@@ -3143,22 +3135,30 @@
       </c>
       <c r="J36" s="54" t="inlineStr">
         <is>
-          <t>cross-layer</t>
+          <t>future-scope</t>
         </is>
       </c>
       <c r="K36" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests where the invariant is owned | DOM/Integration test for the affected journey | Live scenario with before/after evidence | Retry, partial failure, concurrency, or stale-read test as applicable | No regression in existing financial calculations | Merge and verification evidence on main</t>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
       <c r="L36" s="54" t="inlineStr"/>
-      <c r="M36" s="54" t="inlineStr"/>
+      <c r="M36" s="54" t="inlineStr">
+        <is>
+          <t>تحديد بوابة مستقلة لكل توسع مستقبلًا.</t>
+        </is>
+      </c>
       <c r="N36" s="54" t="inlineStr">
         <is>
-          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
-        </is>
-      </c>
-      <c r="O36" s="54" t="inlineStr"/>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+        </is>
+      </c>
+      <c r="O36" s="54" t="inlineStr">
+        <is>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+        </is>
+      </c>
       <c r="P36" s="54" t="inlineStr">
         <is>
           <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
@@ -3173,22 +3173,22 @@
     <row r="37">
       <c r="A37" s="54" t="inlineStr">
         <is>
-          <t>G-006</t>
+          <t>UX-001</t>
         </is>
       </c>
       <c r="B37" s="54" t="inlineStr">
         <is>
-          <t>توحيد حرس السحب بين مساري مال المالك</t>
+          <t>إعادة تصميم UI وUX جذرية</t>
         </is>
       </c>
       <c r="C37" s="54" t="inlineStr">
         <is>
-          <t>DEFECT</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D37" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="E37" s="54" t="inlineStr">
@@ -3198,17 +3198,17 @@
       </c>
       <c r="F37" s="54" t="inlineStr">
         <is>
-          <t>NOT_APPLICABLE</t>
+          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="G37" s="54" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H37" s="54" t="inlineStr">
         <is>
-          <t>audit-2026-09-19</t>
+          <t>stage-5</t>
         </is>
       </c>
       <c r="I37" s="54" t="inlineStr">
@@ -3218,25 +3218,37 @@
       </c>
       <c r="J37" s="54" t="inlineStr">
         <is>
-          <t>cross-layer</t>
+          <t>ui/ux, presentation</t>
         </is>
       </c>
       <c r="K37" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests where the invariant is owned | DOM/Integration test for the affected journey | Live scenario with before/after evidence | Retry, partial failure, concurrency, or stale-read test as applicable | No regression in existing financial calculations | Merge and verification evidence on main</t>
-        </is>
-      </c>
-      <c r="L37" s="54" t="inlineStr"/>
-      <c r="M37" s="54" t="inlineStr"/>
+          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
+        </is>
+      </c>
+      <c r="L37" s="54" t="inlineStr">
+        <is>
+          <t>CLEAN-001</t>
+        </is>
+      </c>
+      <c r="M37" s="54" t="inlineStr">
+        <is>
+          <t>اعتماد الاتجاه البصري النهائي ونتائج Benchmark قبل التنفيذ.</t>
+        </is>
+      </c>
       <c r="N37" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
-        </is>
-      </c>
-      <c r="O37" s="54" t="inlineStr"/>
+          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
+        </is>
+      </c>
+      <c r="O37" s="54" t="inlineStr">
+        <is>
+          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+        </is>
+      </c>
       <c r="P37" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
         </is>
       </c>
       <c r="Q37" s="54" t="inlineStr">
@@ -3248,17 +3260,17 @@
     <row r="38">
       <c r="A38" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-001</t>
+          <t>BE-001</t>
         </is>
       </c>
       <c r="B38" s="54" t="inlineStr">
         <is>
-          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
+          <t>مصاريف متكررة محلية</t>
         </is>
       </c>
       <c r="C38" s="54" t="inlineStr">
         <is>
-          <t>DECISION</t>
+          <t>FEATURE</t>
         </is>
       </c>
       <c r="D38" s="54" t="inlineStr">
@@ -3268,22 +3280,22 @@
       </c>
       <c r="E38" s="54" t="inlineStr">
         <is>
-          <t>FUTURE_SCOPE</t>
+          <t>HISTORICAL</t>
         </is>
       </c>
       <c r="F38" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE</t>
+          <t>DUPLICATE_HISTORICAL</t>
         </is>
       </c>
       <c r="G38" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H38" s="54" t="inlineStr">
         <is>
-          <t>future-scope</t>
+          <t>build-after-evidence</t>
         </is>
       </c>
       <c r="I38" s="54" t="inlineStr">
@@ -3293,7 +3305,7 @@
       </c>
       <c r="J38" s="54" t="inlineStr">
         <is>
-          <t>future-scope</t>
+          <t>future-capability</t>
         </is>
       </c>
       <c r="K38" s="54" t="inlineStr">
@@ -3302,19 +3314,15 @@
         </is>
       </c>
       <c r="L38" s="54" t="inlineStr"/>
-      <c r="M38" s="54" t="inlineStr">
-        <is>
-          <t>تحديد بوابة مستقلة لكل توسع مستقبلًا.</t>
-        </is>
-      </c>
+      <c r="M38" s="54" t="inlineStr"/>
       <c r="N38" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
       <c r="O38" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
         </is>
       </c>
       <c r="P38" s="54" t="inlineStr">
@@ -3331,12 +3339,12 @@
     <row r="39">
       <c r="A39" s="54" t="inlineStr">
         <is>
-          <t>UX-001</t>
+          <t>BE-002</t>
         </is>
       </c>
       <c r="B39" s="54" t="inlineStr">
         <is>
-          <t>إعادة تصميم UI وUX جذرية</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="C39" s="54" t="inlineStr">
@@ -3351,22 +3359,22 @@
       </c>
       <c r="E39" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>HISTORICAL</t>
         </is>
       </c>
       <c r="F39" s="54" t="inlineStr">
         <is>
-          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
+          <t>DUPLICATE_HISTORICAL</t>
         </is>
       </c>
       <c r="G39" s="54" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="H39" s="54" t="inlineStr">
         <is>
-          <t>stage-5</t>
+          <t>build-after-evidence</t>
         </is>
       </c>
       <c r="I39" s="54" t="inlineStr">
@@ -3376,7 +3384,7 @@
       </c>
       <c r="J39" s="54" t="inlineStr">
         <is>
-          <t>ui/ux, presentation</t>
+          <t>future-capability</t>
         </is>
       </c>
       <c r="K39" s="54" t="inlineStr">
@@ -3384,29 +3392,21 @@
           <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
-      <c r="L39" s="54" t="inlineStr">
-        <is>
-          <t>CLEAN-001</t>
-        </is>
-      </c>
-      <c r="M39" s="54" t="inlineStr">
-        <is>
-          <t>اعتماد الاتجاه البصري النهائي ونتائج Benchmark قبل التنفيذ.</t>
-        </is>
-      </c>
+      <c r="L39" s="54" t="inlineStr"/>
+      <c r="M39" s="54" t="inlineStr"/>
       <c r="N39" s="54" t="inlineStr">
         <is>
-          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
       <c r="O39" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
         </is>
       </c>
       <c r="P39" s="54" t="inlineStr">
         <is>
-          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q39" s="54" t="inlineStr">
@@ -3418,12 +3418,12 @@
     <row r="40">
       <c r="A40" s="54" t="inlineStr">
         <is>
-          <t>BE-001</t>
+          <t>BE-003</t>
         </is>
       </c>
       <c r="B40" s="54" t="inlineStr">
         <is>
-          <t>مصاريف متكررة محلية</t>
+          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="C40" s="54" t="inlineStr">
@@ -3475,7 +3475,7 @@
       <c r="M40" s="54" t="inlineStr"/>
       <c r="N40" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
       <c r="O40" s="54" t="inlineStr">
@@ -3497,12 +3497,12 @@
     <row r="41">
       <c r="A41" s="54" t="inlineStr">
         <is>
-          <t>BE-002</t>
+          <t>BE-004</t>
         </is>
       </c>
       <c r="B41" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>إغلاق فترة رسمي</t>
         </is>
       </c>
       <c r="C41" s="54" t="inlineStr">
@@ -3517,12 +3517,12 @@
       </c>
       <c r="E41" s="54" t="inlineStr">
         <is>
-          <t>HISTORICAL</t>
+          <t>PILOT_VALIDATION</t>
         </is>
       </c>
       <c r="F41" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL</t>
+          <t>PILOT_EVIDENCE_REQUIRED</t>
         </is>
       </c>
       <c r="G41" s="54" t="inlineStr">
@@ -3554,12 +3554,12 @@
       <c r="M41" s="54" t="inlineStr"/>
       <c r="N41" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
       <c r="O41" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="P41" s="54" t="inlineStr">
@@ -3576,12 +3576,12 @@
     <row r="42">
       <c r="A42" s="54" t="inlineStr">
         <is>
-          <t>BE-003</t>
+          <t>BE-005</t>
         </is>
       </c>
       <c r="B42" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
+          <t>تقادم الديون بشرائح 30/60/90</t>
         </is>
       </c>
       <c r="C42" s="54" t="inlineStr">
@@ -3596,12 +3596,12 @@
       </c>
       <c r="E42" s="54" t="inlineStr">
         <is>
-          <t>HISTORICAL</t>
+          <t>PILOT_VALIDATION</t>
         </is>
       </c>
       <c r="F42" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL</t>
+          <t>PILOT_EVIDENCE_REQUIRED</t>
         </is>
       </c>
       <c r="G42" s="54" t="inlineStr">
@@ -3633,12 +3633,12 @@
       <c r="M42" s="54" t="inlineStr"/>
       <c r="N42" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
       <c r="O42" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="P42" s="54" t="inlineStr">
@@ -3655,12 +3655,12 @@
     <row r="43">
       <c r="A43" s="54" t="inlineStr">
         <is>
-          <t>BE-004</t>
+          <t>FIN-002</t>
         </is>
       </c>
       <c r="B43" s="54" t="inlineStr">
         <is>
-          <t>إغلاق فترة رسمي</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="C43" s="54" t="inlineStr">
@@ -3675,12 +3675,12 @@
       </c>
       <c r="E43" s="54" t="inlineStr">
         <is>
-          <t>PILOT_VALIDATION</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F43" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED</t>
+          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="G43" s="54" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="H43" s="54" t="inlineStr">
         <is>
-          <t>build-after-evidence</t>
+          <t>stage-3</t>
         </is>
       </c>
       <c r="I43" s="54" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="J43" s="54" t="inlineStr">
         <is>
-          <t>future-capability</t>
+          <t>Layer 3, domain, application, presentation</t>
         </is>
       </c>
       <c r="K43" s="54" t="inlineStr">
@@ -3708,21 +3708,25 @@
           <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
-      <c r="L43" s="54" t="inlineStr"/>
+      <c r="L43" s="54" t="inlineStr">
+        <is>
+          <t>CTRL-001</t>
+        </is>
+      </c>
       <c r="M43" s="54" t="inlineStr"/>
       <c r="N43" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
         </is>
       </c>
       <c r="O43" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="P43" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q43" s="54" t="inlineStr">
@@ -3734,12 +3738,12 @@
     <row r="44">
       <c r="A44" s="54" t="inlineStr">
         <is>
-          <t>BE-005</t>
+          <t>FIN-006</t>
         </is>
       </c>
       <c r="B44" s="54" t="inlineStr">
         <is>
-          <t>تقادم الديون بشرائح 30/60/90</t>
+          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="C44" s="54" t="inlineStr">
@@ -3754,12 +3758,12 @@
       </c>
       <c r="E44" s="54" t="inlineStr">
         <is>
-          <t>PILOT_VALIDATION</t>
+          <t>FIX_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="F44" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED</t>
+          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
         </is>
       </c>
       <c r="G44" s="54" t="inlineStr">
@@ -3769,7 +3773,7 @@
       </c>
       <c r="H44" s="54" t="inlineStr">
         <is>
-          <t>build-after-evidence</t>
+          <t>stage-3</t>
         </is>
       </c>
       <c r="I44" s="54" t="inlineStr">
@@ -3779,7 +3783,7 @@
       </c>
       <c r="J44" s="54" t="inlineStr">
         <is>
-          <t>future-capability</t>
+          <t>Layer 3, domain, application, presentation</t>
         </is>
       </c>
       <c r="K44" s="54" t="inlineStr">
@@ -3787,21 +3791,25 @@
           <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
         </is>
       </c>
-      <c r="L44" s="54" t="inlineStr"/>
+      <c r="L44" s="54" t="inlineStr">
+        <is>
+          <t>OPS-004</t>
+        </is>
+      </c>
       <c r="M44" s="54" t="inlineStr"/>
       <c r="N44" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
         </is>
       </c>
       <c r="O44" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="P44" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q44" s="54" t="inlineStr">
@@ -3813,17 +3821,17 @@
     <row r="45">
       <c r="A45" s="54" t="inlineStr">
         <is>
-          <t>FIN-002</t>
+          <t>FIN-008</t>
         </is>
       </c>
       <c r="B45" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>تحقق الإهلاك بعد مرور الزمن</t>
         </is>
       </c>
       <c r="C45" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D45" s="54" t="inlineStr">
@@ -3863,23 +3871,23 @@
       </c>
       <c r="K45" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
-        </is>
-      </c>
-      <c r="L45" s="54" t="inlineStr">
-        <is>
-          <t>CTRL-001</t>
-        </is>
-      </c>
-      <c r="M45" s="54" t="inlineStr"/>
+          <t>اختبار Domain/Service مع Clock قابل للحقن يثبت تاريخ الاستحقاق قبل/بعد نقطة زمنية اصطناعية | اختبار idempotency يمنع تسجيل الإهلاك نفسه مرتين عند إعادة تشغيل الساعة/الفعل | اختبار DOM يثبت أن الإهلاك غير النقدي لا يخصم من الكاش ويعرض الحالة الصادقة | اختبار export/import يحافظ على أصل الإهلاك وتاريخه إن دخلت البيانات الدائمة | دليل CI وMerge SHA وverified_on_main_sha قبل VERIFIED</t>
+        </is>
+      </c>
+      <c r="L45" s="54" t="inlineStr"/>
+      <c r="M45" s="54" t="inlineStr">
+        <is>
+          <t>تحديد نافذة اختبار الإهلاك أو آلية ساعة اختبار معتمدة قبل فتح Claim.</t>
+        </is>
+      </c>
       <c r="N45" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
+          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
         </is>
       </c>
       <c r="O45" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
         </is>
       </c>
       <c r="P45" s="54" t="inlineStr">
@@ -3896,12 +3904,12 @@
     <row r="46">
       <c r="A46" s="54" t="inlineStr">
         <is>
-          <t>FIN-006</t>
+          <t>OPS-003</t>
         </is>
       </c>
       <c r="B46" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
+          <t>المصروفات المتكررة المحلية</t>
         </is>
       </c>
       <c r="C46" s="54" t="inlineStr">
@@ -3931,7 +3939,7 @@
       </c>
       <c r="H46" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>stage-2</t>
         </is>
       </c>
       <c r="I46" s="54" t="inlineStr">
@@ -3941,7 +3949,7 @@
       </c>
       <c r="J46" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>Layer 2, application, presentation</t>
         </is>
       </c>
       <c r="K46" s="54" t="inlineStr">
@@ -3951,18 +3959,22 @@
       </c>
       <c r="L46" s="54" t="inlineStr">
         <is>
-          <t>OPS-004</t>
-        </is>
-      </c>
-      <c r="M46" s="54" t="inlineStr"/>
+          <t>CTRL-001</t>
+        </is>
+      </c>
+      <c r="M46" s="54" t="inlineStr">
+        <is>
+          <t>اعتماد أن المصروف المتكرر تذكير يحتاج تأكيدًا ولا ينشئ حدثًا ماليًا تلقائيًا.</t>
+        </is>
+      </c>
       <c r="N46" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
         </is>
       </c>
       <c r="O46" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
         </is>
       </c>
       <c r="P46" s="54" t="inlineStr">
@@ -3979,17 +3991,17 @@
     <row r="47">
       <c r="A47" s="54" t="inlineStr">
         <is>
-          <t>FIN-008</t>
+          <t>SCOPE-002</t>
         </is>
       </c>
       <c r="B47" s="54" t="inlineStr">
         <is>
-          <t>تحقق الإهلاك بعد مرور الزمن</t>
+          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
         </is>
       </c>
       <c r="C47" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>RESEARCH</t>
         </is>
       </c>
       <c r="D47" s="54" t="inlineStr">
@@ -3999,12 +4011,12 @@
       </c>
       <c r="E47" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>FUTURE_SCOPE</t>
         </is>
       </c>
       <c r="F47" s="54" t="inlineStr">
         <is>
-          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
+          <t>OUT_OF_SCOPE</t>
         </is>
       </c>
       <c r="G47" s="54" t="inlineStr">
@@ -4014,7 +4026,7 @@
       </c>
       <c r="H47" s="54" t="inlineStr">
         <is>
-          <t>stage-3</t>
+          <t>future-scope</t>
         </is>
       </c>
       <c r="I47" s="54" t="inlineStr">
@@ -4024,33 +4036,29 @@
       </c>
       <c r="J47" s="54" t="inlineStr">
         <is>
-          <t>Layer 3, domain, application, presentation</t>
+          <t>future-scope</t>
         </is>
       </c>
       <c r="K47" s="54" t="inlineStr">
         <is>
-          <t>اختبار Domain/Service مع Clock قابل للحقن يثبت تاريخ الاستحقاق قبل/بعد نقطة زمنية اصطناعية | اختبار idempotency يمنع تسجيل الإهلاك نفسه مرتين عند إعادة تشغيل الساعة/الفعل | اختبار DOM يثبت أن الإهلاك غير النقدي لا يخصم من الكاش ويعرض الحالة الصادقة | اختبار export/import يحافظ على أصل الإهلاك وتاريخه إن دخلت البيانات الدائمة | دليل CI وMerge SHA وverified_on_main_sha قبل VERIFIED</t>
+          <t>Source/report comparison | Explicit unknowns and limits | Owner decision or pilot evidence</t>
         </is>
       </c>
       <c r="L47" s="54" t="inlineStr"/>
-      <c r="M47" s="54" t="inlineStr">
-        <is>
-          <t>تحديد نافذة اختبار الإهلاك أو آلية ساعة اختبار معتمدة قبل فتح Claim.</t>
-        </is>
-      </c>
+      <c r="M47" s="54" t="inlineStr"/>
       <c r="N47" s="54" t="inlineStr">
         <is>
-          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
       <c r="O47" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="P47" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q47" s="54" t="inlineStr">
@@ -4062,17 +4070,17 @@
     <row r="48">
       <c r="A48" s="54" t="inlineStr">
         <is>
-          <t>OPS-003</t>
+          <t>UX-002</t>
         </is>
       </c>
       <c r="B48" s="54" t="inlineStr">
         <is>
-          <t>المصروفات المتكررة المحلية</t>
+          <t>Backlog الموجة الرابعة في عقد الملكية</t>
         </is>
       </c>
       <c r="C48" s="54" t="inlineStr">
         <is>
-          <t>FEATURE</t>
+          <t>QUALITY</t>
         </is>
       </c>
       <c r="D48" s="54" t="inlineStr">
@@ -4082,12 +4090,12 @@
       </c>
       <c r="E48" s="54" t="inlineStr">
         <is>
-          <t>FIX_BEFORE_PILOT</t>
+          <t>FUTURE_SCOPE</t>
         </is>
       </c>
       <c r="F48" s="54" t="inlineStr">
         <is>
-          <t>DEPENDENCY_GATE_REQUIRED_BEFORE_PILOT</t>
+          <t>OUT_OF_SCOPE</t>
         </is>
       </c>
       <c r="G48" s="54" t="inlineStr">
@@ -4097,7 +4105,7 @@
       </c>
       <c r="H48" s="54" t="inlineStr">
         <is>
-          <t>stage-2</t>
+          <t>post-pilot-gate</t>
         </is>
       </c>
       <c r="I48" s="54" t="inlineStr">
@@ -4107,37 +4115,29 @@
       </c>
       <c r="J48" s="54" t="inlineStr">
         <is>
-          <t>Layer 2, application, presentation</t>
+          <t>post-pilot</t>
         </is>
       </c>
       <c r="K48" s="54" t="inlineStr">
         <is>
-          <t>Domain/Service tests | DOM/Integration tests where UI is involved | Export/import or migration evidence where persistence changes | Merge and verification evidence on main</t>
-        </is>
-      </c>
-      <c r="L48" s="54" t="inlineStr">
-        <is>
-          <t>CTRL-001</t>
-        </is>
-      </c>
-      <c r="M48" s="54" t="inlineStr">
-        <is>
-          <t>اعتماد أن المصروف المتكرر تذكير يحتاج تأكيدًا ولا ينشئ حدثًا ماليًا تلقائيًا.</t>
-        </is>
-      </c>
+          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
+        </is>
+      </c>
+      <c r="L48" s="54" t="inlineStr"/>
+      <c r="M48" s="54" t="inlineStr"/>
       <c r="N48" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
       <c r="O48" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="P48" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/control/README.md</t>
+          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
         </is>
       </c>
       <c r="Q48" s="54" t="inlineStr">
@@ -4149,12 +4149,12 @@
     <row r="49">
       <c r="A49" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-002</t>
+          <t>V-001</t>
         </is>
       </c>
       <c r="B49" s="54" t="inlineStr">
         <is>
-          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
+          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
         </is>
       </c>
       <c r="C49" s="54" t="inlineStr">
@@ -4169,12 +4169,12 @@
       </c>
       <c r="E49" s="54" t="inlineStr">
         <is>
-          <t>FUTURE_SCOPE</t>
+          <t>PILOT_VALIDATION</t>
         </is>
       </c>
       <c r="F49" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE</t>
+          <t>PILOT_EVIDENCE_REQUIRED</t>
         </is>
       </c>
       <c r="G49" s="54" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="H49" s="54" t="inlineStr">
         <is>
-          <t>future-scope</t>
+          <t>pilot-validation</t>
         </is>
       </c>
       <c r="I49" s="54" t="inlineStr">
@@ -4194,24 +4194,24 @@
       </c>
       <c r="J49" s="54" t="inlineStr">
         <is>
-          <t>future-scope</t>
+          <t>pilot-validation</t>
         </is>
       </c>
       <c r="K49" s="54" t="inlineStr">
         <is>
-          <t>Source/report comparison | Explicit unknowns and limits | Owner decision or pilot evidence</t>
+          <t>Pilot observation protocol | Evidence log with denominator and outcome | Owner decision before any Feature claim</t>
         </is>
       </c>
       <c r="L49" s="54" t="inlineStr"/>
       <c r="M49" s="54" t="inlineStr"/>
       <c r="N49" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
       <c r="O49" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="P49" s="54" t="inlineStr">
@@ -4228,17 +4228,17 @@
     <row r="50">
       <c r="A50" s="54" t="inlineStr">
         <is>
-          <t>UX-002</t>
+          <t>V-002</t>
         </is>
       </c>
       <c r="B50" s="54" t="inlineStr">
         <is>
-          <t>Backlog الموجة الرابعة في عقد الملكية</t>
+          <t>V-02 — متوقعات الكاش القصيرة</t>
         </is>
       </c>
       <c r="C50" s="54" t="inlineStr">
         <is>
-          <t>QUALITY</t>
+          <t>RESEARCH</t>
         </is>
       </c>
       <c r="D50" s="54" t="inlineStr">
@@ -4248,12 +4248,12 @@
       </c>
       <c r="E50" s="54" t="inlineStr">
         <is>
-          <t>FUTURE_SCOPE</t>
+          <t>PILOT_VALIDATION</t>
         </is>
       </c>
       <c r="F50" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE</t>
+          <t>PILOT_EVIDENCE_REQUIRED</t>
         </is>
       </c>
       <c r="G50" s="54" t="inlineStr">
@@ -4263,7 +4263,7 @@
       </c>
       <c r="H50" s="54" t="inlineStr">
         <is>
-          <t>post-pilot-gate</t>
+          <t>pilot-validation</t>
         </is>
       </c>
       <c r="I50" s="54" t="inlineStr">
@@ -4273,24 +4273,24 @@
       </c>
       <c r="J50" s="54" t="inlineStr">
         <is>
-          <t>post-pilot</t>
+          <t>pilot-validation</t>
         </is>
       </c>
       <c r="K50" s="54" t="inlineStr">
         <is>
-          <t>Focused automated tests | Failure/recovery path where applicable | Evidence on main or explicit device limitation</t>
+          <t>Pilot observation protocol | Evidence log with denominator and outcome | Owner decision before any Feature claim</t>
         </is>
       </c>
       <c r="L50" s="54" t="inlineStr"/>
       <c r="M50" s="54" t="inlineStr"/>
       <c r="N50" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
       <c r="O50" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="P50" s="54" t="inlineStr">
@@ -4307,12 +4307,12 @@
     <row r="51">
       <c r="A51" s="54" t="inlineStr">
         <is>
-          <t>V-001</t>
+          <t>V-003</t>
         </is>
       </c>
       <c r="B51" s="54" t="inlineStr">
         <is>
-          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
+          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
         </is>
       </c>
       <c r="C51" s="54" t="inlineStr">
@@ -4386,12 +4386,12 @@
     <row r="52">
       <c r="A52" s="54" t="inlineStr">
         <is>
-          <t>V-002</t>
+          <t>V-004</t>
         </is>
       </c>
       <c r="B52" s="54" t="inlineStr">
         <is>
-          <t>V-02 — متوقعات الكاش القصيرة</t>
+          <t>V-04 — عرض التغطية عند قرار السحب</t>
         </is>
       </c>
       <c r="C52" s="54" t="inlineStr">
@@ -4465,12 +4465,12 @@
     <row r="53">
       <c r="A53" s="54" t="inlineStr">
         <is>
-          <t>V-003</t>
+          <t>V-005</t>
         </is>
       </c>
       <c r="B53" s="54" t="inlineStr">
         <is>
-          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
+          <t>V-05 — مقارنة فترتين بسيطة</t>
         </is>
       </c>
       <c r="C53" s="54" t="inlineStr">
@@ -4544,12 +4544,12 @@
     <row r="54">
       <c r="A54" s="54" t="inlineStr">
         <is>
-          <t>V-004</t>
+          <t>V-006</t>
         </is>
       </c>
       <c r="B54" s="54" t="inlineStr">
         <is>
-          <t>V-04 — عرض التغطية عند قرار السحب</t>
+          <t>V-06 — جسر ربح إلى كاش رقمي</t>
         </is>
       </c>
       <c r="C54" s="54" t="inlineStr">
@@ -4623,12 +4623,12 @@
     <row r="55">
       <c r="A55" s="54" t="inlineStr">
         <is>
-          <t>V-005</t>
+          <t>V-007</t>
         </is>
       </c>
       <c r="B55" s="54" t="inlineStr">
         <is>
-          <t>V-05 — مقارنة فترتين بسيطة</t>
+          <t>V-07 — تنبيه انخفاض المواد</t>
         </is>
       </c>
       <c r="C55" s="54" t="inlineStr">
@@ -4702,12 +4702,12 @@
     <row r="56">
       <c r="A56" s="54" t="inlineStr">
         <is>
-          <t>V-006</t>
+          <t>V-008</t>
         </is>
       </c>
       <c r="B56" s="54" t="inlineStr">
         <is>
-          <t>V-06 — جسر ربح إلى كاش رقمي</t>
+          <t>V-08 — مصروف اليوم على الرئيسية</t>
         </is>
       </c>
       <c r="C56" s="54" t="inlineStr">
@@ -4781,12 +4781,12 @@
     <row r="57">
       <c r="A57" s="54" t="inlineStr">
         <is>
-          <t>V-007</t>
+          <t>V-009</t>
         </is>
       </c>
       <c r="B57" s="54" t="inlineStr">
         <is>
-          <t>V-07 — تنبيه انخفاض المواد</t>
+          <t>V-09 — رقم السحب الآمن الموحد</t>
         </is>
       </c>
       <c r="C57" s="54" t="inlineStr">
@@ -4860,12 +4860,12 @@
     <row r="58">
       <c r="A58" s="54" t="inlineStr">
         <is>
-          <t>V-008</t>
+          <t>V-010</t>
         </is>
       </c>
       <c r="B58" s="54" t="inlineStr">
         <is>
-          <t>V-08 — مصروف اليوم على الرئيسية</t>
+          <t>V-10 — كثافة صفحة المالية</t>
         </is>
       </c>
       <c r="C58" s="54" t="inlineStr">
@@ -4939,12 +4939,12 @@
     <row r="59">
       <c r="A59" s="54" t="inlineStr">
         <is>
-          <t>V-009</t>
+          <t>V-011</t>
         </is>
       </c>
       <c r="B59" s="54" t="inlineStr">
         <is>
-          <t>V-09 — رقم السحب الآمن الموحد</t>
+          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
         </is>
       </c>
       <c r="C59" s="54" t="inlineStr">
@@ -5018,12 +5018,12 @@
     <row r="60">
       <c r="A60" s="54" t="inlineStr">
         <is>
-          <t>V-010</t>
+          <t>V-012</t>
         </is>
       </c>
       <c r="B60" s="54" t="inlineStr">
         <is>
-          <t>V-10 — كثافة صفحة المالية</t>
+          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
         </is>
       </c>
       <c r="C60" s="54" t="inlineStr">
@@ -5097,42 +5097,42 @@
     <row r="61">
       <c r="A61" s="54" t="inlineStr">
         <is>
-          <t>V-011</t>
+          <t>CTRL-001</t>
         </is>
       </c>
       <c r="B61" s="54" t="inlineStr">
         <is>
-          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
+          <t>اعتماد Operations Control v2</t>
         </is>
       </c>
       <c r="C61" s="54" t="inlineStr">
         <is>
-          <t>RESEARCH</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="D61" s="54" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E61" s="54" t="inlineStr">
         <is>
-          <t>PILOT_VALIDATION</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="F61" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED</t>
+          <t>NOT_APPLICABLE</t>
         </is>
       </c>
       <c r="G61" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H61" s="54" t="inlineStr">
         <is>
-          <t>pilot-validation</t>
+          <t>stage-0</t>
         </is>
       </c>
       <c r="I61" s="54" t="inlineStr">
@@ -5142,29 +5142,29 @@
       </c>
       <c r="J61" s="54" t="inlineStr">
         <is>
-          <t>pilot-validation</t>
+          <t>governance, documentation</t>
         </is>
       </c>
       <c r="K61" s="54" t="inlineStr">
         <is>
-          <t>Pilot observation protocol | Evidence log with denominator and outcome | Owner decision before any Feature claim</t>
+          <t>Validator/schema test | Generated-view freshness check | Owner review evidence</t>
         </is>
       </c>
       <c r="L61" s="54" t="inlineStr"/>
-      <c r="M61" s="54" t="inlineStr"/>
+      <c r="M61" s="54" t="inlineStr">
+        <is>
+          <t>تم اعتماد الإغلاق بعد دمج PR #188 والتحقق من main؛ لا يفتح Claim كودي بهذا السجل.</t>
+        </is>
+      </c>
       <c r="N61" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-      <c r="O61" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
+          <t>لا إجراء؛ سجل Operations Control v2 مدموج ومثبت على main. التنفيذ التالي يبدأ من G-001..G-006 في Claim مستقل.</t>
+        </is>
+      </c>
+      <c r="O61" s="54" t="inlineStr"/>
       <c r="P61" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q61" s="54" t="inlineStr">
@@ -5176,42 +5176,42 @@
     <row r="62">
       <c r="A62" s="54" t="inlineStr">
         <is>
-          <t>V-012</t>
+          <t>CTRL-002</t>
         </is>
       </c>
       <c r="B62" s="54" t="inlineStr">
         <is>
-          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
+          <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
         </is>
       </c>
       <c r="C62" s="54" t="inlineStr">
         <is>
-          <t>RESEARCH</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="D62" s="54" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E62" s="54" t="inlineStr">
         <is>
-          <t>PILOT_VALIDATION</t>
+          <t>GOVERNANCE</t>
         </is>
       </c>
       <c r="F62" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED</t>
+          <t>EVIDENCE_RECONCILIATION_REQUIRED</t>
         </is>
       </c>
       <c r="G62" s="54" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="H62" s="54" t="inlineStr">
         <is>
-          <t>pilot-validation</t>
+          <t>stage-0</t>
         </is>
       </c>
       <c r="I62" s="54" t="inlineStr">
@@ -5221,29 +5221,29 @@
       </c>
       <c r="J62" s="54" t="inlineStr">
         <is>
-          <t>pilot-validation</t>
+          <t>governance, documentation</t>
         </is>
       </c>
       <c r="K62" s="54" t="inlineStr">
         <is>
-          <t>Pilot observation protocol | Evidence log with denominator and outcome | Owner decision before any Feature claim</t>
+          <t>Validator/schema test | Generated-view freshness check | Owner review evidence</t>
         </is>
       </c>
       <c r="L62" s="54" t="inlineStr"/>
-      <c r="M62" s="54" t="inlineStr"/>
+      <c r="M62" s="54" t="inlineStr">
+        <is>
+          <t>تم اعتماد الإغلاق بعد دمج PR #188 والتحقق من main؛ لا يفتح Claim كودي بهذا السجل.</t>
+        </is>
+      </c>
       <c r="N62" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-      <c r="O62" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
+          <t>لا إجراء؛ المصالحة والبوابات مدموجة ومثبتة. لا تبدأ معالجة 49/46 أو Claim كودي جديد دون دليل جديد.</t>
+        </is>
+      </c>
+      <c r="O62" s="54" t="inlineStr"/>
       <c r="P62" s="54" t="inlineStr">
         <is>
-          <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+          <t>docs/operations/control/README.md</t>
         </is>
       </c>
       <c r="Q62" s="54" t="inlineStr">
@@ -6217,7 +6217,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6232,7 +6232,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="B5" s="53" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C5" s="53" t="inlineStr">
@@ -6640,7 +6640,7 @@
       </c>
       <c r="F5" s="53" t="inlineStr">
         <is>
-          <t>مراجعة المالك وAgent مستقل؛ لا دمج قبل قبول الملاحظات.</t>
+          <t>لا إجراء؛ Workstream التوثيقي مغلق. يبدأ أي تنفيذ لاحق في Workstream مستقل من G-001..G-006.</t>
         </is>
       </c>
     </row>
@@ -6718,7 +6718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6774,221 +6774,271 @@
     <row r="5">
       <c r="A5" s="53" t="inlineStr">
         <is>
+          <t>CTRL-001</t>
+        </is>
+      </c>
+      <c r="B5" s="53" t="inlineStr">
+        <is>
+          <t>اعتماد Operations Control v2</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="inlineStr">
+        <is>
+          <t>e75419504d61a60141c1776a5bfa69ed1faeb529</t>
+        </is>
+      </c>
+      <c r="D5" s="53" t="inlineStr">
+        <is>
+          <t>docs/operations/control/README.md
+https://github.com/Qays7753/Micro/pull/188
+docs/operations/control/generated/MASTER-TRACKER.md
+docs/operations/control/generated/MASTER-TRACKER.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="54" t="inlineStr">
+        <is>
+          <t>CTRL-002</t>
+        </is>
+      </c>
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>e75419504d61a60141c1776a5bfa69ed1faeb529</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="inlineStr">
+        <is>
+          <t>docs/operations/control/migration-map.md
+docs/operations/control/evidence/capability-reconciliation.md
+https://github.com/Qays7753/Micro/pull/188
+docs/operations/control/releases/pre-pilot.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="54" t="inlineStr">
+        <is>
           <t>HARD-009</t>
         </is>
       </c>
-      <c r="B5" s="53" t="inlineStr">
+      <c r="B7" s="54" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 9</t>
         </is>
       </c>
-      <c r="C5" s="53" t="inlineStr">
+      <c r="C7" s="54" t="inlineStr">
         <is>
           <t>255974a8cf66674e0a3dba477da9d9400cb28306</t>
         </is>
       </c>
-      <c r="D5" s="53" t="inlineStr">
+      <c r="D7" s="54" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="54" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="53" t="inlineStr">
         <is>
           <t>HARD-010</t>
         </is>
       </c>
-      <c r="B6" s="54" t="inlineStr">
+      <c r="B8" s="53" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 10</t>
         </is>
       </c>
-      <c r="C6" s="54" t="inlineStr">
+      <c r="C8" s="53" t="inlineStr">
         <is>
           <t>dcf60dbed79c09a06a46fcbad07e104277cb17de</t>
         </is>
       </c>
-      <c r="D6" s="54" t="inlineStr">
+      <c r="D8" s="53" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="54" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="54" t="inlineStr">
         <is>
           <t>HARD-011</t>
         </is>
       </c>
-      <c r="B7" s="54" t="inlineStr">
+      <c r="B9" s="54" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 11</t>
         </is>
       </c>
-      <c r="C7" s="54" t="inlineStr">
+      <c r="C9" s="54" t="inlineStr">
         <is>
           <t>79dac8e726b3cf5e682cb912b90d7c3757636f71</t>
         </is>
       </c>
-      <c r="D7" s="54" t="inlineStr">
+      <c r="D9" s="54" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="53" t="inlineStr">
-        <is>
-          <t>HIST-001</t>
-        </is>
-      </c>
-      <c r="B8" s="53" t="inlineStr">
-        <is>
-          <t>الموجة الأولى: إصلاحات حرجة محددة</t>
-        </is>
-      </c>
-      <c r="C8" s="53" t="inlineStr">
-        <is>
-          <t>5c54d8a</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="inlineStr">
-        <is>
-          <t>docs/operations/current-state.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
-        <is>
-          <t>HIST-002</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>الموجة الثانية: الأساسات المالية والبيانية</t>
-        </is>
-      </c>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>81d8d253984dee410c7fd6c3e461fcd0e76f327e</t>
-        </is>
-      </c>
-      <c r="D9" s="54" t="inlineStr">
-        <is>
-          <t>reports/agent-report/2026-09-17_wave-2-financial-data-foundations/report.md</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>HIST-007</t>
+          <t>HIST-001</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>الموجة 4.4: الجودة النظامية والقبول المحلي</t>
+          <t>الموجة الأولى: إصلاحات حرجة محددة</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>87ebcf2ffa74752bf385eff3a10962454b45d33e</t>
+          <t>5c54d8a</t>
         </is>
       </c>
       <c r="D10" s="54" t="inlineStr">
         <is>
-          <t>reports/agent-report/2026-09-18_wave-4-4-system-quality-final-qa/report.md</t>
+          <t>docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>HIST-003</t>
+          <t>HIST-002</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>الموجة الثالثة: العقود والملكية التقنية</t>
+          <t>الموجة الثانية: الأساسات المالية والبيانية</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t>f8b37062c14aecf85abf5f64e11a191b00eb3c0d</t>
+          <t>81d8d253984dee410c7fd6c3e461fcd0e76f327e</t>
         </is>
       </c>
       <c r="D11" s="54" t="inlineStr">
         <is>
-          <t>docs/operations/current-state.md</t>
+          <t>reports/agent-report/2026-09-17_wave-2-financial-data-foundations/report.md</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="54" t="inlineStr">
         <is>
-          <t>HIST-004</t>
+          <t>HIST-007</t>
         </is>
       </c>
       <c r="B12" s="54" t="inlineStr">
         <is>
-          <t>الموجة 4.1: مخطط تجربة المنتج</t>
+          <t>الموجة 4.4: الجودة النظامية والقبول المحلي</t>
         </is>
       </c>
       <c r="C12" s="54" t="inlineStr">
         <is>
-          <t>281a2878b61870792f76d651d0d822c7f0a5c0e1</t>
+          <t>87ebcf2ffa74752bf385eff3a10962454b45d33e</t>
         </is>
       </c>
       <c r="D12" s="54" t="inlineStr">
         <is>
-          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
+          <t>reports/agent-report/2026-09-18_wave-4-4-system-quality-final-qa/report.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="54" t="inlineStr">
         <is>
-          <t>HIST-005</t>
+          <t>HIST-003</t>
         </is>
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>الموجة 4.2: الهيكل والتنقل والتسمية</t>
+          <t>الموجة الثالثة: العقود والملكية التقنية</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">
         <is>
-          <t>9179ea785d7c35790c422a997fa210aaf7e875a6</t>
+          <t>f8b37062c14aecf85abf5f64e11a191b00eb3c0d</t>
         </is>
       </c>
       <c r="D13" s="54" t="inlineStr">
         <is>
-          <t>reports/agent-report/2026-09-17_wave-4-2-structure-navigation-naming/report.md</t>
+          <t>docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="54" t="inlineStr">
         <is>
+          <t>HIST-004</t>
+        </is>
+      </c>
+      <c r="B14" s="54" t="inlineStr">
+        <is>
+          <t>الموجة 4.1: مخطط تجربة المنتج</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>281a2878b61870792f76d651d0d822c7f0a5c0e1</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="54" t="inlineStr">
+        <is>
+          <t>HIST-005</t>
+        </is>
+      </c>
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>الموجة 4.2: الهيكل والتنقل والتسمية</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>9179ea785d7c35790c422a997fa210aaf7e875a6</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-17_wave-4-2-structure-navigation-naming/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="54" t="inlineStr">
+        <is>
           <t>HIST-006</t>
         </is>
       </c>
-      <c r="B14" s="54" t="inlineStr">
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>الموجة 4.3: إعادة بناء أسطح المنتج</t>
         </is>
       </c>
-      <c r="C14" s="54" t="inlineStr">
+      <c r="C16" s="54" t="inlineStr">
         <is>
           <t>e8a7b5a5f6678a4a93e3ab4c21814764f5895335</t>
         </is>
       </c>
-      <c r="D14" s="54" t="inlineStr">
+      <c r="D16" s="54" t="inlineStr">
         <is>
           <t>docs/operations/current-state.md</t>
         </is>
@@ -7008,7 +7058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7154,61 +7204,57 @@
     <row r="8">
       <c r="A8" s="53" t="inlineStr">
         <is>
-          <t>CTRL-001</t>
+          <t>G-001</t>
         </is>
       </c>
       <c r="B8" s="53" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="C8" s="53" t="inlineStr">
         <is>
-          <t>اعتماد Operations Control v2</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="inlineStr">
-        <is>
-          <t>اعتماد النظام بعد مراجعة المالك وAgent مستقل.</t>
-        </is>
-      </c>
+          <t>فخ الاستهلاك المزدوج عند التسليم</t>
+        </is>
+      </c>
+      <c r="D8" s="53" t="inlineStr"/>
       <c r="E8" s="53" t="inlineStr">
         <is>
-          <t>استكمل مراجعة المالك والمراجع المستقل ثم حدّث الحالة في PR نفسه.</t>
+          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="54" t="inlineStr">
         <is>
-          <t>CTRL-002</t>
+          <t>GOV-001</t>
         </is>
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
         <is>
-          <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
+          <t>مصالحة G10-A مع تعارض عقد C1</t>
         </is>
       </c>
       <c r="D9" s="54" t="inlineStr">
         <is>
-          <t>تسجيل تعريف العد ومراجعة الأدلة؛ لا يجوز حسم فرق 49/46 بقرار وصفي بلا مصفوفة مصادر.</t>
+          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
         </is>
       </c>
       <c r="E9" s="54" t="inlineStr">
         <is>
-          <t>أرفق مصفوفة الأدلة التي تحسم تعريف 49/46 ومسارات القدرة، ثم اطلب مراجعة المالك قبل فتح أي Claim كودي.</t>
+          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>G-001</t>
+          <t>G-002</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
@@ -7218,20 +7264,20 @@
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>فخ الاستهلاك المزدوج عند التسليم</t>
+          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
         </is>
       </c>
       <c r="D10" s="54" t="inlineStr"/>
       <c r="E10" s="54" t="inlineStr">
         <is>
-          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
+          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>GOV-001</t>
+          <t>G-003</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
@@ -7241,24 +7287,20 @@
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t>مصالحة G10-A مع تعارض عقد C1</t>
-        </is>
-      </c>
-      <c r="D11" s="54" t="inlineStr">
-        <is>
-          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
-        </is>
-      </c>
+          <t>حرس القراءة القديمة عند حفظ الطلب</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="inlineStr"/>
       <c r="E11" s="54" t="inlineStr">
         <is>
-          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
+          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="54" t="inlineStr">
         <is>
-          <t>G-002</t>
+          <t>G-004</t>
         </is>
       </c>
       <c r="B12" s="54" t="inlineStr">
@@ -7268,20 +7310,20 @@
       </c>
       <c r="C12" s="54" t="inlineStr">
         <is>
-          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
+          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
         </is>
       </c>
       <c r="D12" s="54" t="inlineStr"/>
       <c r="E12" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
+          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="54" t="inlineStr">
         <is>
-          <t>G-003</t>
+          <t>G-005</t>
         </is>
       </c>
       <c r="B13" s="54" t="inlineStr">
@@ -7291,20 +7333,20 @@
       </c>
       <c r="C13" s="54" t="inlineStr">
         <is>
-          <t>حرس القراءة القديمة عند حفظ الطلب</t>
+          <t>عزل فشل قراءات صفحة المالية</t>
         </is>
       </c>
       <c r="D13" s="54" t="inlineStr"/>
       <c r="E13" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
+          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="54" t="inlineStr">
         <is>
-          <t>G-004</t>
+          <t>G-006</t>
         </is>
       </c>
       <c r="B14" s="54" t="inlineStr">
@@ -7314,66 +7356,74 @@
       </c>
       <c r="C14" s="54" t="inlineStr">
         <is>
-          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
+          <t>توحيد حرس السحب بين مساري مال المالك</t>
         </is>
       </c>
       <c r="D14" s="54" t="inlineStr"/>
       <c r="E14" s="54" t="inlineStr">
         <is>
-          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
+          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="54" t="inlineStr">
         <is>
-          <t>G-005</t>
+          <t>SCOPE-001</t>
         </is>
       </c>
       <c r="B15" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C15" s="54" t="inlineStr">
         <is>
-          <t>عزل فشل قراءات صفحة المالية</t>
-        </is>
-      </c>
-      <c r="D15" s="54" t="inlineStr"/>
+          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+        </is>
+      </c>
       <c r="E15" s="54" t="inlineStr">
         <is>
-          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="54" t="inlineStr">
         <is>
-          <t>G-006</t>
+          <t>UX-001</t>
         </is>
       </c>
       <c r="B16" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C16" s="54" t="inlineStr">
         <is>
-          <t>توحيد حرس السحب بين مساري مال المالك</t>
-        </is>
-      </c>
-      <c r="D16" s="54" t="inlineStr"/>
+          <t>إعادة تصميم UI وUX جذرية</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="inlineStr">
+        <is>
+          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+        </is>
+      </c>
       <c r="E16" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
+          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-001</t>
+          <t>BE-001</t>
         </is>
       </c>
       <c r="B17" s="54" t="inlineStr">
@@ -7383,24 +7433,24 @@
       </c>
       <c r="C17" s="54" t="inlineStr">
         <is>
-          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
+          <t>مصاريف متكررة محلية</t>
         </is>
       </c>
       <c r="D17" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
         </is>
       </c>
       <c r="E17" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="54" t="inlineStr">
         <is>
-          <t>UX-001</t>
+          <t>BE-002</t>
         </is>
       </c>
       <c r="B18" s="54" t="inlineStr">
@@ -7410,24 +7460,24 @@
       </c>
       <c r="C18" s="54" t="inlineStr">
         <is>
-          <t>إعادة تصميم UI وUX جذرية</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="D18" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
         </is>
       </c>
       <c r="E18" s="54" t="inlineStr">
         <is>
-          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="54" t="inlineStr">
         <is>
-          <t>BE-001</t>
+          <t>BE-003</t>
         </is>
       </c>
       <c r="B19" s="54" t="inlineStr">
@@ -7437,7 +7487,7 @@
       </c>
       <c r="C19" s="54" t="inlineStr">
         <is>
-          <t>مصاريف متكررة محلية</t>
+          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="D19" s="54" t="inlineStr">
@@ -7447,14 +7497,14 @@
       </c>
       <c r="E19" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="54" t="inlineStr">
         <is>
-          <t>BE-002</t>
+          <t>BE-004</t>
         </is>
       </c>
       <c r="B20" s="54" t="inlineStr">
@@ -7464,24 +7514,24 @@
       </c>
       <c r="C20" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>إغلاق فترة رسمي</t>
         </is>
       </c>
       <c r="D20" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="E20" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="54" t="inlineStr">
         <is>
-          <t>BE-003</t>
+          <t>BE-005</t>
         </is>
       </c>
       <c r="B21" s="54" t="inlineStr">
@@ -7491,24 +7541,24 @@
       </c>
       <c r="C21" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
+          <t>تقادم الديون بشرائح 30/60/90</t>
         </is>
       </c>
       <c r="D21" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="E21" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="54" t="inlineStr">
         <is>
-          <t>BE-004</t>
+          <t>FIN-002</t>
         </is>
       </c>
       <c r="B22" s="54" t="inlineStr">
@@ -7518,24 +7568,24 @@
       </c>
       <c r="C22" s="54" t="inlineStr">
         <is>
-          <t>إغلاق فترة رسمي</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="D22" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="E22" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="54" t="inlineStr">
         <is>
-          <t>BE-005</t>
+          <t>FIN-006</t>
         </is>
       </c>
       <c r="B23" s="54" t="inlineStr">
@@ -7545,24 +7595,24 @@
       </c>
       <c r="C23" s="54" t="inlineStr">
         <is>
-          <t>تقادم الديون بشرائح 30/60/90</t>
+          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="D23" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="E23" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="54" t="inlineStr">
         <is>
-          <t>FIN-002</t>
+          <t>FIN-008</t>
         </is>
       </c>
       <c r="B24" s="54" t="inlineStr">
@@ -7572,24 +7622,24 @@
       </c>
       <c r="C24" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>تحقق الإهلاك بعد مرور الزمن</t>
         </is>
       </c>
       <c r="D24" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
         </is>
       </c>
       <c r="E24" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
+          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="54" t="inlineStr">
         <is>
-          <t>FIN-006</t>
+          <t>OPS-003</t>
         </is>
       </c>
       <c r="B25" s="54" t="inlineStr">
@@ -7599,24 +7649,24 @@
       </c>
       <c r="C25" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
+          <t>المصروفات المتكررة المحلية</t>
         </is>
       </c>
       <c r="D25" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
         </is>
       </c>
       <c r="E25" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="54" t="inlineStr">
         <is>
-          <t>FIN-008</t>
+          <t>SCOPE-002</t>
         </is>
       </c>
       <c r="B26" s="54" t="inlineStr">
@@ -7626,24 +7676,24 @@
       </c>
       <c r="C26" s="54" t="inlineStr">
         <is>
-          <t>تحقق الإهلاك بعد مرور الزمن</t>
+          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
         </is>
       </c>
       <c r="D26" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="E26" s="54" t="inlineStr">
         <is>
-          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="54" t="inlineStr">
         <is>
-          <t>OPS-003</t>
+          <t>UX-002</t>
         </is>
       </c>
       <c r="B27" s="54" t="inlineStr">
@@ -7653,24 +7703,24 @@
       </c>
       <c r="C27" s="54" t="inlineStr">
         <is>
-          <t>المصروفات المتكررة المحلية</t>
+          <t>Backlog الموجة الرابعة في عقد الملكية</t>
         </is>
       </c>
       <c r="D27" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="E27" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-002</t>
+          <t>V-001</t>
         </is>
       </c>
       <c r="B28" s="54" t="inlineStr">
@@ -7680,24 +7730,24 @@
       </c>
       <c r="C28" s="54" t="inlineStr">
         <is>
-          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
+          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
         </is>
       </c>
       <c r="D28" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E28" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="54" t="inlineStr">
         <is>
-          <t>UX-002</t>
+          <t>V-002</t>
         </is>
       </c>
       <c r="B29" s="54" t="inlineStr">
@@ -7707,24 +7757,24 @@
       </c>
       <c r="C29" s="54" t="inlineStr">
         <is>
-          <t>Backlog الموجة الرابعة في عقد الملكية</t>
+          <t>V-02 — متوقعات الكاش القصيرة</t>
         </is>
       </c>
       <c r="D29" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E29" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="54" t="inlineStr">
         <is>
-          <t>V-001</t>
+          <t>V-003</t>
         </is>
       </c>
       <c r="B30" s="54" t="inlineStr">
@@ -7734,7 +7784,7 @@
       </c>
       <c r="C30" s="54" t="inlineStr">
         <is>
-          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
+          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
         </is>
       </c>
       <c r="D30" s="54" t="inlineStr">
@@ -7751,7 +7801,7 @@
     <row r="31">
       <c r="A31" s="54" t="inlineStr">
         <is>
-          <t>V-002</t>
+          <t>V-004</t>
         </is>
       </c>
       <c r="B31" s="54" t="inlineStr">
@@ -7761,7 +7811,7 @@
       </c>
       <c r="C31" s="54" t="inlineStr">
         <is>
-          <t>V-02 — متوقعات الكاش القصيرة</t>
+          <t>V-04 — عرض التغطية عند قرار السحب</t>
         </is>
       </c>
       <c r="D31" s="54" t="inlineStr">
@@ -7778,7 +7828,7 @@
     <row r="32">
       <c r="A32" s="54" t="inlineStr">
         <is>
-          <t>V-003</t>
+          <t>V-005</t>
         </is>
       </c>
       <c r="B32" s="54" t="inlineStr">
@@ -7788,7 +7838,7 @@
       </c>
       <c r="C32" s="54" t="inlineStr">
         <is>
-          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
+          <t>V-05 — مقارنة فترتين بسيطة</t>
         </is>
       </c>
       <c r="D32" s="54" t="inlineStr">
@@ -7805,7 +7855,7 @@
     <row r="33">
       <c r="A33" s="54" t="inlineStr">
         <is>
-          <t>V-004</t>
+          <t>V-006</t>
         </is>
       </c>
       <c r="B33" s="54" t="inlineStr">
@@ -7815,7 +7865,7 @@
       </c>
       <c r="C33" s="54" t="inlineStr">
         <is>
-          <t>V-04 — عرض التغطية عند قرار السحب</t>
+          <t>V-06 — جسر ربح إلى كاش رقمي</t>
         </is>
       </c>
       <c r="D33" s="54" t="inlineStr">
@@ -7832,7 +7882,7 @@
     <row r="34">
       <c r="A34" s="54" t="inlineStr">
         <is>
-          <t>V-005</t>
+          <t>V-007</t>
         </is>
       </c>
       <c r="B34" s="54" t="inlineStr">
@@ -7842,7 +7892,7 @@
       </c>
       <c r="C34" s="54" t="inlineStr">
         <is>
-          <t>V-05 — مقارنة فترتين بسيطة</t>
+          <t>V-07 — تنبيه انخفاض المواد</t>
         </is>
       </c>
       <c r="D34" s="54" t="inlineStr">
@@ -7859,7 +7909,7 @@
     <row r="35">
       <c r="A35" s="54" t="inlineStr">
         <is>
-          <t>V-006</t>
+          <t>V-008</t>
         </is>
       </c>
       <c r="B35" s="54" t="inlineStr">
@@ -7869,7 +7919,7 @@
       </c>
       <c r="C35" s="54" t="inlineStr">
         <is>
-          <t>V-06 — جسر ربح إلى كاش رقمي</t>
+          <t>V-08 — مصروف اليوم على الرئيسية</t>
         </is>
       </c>
       <c r="D35" s="54" t="inlineStr">
@@ -7886,7 +7936,7 @@
     <row r="36">
       <c r="A36" s="54" t="inlineStr">
         <is>
-          <t>V-007</t>
+          <t>V-009</t>
         </is>
       </c>
       <c r="B36" s="54" t="inlineStr">
@@ -7896,7 +7946,7 @@
       </c>
       <c r="C36" s="54" t="inlineStr">
         <is>
-          <t>V-07 — تنبيه انخفاض المواد</t>
+          <t>V-09 — رقم السحب الآمن الموحد</t>
         </is>
       </c>
       <c r="D36" s="54" t="inlineStr">
@@ -7913,7 +7963,7 @@
     <row r="37">
       <c r="A37" s="54" t="inlineStr">
         <is>
-          <t>V-008</t>
+          <t>V-010</t>
         </is>
       </c>
       <c r="B37" s="54" t="inlineStr">
@@ -7923,7 +7973,7 @@
       </c>
       <c r="C37" s="54" t="inlineStr">
         <is>
-          <t>V-08 — مصروف اليوم على الرئيسية</t>
+          <t>V-10 — كثافة صفحة المالية</t>
         </is>
       </c>
       <c r="D37" s="54" t="inlineStr">
@@ -7940,7 +7990,7 @@
     <row r="38">
       <c r="A38" s="54" t="inlineStr">
         <is>
-          <t>V-009</t>
+          <t>V-011</t>
         </is>
       </c>
       <c r="B38" s="54" t="inlineStr">
@@ -7950,7 +8000,7 @@
       </c>
       <c r="C38" s="54" t="inlineStr">
         <is>
-          <t>V-09 — رقم السحب الآمن الموحد</t>
+          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
         </is>
       </c>
       <c r="D38" s="54" t="inlineStr">
@@ -7967,7 +8017,7 @@
     <row r="39">
       <c r="A39" s="54" t="inlineStr">
         <is>
-          <t>V-010</t>
+          <t>V-012</t>
         </is>
       </c>
       <c r="B39" s="54" t="inlineStr">
@@ -7977,7 +8027,7 @@
       </c>
       <c r="C39" s="54" t="inlineStr">
         <is>
-          <t>V-10 — كثافة صفحة المالية</t>
+          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
         </is>
       </c>
       <c r="D39" s="54" t="inlineStr">
@@ -7986,60 +8036,6 @@
         </is>
       </c>
       <c r="E39" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="54" t="inlineStr">
-        <is>
-          <t>V-011</t>
-        </is>
-      </c>
-      <c r="B40" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C40" s="54" t="inlineStr">
-        <is>
-          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
-        </is>
-      </c>
-      <c r="D40" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E40" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="54" t="inlineStr">
-        <is>
-          <t>V-012</t>
-        </is>
-      </c>
-      <c r="B41" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C41" s="54" t="inlineStr">
-        <is>
-          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
-        </is>
-      </c>
-      <c r="D41" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E41" s="54" t="inlineStr">
         <is>
           <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
@@ -8606,7 +8602,7 @@
       </c>
       <c r="B5" s="53" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C5" s="53" t="inlineStr">
@@ -8638,7 +8634,7 @@
       </c>
       <c r="B6" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C6" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): claim WS-162 for pre-pilot safety Package A (G-001/G-002/G-003/G-006)
Items move REVIEW_REQUIRED -> IN_PROGRESS per the Operations Control v2 cycle.
Base SHA 3702c90 (origin/main, CI green). Branch fix/pre-pilot-safety-a-b.
Scope: four safety fixes only; no schema/export change (35/27); no refactoring.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -684,14 +684,6 @@
           <t>Micro Operations Control</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
-      <c r="D2" s="53" t="n"/>
-      <c r="E2" s="53" t="n"/>
-      <c r="F2" s="53" t="n"/>
-      <c r="G2" s="53" t="n"/>
-      <c r="H2" s="53" t="n"/>
-      <c r="I2" s="53" t="n"/>
       <c r="J2" s="53" t="n"/>
       <c r="K2" s="53" t="n"/>
       <c r="L2" s="53" t="n"/>
@@ -707,14 +699,6 @@
           <t>واجهة قراءة مولّدة من JSON المصدر. لا تُحرّر يدويًا.</t>
         </is>
       </c>
-      <c r="B3" s="54" t="n"/>
-      <c r="C3" s="54" t="n"/>
-      <c r="D3" s="54" t="n"/>
-      <c r="E3" s="54" t="n"/>
-      <c r="F3" s="54" t="n"/>
-      <c r="G3" s="54" t="n"/>
-      <c r="H3" s="54" t="n"/>
-      <c r="I3" s="54" t="n"/>
       <c r="J3" s="54" t="n"/>
       <c r="K3" s="54" t="n"/>
       <c r="L3" s="54" t="n"/>
@@ -2576,7 +2560,7 @@
       </c>
       <c r="D29" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E29" s="54" t="inlineStr">
@@ -2618,7 +2602,7 @@
       <c r="M29" s="54" t="inlineStr"/>
       <c r="N29" s="54" t="inlineStr">
         <is>
-          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
+          <t>تنفيذ الحارس على مستوى العرض وحد الكتابة مع اختبارات المسارين داخل WS-162.</t>
         </is>
       </c>
       <c r="O29" s="54" t="inlineStr"/>
@@ -2629,7 +2613,7 @@
       </c>
       <c r="Q29" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2714,7 @@
       </c>
       <c r="D31" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E31" s="54" t="inlineStr">
@@ -2772,7 +2756,7 @@
       <c r="M31" s="54" t="inlineStr"/>
       <c r="N31" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
+          <t>تنفيذ الالتزام الذرّي/الشفاء الحتمي لتخصيص المحفظة مع اختبارات الفشل المحقون داخل WS-162.</t>
         </is>
       </c>
       <c r="O31" s="54" t="inlineStr"/>
@@ -2783,7 +2767,7 @@
       </c>
       <c r="Q31" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2789,7 @@
       </c>
       <c r="D32" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E32" s="54" t="inlineStr">
@@ -2847,7 +2831,7 @@
       <c r="M32" s="54" t="inlineStr"/>
       <c r="N32" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
+          <t>تنفيذ حارس storage_stale لمسارات كتابة الطلب وفق العقد المعتمد داخل WS-162.</t>
         </is>
       </c>
       <c r="O32" s="54" t="inlineStr"/>
@@ -2858,7 +2842,7 @@
       </c>
       <c r="Q32" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3014,7 @@
       </c>
       <c r="D35" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E35" s="54" t="inlineStr">
@@ -3072,7 +3056,7 @@
       <c r="M35" s="54" t="inlineStr"/>
       <c r="N35" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
+          <t>توحيد حرس تغطية المحفظة لمساري سحب المالك مع اختبارات التكافؤ داخل WS-162.</t>
         </is>
       </c>
       <c r="O35" s="54" t="inlineStr"/>
@@ -3083,7 +3067,7 @@
       </c>
       <c r="Q35" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6044,8 +6028,6 @@
           <t>سجل تحديث نظام التحكم</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="54" t="n"/>
@@ -6134,6 +6116,23 @@
       <c r="C8" s="53" t="inlineStr">
         <is>
           <t>CTRL-002 / evidence/hardening-main-verification.md / pre-pilot.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>فتح Claim WS-162 وتحرك G-001/G-002/G-003/G-006 إلى IN_PROGRESS (الحزمة أ)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>WS-162</t>
         </is>
       </c>
     </row>
@@ -6151,7 +6150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6170,8 +6169,6 @@
           <t>حالة البرنامج</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="54" t="n"/>
@@ -6232,7 +6229,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6241,71 +6238,87 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="53" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>تنفيذ جارٍ ضمن Claim نشط</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="53" t="inlineStr">
         <is>
           <t>BLOCKED / DEFERRED</t>
         </is>
       </c>
-      <c r="B8" s="53" t="n">
+      <c r="B9" s="53" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="53" t="inlineStr">
+      <c r="C9" s="53" t="inlineStr">
         <is>
           <t>بوابة أو دليل مؤجل</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
-        <is>
-          <t>main SHA</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>87ebcf2ffa74752bf385eff3a10962454b45d33e</t>
-        </is>
-      </c>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>PRE-PILOT</t>
+          <t>main SHA</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>3702c90131472c7ebb117dc0d7d67cd96a47cfc6</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
+          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
+          <t>PRE-PILOT</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
           <t>السياق الدائم</t>
         </is>
       </c>
-      <c r="B11" s="54" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>docs/operations/control/context.md</t>
         </is>
       </c>
-      <c r="C11" s="54" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>الخطة والأدوار ومصادر السلطة</t>
         </is>
       </c>
     </row>
+    <row r="13"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:C2"/>
@@ -6339,8 +6352,6 @@
           <t>خارطة Micro الكاملة قبل الـPilot</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="54" t="n"/>
@@ -6543,7 +6554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6568,11 +6579,6 @@
           <t>العمل الجاري والمراجعة</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
-      <c r="D2" s="53" t="n"/>
-      <c r="E2" s="53" t="n"/>
-      <c r="F2" s="53" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="54" t="n"/>
@@ -6701,6 +6707,33 @@
       <c r="F7" s="54" t="inlineStr">
         <is>
           <t>لا إجراء؛ PR #161 مغلق موثقًا. احتفظ بالرابط كسجل تاريخي ولا تعاود المطالبة به.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WS-162</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CLAIMED</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>fix/pre-pilot-safety-a-b</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>G-001, G-002, G-003, G-006</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>تنفيذ إصلاحات الحزمة أ مع الاختبارات المركزة ثم فتح PR للحزمة أ على الفرع fix/pre-pilot-safety-a-b.</t>
         </is>
       </c>
     </row>
@@ -6739,9 +6772,6 @@
           <t>المنجز والمتحقق على main</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
-      <c r="D2" s="53" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="54" t="n"/>
@@ -7081,9 +7111,6 @@
           <t>المحجوب والمؤجل والمحتاج مراجعة</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
-      <c r="D2" s="53" t="n"/>
       <c r="E2" s="53" t="n"/>
     </row>
     <row r="3">
@@ -8072,7 +8099,6 @@
           <t>قرارات ثابتة لا يعاد اختراعها</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="54" t="n"/>
@@ -8257,9 +8283,6 @@
           <t>فهرس التقارير</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
-      <c r="D2" s="53" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="54" t="n"/>
@@ -8548,8 +8571,6 @@
           <t>بوابات ما قبل الـPilot</t>
         </is>
       </c>
-      <c r="B2" s="53" t="n"/>
-      <c r="C2" s="53" t="n"/>
       <c r="D2" s="53" t="n"/>
       <c r="E2" s="53" t="n"/>
       <c r="F2" s="53" t="n"/>

</xml_diff>

<commit_message>
docs(operations): Package A IN_REVIEW — PR #190, execution report, QA record, current-state §41
Items G-001/G-002/G-003/G-006 and WS-162 move to IN_REVIEW (actor pr:190).
Report + test-results under reports/agent-report/2026-09-20_pre-pilot-safety-package-a/.
QA record under docs/quality/. Views/Excel/meta regenerated and validated.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2560,7 +2560,7 @@
       </c>
       <c r="D29" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E29" s="54" t="inlineStr">
@@ -2602,7 +2602,7 @@
       <c r="M29" s="54" t="inlineStr"/>
       <c r="N29" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ الحارس على مستوى العرض وحد الكتابة مع اختبارات المسارين داخل WS-162.</t>
+          <t>مراجعة المالك لـPR #190 (الحزمة أ) ثم الدمج والتحقق على main.</t>
         </is>
       </c>
       <c r="O29" s="54" t="inlineStr"/>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="D31" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E31" s="54" t="inlineStr">
@@ -2756,7 +2756,7 @@
       <c r="M31" s="54" t="inlineStr"/>
       <c r="N31" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ الالتزام الذرّي/الشفاء الحتمي لتخصيص المحفظة مع اختبارات الفشل المحقون داخل WS-162.</t>
+          <t>مراجعة المالك لـPR #190 (الحزمة أ) ثم الدمج والتحقق على main.</t>
         </is>
       </c>
       <c r="O31" s="54" t="inlineStr"/>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="D32" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E32" s="54" t="inlineStr">
@@ -2831,7 +2831,7 @@
       <c r="M32" s="54" t="inlineStr"/>
       <c r="N32" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ حارس storage_stale لمسارات كتابة الطلب وفق العقد المعتمد داخل WS-162.</t>
+          <t>مراجعة المالك لـPR #190 (الحزمة أ) ثم الدمج والتحقق على main.</t>
         </is>
       </c>
       <c r="O32" s="54" t="inlineStr"/>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="D35" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E35" s="54" t="inlineStr">
@@ -3056,7 +3056,7 @@
       <c r="M35" s="54" t="inlineStr"/>
       <c r="N35" s="54" t="inlineStr">
         <is>
-          <t>توحيد حرس تغطية المحفظة لمساري سحب المالك مع اختبارات التكافؤ داخل WS-162.</t>
+          <t>مراجعة المالك لـPR #190 (الحزمة أ) ثم الدمج والتحقق على main.</t>
         </is>
       </c>
       <c r="O35" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6133,6 +6133,23 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>WS-162</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>اكتمال تنفيذ الحزمة أ وفتح PR #190 — G-001/G-002/G-003/G-006 إلى IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>WS-162 / PR #190</t>
         </is>
       </c>
     </row>
@@ -6150,7 +6167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6229,7 +6246,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6244,7 +6261,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -6318,7 +6335,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:C2"/>
@@ -6718,13 +6734,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
           <t>fix/pre-pilot-safety-a-b</t>
         </is>
+      </c>
+      <c r="D8" t="n">
+        <v>190</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs(operations): claim WS-163 (stacked on Package A head) for Package B (G-004/G-005)
Items move REVIEW_REQUIRED -> IN_PROGRESS. Disjoint areas/contracts from active WS-162
per validator overlap rules. Branch fix/pre-pilot-safety-b from b44edcd.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2864,7 +2864,7 @@
       </c>
       <c r="D33" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E33" s="54" t="inlineStr">
@@ -2906,7 +2906,7 @@
       <c r="M33" s="54" t="inlineStr"/>
       <c r="N33" s="54" t="inlineStr">
         <is>
-          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
+          <t>تنفيذ حرس تعطيل القدرات المركزي على كل أسطح الإنشاء والروابط العميقة داخل WS-163.</t>
         </is>
       </c>
       <c r="O33" s="54" t="inlineStr"/>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="Q33" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="D34" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E34" s="54" t="inlineStr">
@@ -2981,7 +2981,7 @@
       <c r="M34" s="54" t="inlineStr"/>
       <c r="N34" s="54" t="inlineStr">
         <is>
-          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
+          <t>تنفيذ عزل فشل قراءات صفحة المالية في كتل مستقلة داخل WS-163.</t>
         </is>
       </c>
       <c r="O34" s="54" t="inlineStr"/>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="Q34" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6150,6 +6150,23 @@
       <c r="C10" t="inlineStr">
         <is>
           <t>WS-162 / PR #190</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>فتح Claim WS-163 المكدّس لتحرك G-004/G-005 إلى IN_PROGRESS (الحزمة ب)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>WS-163</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6263,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6261,7 +6278,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -6570,7 +6587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6753,6 +6770,33 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>تنفيذ إصلاحات الحزمة أ مع الاختبارات المركزة ثم فتح PR للحزمة أ على الفرع fix/pre-pilot-safety-a-b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WS-163</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CLAIMED</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>fix/pre-pilot-safety-b</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>G-004, G-005</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>تنفيذ إصلاحات الحزمة ب مع الاختبارات المركزة ثم فتح PR للحزمة ب من رأس الحزمة أ نفسه (b44edcd).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(operations): Package B IN_REVIEW — PR #191, execution report, QA record, current-state §42
Items G-004/G-005 and WS-163 move to IN_REVIEW (actor pr:191).
Report + test-results under reports/agent-report/2026-09-20_pre-pilot-safety-package-b/.
QA record under docs/quality/. Views/Excel/meta regenerated and validated; the
workbook rebuild also completes the sheet refresh Package A's edit had left
partial (Blocked-Deferred G-rows now correctly leave the review-needed sheet,
Release-Gate current-status column updated, and the PRE-PILOT-SAFETY-A report
row added alongside PRE-PILOT-SAFETY-B).
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2864,7 +2864,7 @@
       </c>
       <c r="D33" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E33" s="54" t="inlineStr">
@@ -2906,7 +2906,7 @@
       <c r="M33" s="54" t="inlineStr"/>
       <c r="N33" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ حرس تعطيل القدرات المركزي على كل أسطح الإنشاء والروابط العميقة داخل WS-163.</t>
+          <t>مراجعة المالك لـPR #191 (الحزمة ب) ثم الدمج والتحقق على main بعد دمج الحزمة أ (PR #190).</t>
         </is>
       </c>
       <c r="O33" s="54" t="inlineStr"/>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="D34" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E34" s="54" t="inlineStr">
@@ -2981,7 +2981,7 @@
       <c r="M34" s="54" t="inlineStr"/>
       <c r="N34" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ عزل فشل قراءات صفحة المالية في كتل مستقلة داخل WS-163.</t>
+          <t>مراجعة المالك لـPR #191 (الحزمة ب) ثم الدمج والتحقق على main بعد دمج الحزمة أ (PR #190).</t>
         </is>
       </c>
       <c r="O34" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6167,6 +6167,23 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>WS-163</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>اكتمال تنفيذ الحزمة ب وفتح PR #191 المكدّس — G-004/G-005 إلى IN_REVIEW وتحديث صفحة Excel كاملة (المحجوب/بوابات ما قبل الـPilot/فهرس التقارير)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>WS-163 / PR #191</t>
         </is>
       </c>
     </row>
@@ -6184,7 +6201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6263,7 +6280,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6272,81 +6289,66 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>تنفيذ جارٍ ضمن Claim نشط</t>
+      <c r="A8" s="53" t="inlineStr">
+        <is>
+          <t>BLOCKED / DEFERRED</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>بوابة أو دليل مؤجل</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="53" t="inlineStr">
-        <is>
-          <t>BLOCKED / DEFERRED</t>
-        </is>
-      </c>
-      <c r="B9" s="53" t="n">
-        <v>28</v>
-      </c>
-      <c r="C9" s="53" t="inlineStr">
-        <is>
-          <t>بوابة أو دليل مؤجل</t>
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>main SHA</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>3702c90131472c7ebb117dc0d7d67cd96a47cfc6</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>main SHA</t>
+          <t>PRE-PILOT</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>3702c90131472c7ebb117dc0d7d67cd96a47cfc6</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>يجب تثبيته قبل أي تنفيذ</t>
+          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>PRE-PILOT</t>
+          <t>السياق الدائم</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>docs/operations/control/context.md</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
-        <is>
-          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="54" t="inlineStr">
-        <is>
-          <t>السياق الدائم</t>
-        </is>
-      </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>docs/operations/control/context.md</t>
-        </is>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>الخطة والأدوار ومصادر السلطة</t>
         </is>
@@ -6781,7 +6783,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -6789,6 +6791,9 @@
           <t>fix/pre-pilot-safety-b</t>
         </is>
       </c>
+      <c r="D9" t="n">
+        <v>191</v>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>G-004, G-005</t>
@@ -6796,7 +6801,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>تنفيذ إصلاحات الحزمة ب مع الاختبارات المركزة ثم فتح PR للحزمة ب من رأس الحزمة أ نفسه (b44edcd).</t>
+          <t>مراجعة المالك لـPR #191 ثم الدمج والتحقق على main بعد دمج الحزمة أ (PR #190).</t>
         </is>
       </c>
     </row>
@@ -7151,7 +7156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7292,174 +7297,198 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="53" t="inlineStr">
-        <is>
-          <t>G-001</t>
-        </is>
-      </c>
-      <c r="B8" s="53" t="inlineStr">
+      <c r="A8" s="54" t="inlineStr">
+        <is>
+          <t>GOV-001</t>
+        </is>
+      </c>
+      <c r="B8" s="54" t="inlineStr">
         <is>
           <t>REVIEW_REQUIRED</t>
         </is>
       </c>
-      <c r="C8" s="53" t="inlineStr">
-        <is>
-          <t>فخ الاستهلاك المزدوج عند التسليم</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="inlineStr"/>
-      <c r="E8" s="53" t="inlineStr">
-        <is>
-          <t>إغلاق الحارس على مستوى العرض والكتابة واختبار المسارين معًا.</t>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>مصالحة G10-A مع تعارض عقد C1</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="inlineStr">
+        <is>
+          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
+        </is>
+      </c>
+      <c r="E8" s="54" t="inlineStr">
+        <is>
+          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="54" t="inlineStr">
         <is>
-          <t>GOV-001</t>
+          <t>SCOPE-001</t>
         </is>
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
         <is>
-          <t>مصالحة G10-A مع تعارض عقد C1</t>
+          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
         </is>
       </c>
       <c r="D9" s="54" t="inlineStr">
         <is>
-          <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="E9" s="54" t="inlineStr">
         <is>
-          <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>G-002</t>
+          <t>UX-001</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
-        </is>
-      </c>
-      <c r="D10" s="54" t="inlineStr"/>
+          <t>إعادة تصميم UI وUX جذرية</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="inlineStr">
+        <is>
+          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+        </is>
+      </c>
       <c r="E10" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم فتح Claim مستقل لإصلاح الذرية وإعادة المحاولة.</t>
+          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>G-003</t>
+          <t>BE-001</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t>حرس القراءة القديمة عند حفظ الطلب</t>
-        </is>
-      </c>
-      <c r="D11" s="54" t="inlineStr"/>
+          <t>مصاريف متكررة محلية</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="inlineStr">
+        <is>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+        </is>
+      </c>
       <c r="E11" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الدليل ثم اعتماد عقد storage_stale قبل أي إصلاح.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="54" t="inlineStr">
         <is>
-          <t>G-004</t>
+          <t>BE-002</t>
         </is>
       </c>
       <c r="B12" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C12" s="54" t="inlineStr">
         <is>
-          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
-        </is>
-      </c>
-      <c r="D12" s="54" t="inlineStr"/>
+          <t>ميزانيات وأهداف بسيطة</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
+        <is>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+        </is>
+      </c>
       <c r="E12" s="54" t="inlineStr">
         <is>
-          <t>مراجعة قرار الوعد ثم اختيار إصلاح العرض أو تضييق النص بعقد واضح.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="54" t="inlineStr">
         <is>
-          <t>G-005</t>
+          <t>BE-003</t>
         </is>
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">
         <is>
-          <t>عزل فشل قراءات صفحة المالية</t>
-        </is>
-      </c>
-      <c r="D13" s="54" t="inlineStr"/>
+          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
+        </is>
+      </c>
+      <c r="D13" s="54" t="inlineStr">
+        <is>
+          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+        </is>
+      </c>
       <c r="E13" s="54" t="inlineStr">
         <is>
-          <t>تقييم خطر القراءة ثم إنشاء Claim للتجزئة إذا أقر المالك النطاق.</t>
+          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="54" t="inlineStr">
         <is>
-          <t>G-006</t>
+          <t>BE-004</t>
         </is>
       </c>
       <c r="B14" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="C14" s="54" t="inlineStr">
         <is>
-          <t>توحيد حرس السحب بين مساري مال المالك</t>
-        </is>
-      </c>
-      <c r="D14" s="54" t="inlineStr"/>
+          <t>إغلاق فترة رسمي</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+        </is>
+      </c>
       <c r="E14" s="54" t="inlineStr">
         <is>
-          <t>مراجعة الملاحظة كتحسين P3 وتحديد ما إذا كان الحارس مطلوبًا قبل Pilot.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-001</t>
+          <t>BE-005</t>
         </is>
       </c>
       <c r="B15" s="54" t="inlineStr">
@@ -7469,24 +7498,24 @@
       </c>
       <c r="C15" s="54" t="inlineStr">
         <is>
-          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
+          <t>تقادم الديون بشرائح 30/60/90</t>
         </is>
       </c>
       <c r="D15" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
         </is>
       </c>
       <c r="E15" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="54" t="inlineStr">
         <is>
-          <t>UX-001</t>
+          <t>FIN-002</t>
         </is>
       </c>
       <c r="B16" s="54" t="inlineStr">
@@ -7496,24 +7525,24 @@
       </c>
       <c r="C16" s="54" t="inlineStr">
         <is>
-          <t>إعادة تصميم UI وUX جذرية</t>
+          <t>ميزانيات وأهداف بسيطة</t>
         </is>
       </c>
       <c r="D16" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="E16" s="54" t="inlineStr">
         <is>
-          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="54" t="inlineStr">
         <is>
-          <t>BE-001</t>
+          <t>FIN-006</t>
         </is>
       </c>
       <c r="B17" s="54" t="inlineStr">
@@ -7523,24 +7552,24 @@
       </c>
       <c r="C17" s="54" t="inlineStr">
         <is>
-          <t>مصاريف متكررة محلية</t>
+          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
         </is>
       </c>
       <c r="D17" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
         </is>
       </c>
       <c r="E17" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="54" t="inlineStr">
         <is>
-          <t>BE-002</t>
+          <t>FIN-008</t>
         </is>
       </c>
       <c r="B18" s="54" t="inlineStr">
@@ -7550,24 +7579,24 @@
       </c>
       <c r="C18" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>تحقق الإهلاك بعد مرور الزمن</t>
         </is>
       </c>
       <c r="D18" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
         </is>
       </c>
       <c r="E18" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="54" t="inlineStr">
         <is>
-          <t>BE-003</t>
+          <t>OPS-003</t>
         </is>
       </c>
       <c r="B19" s="54" t="inlineStr">
@@ -7577,24 +7606,24 @@
       </c>
       <c r="C19" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
+          <t>المصروفات المتكررة المحلية</t>
         </is>
       </c>
       <c r="D19" s="54" t="inlineStr">
         <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
+          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
         </is>
       </c>
       <c r="E19" s="54" t="inlineStr">
         <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
+          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="54" t="inlineStr">
         <is>
-          <t>BE-004</t>
+          <t>SCOPE-002</t>
         </is>
       </c>
       <c r="B20" s="54" t="inlineStr">
@@ -7604,24 +7633,24 @@
       </c>
       <c r="C20" s="54" t="inlineStr">
         <is>
-          <t>إغلاق فترة رسمي</t>
+          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
         </is>
       </c>
       <c r="D20" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="E20" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="54" t="inlineStr">
         <is>
-          <t>BE-005</t>
+          <t>UX-002</t>
         </is>
       </c>
       <c r="B21" s="54" t="inlineStr">
@@ -7631,24 +7660,24 @@
       </c>
       <c r="C21" s="54" t="inlineStr">
         <is>
-          <t>تقادم الديون بشرائح 30/60/90</t>
+          <t>Backlog الموجة الرابعة في عقد الملكية</t>
         </is>
       </c>
       <c r="D21" s="54" t="inlineStr">
         <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
+          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
         </is>
       </c>
       <c r="E21" s="54" t="inlineStr">
         <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
+          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="54" t="inlineStr">
         <is>
-          <t>FIN-002</t>
+          <t>V-001</t>
         </is>
       </c>
       <c r="B22" s="54" t="inlineStr">
@@ -7658,24 +7687,24 @@
       </c>
       <c r="C22" s="54" t="inlineStr">
         <is>
-          <t>ميزانيات وأهداف بسيطة</t>
+          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
         </is>
       </c>
       <c r="D22" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E22" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="54" t="inlineStr">
         <is>
-          <t>FIN-006</t>
+          <t>V-002</t>
         </is>
       </c>
       <c r="B23" s="54" t="inlineStr">
@@ -7685,24 +7714,24 @@
       </c>
       <c r="C23" s="54" t="inlineStr">
         <is>
-          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
+          <t>V-02 — متوقعات الكاش القصيرة</t>
         </is>
       </c>
       <c r="D23" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E23" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="54" t="inlineStr">
         <is>
-          <t>FIN-008</t>
+          <t>V-003</t>
         </is>
       </c>
       <c r="B24" s="54" t="inlineStr">
@@ -7712,24 +7741,24 @@
       </c>
       <c r="C24" s="54" t="inlineStr">
         <is>
-          <t>تحقق الإهلاك بعد مرور الزمن</t>
+          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
         </is>
       </c>
       <c r="D24" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E24" s="54" t="inlineStr">
         <is>
-          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="54" t="inlineStr">
         <is>
-          <t>OPS-003</t>
+          <t>V-004</t>
         </is>
       </c>
       <c r="B25" s="54" t="inlineStr">
@@ -7739,24 +7768,24 @@
       </c>
       <c r="C25" s="54" t="inlineStr">
         <is>
-          <t>المصروفات المتكررة المحلية</t>
+          <t>V-04 — عرض التغطية عند قرار السحب</t>
         </is>
       </c>
       <c r="D25" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E25" s="54" t="inlineStr">
         <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="54" t="inlineStr">
         <is>
-          <t>SCOPE-002</t>
+          <t>V-005</t>
         </is>
       </c>
       <c r="B26" s="54" t="inlineStr">
@@ -7766,24 +7795,24 @@
       </c>
       <c r="C26" s="54" t="inlineStr">
         <is>
-          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
+          <t>V-05 — مقارنة فترتين بسيطة</t>
         </is>
       </c>
       <c r="D26" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E26" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="54" t="inlineStr">
         <is>
-          <t>UX-002</t>
+          <t>V-006</t>
         </is>
       </c>
       <c r="B27" s="54" t="inlineStr">
@@ -7793,24 +7822,24 @@
       </c>
       <c r="C27" s="54" t="inlineStr">
         <is>
-          <t>Backlog الموجة الرابعة في عقد الملكية</t>
+          <t>V-06 — جسر ربح إلى كاش رقمي</t>
         </is>
       </c>
       <c r="D27" s="54" t="inlineStr">
         <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
+          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
         </is>
       </c>
       <c r="E27" s="54" t="inlineStr">
         <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
+          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="54" t="inlineStr">
         <is>
-          <t>V-001</t>
+          <t>V-007</t>
         </is>
       </c>
       <c r="B28" s="54" t="inlineStr">
@@ -7820,7 +7849,7 @@
       </c>
       <c r="C28" s="54" t="inlineStr">
         <is>
-          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
+          <t>V-07 — تنبيه انخفاض المواد</t>
         </is>
       </c>
       <c r="D28" s="54" t="inlineStr">
@@ -7837,7 +7866,7 @@
     <row r="29">
       <c r="A29" s="54" t="inlineStr">
         <is>
-          <t>V-002</t>
+          <t>V-008</t>
         </is>
       </c>
       <c r="B29" s="54" t="inlineStr">
@@ -7847,7 +7876,7 @@
       </c>
       <c r="C29" s="54" t="inlineStr">
         <is>
-          <t>V-02 — متوقعات الكاش القصيرة</t>
+          <t>V-08 — مصروف اليوم على الرئيسية</t>
         </is>
       </c>
       <c r="D29" s="54" t="inlineStr">
@@ -7864,7 +7893,7 @@
     <row r="30">
       <c r="A30" s="54" t="inlineStr">
         <is>
-          <t>V-003</t>
+          <t>V-009</t>
         </is>
       </c>
       <c r="B30" s="54" t="inlineStr">
@@ -7874,7 +7903,7 @@
       </c>
       <c r="C30" s="54" t="inlineStr">
         <is>
-          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
+          <t>V-09 — رقم السحب الآمن الموحد</t>
         </is>
       </c>
       <c r="D30" s="54" t="inlineStr">
@@ -7891,7 +7920,7 @@
     <row r="31">
       <c r="A31" s="54" t="inlineStr">
         <is>
-          <t>V-004</t>
+          <t>V-010</t>
         </is>
       </c>
       <c r="B31" s="54" t="inlineStr">
@@ -7901,7 +7930,7 @@
       </c>
       <c r="C31" s="54" t="inlineStr">
         <is>
-          <t>V-04 — عرض التغطية عند قرار السحب</t>
+          <t>V-10 — كثافة صفحة المالية</t>
         </is>
       </c>
       <c r="D31" s="54" t="inlineStr">
@@ -7918,7 +7947,7 @@
     <row r="32">
       <c r="A32" s="54" t="inlineStr">
         <is>
-          <t>V-005</t>
+          <t>V-011</t>
         </is>
       </c>
       <c r="B32" s="54" t="inlineStr">
@@ -7928,7 +7957,7 @@
       </c>
       <c r="C32" s="54" t="inlineStr">
         <is>
-          <t>V-05 — مقارنة فترتين بسيطة</t>
+          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
         </is>
       </c>
       <c r="D32" s="54" t="inlineStr">
@@ -7945,7 +7974,7 @@
     <row r="33">
       <c r="A33" s="54" t="inlineStr">
         <is>
-          <t>V-006</t>
+          <t>V-012</t>
         </is>
       </c>
       <c r="B33" s="54" t="inlineStr">
@@ -7955,7 +7984,7 @@
       </c>
       <c r="C33" s="54" t="inlineStr">
         <is>
-          <t>V-06 — جسر ربح إلى كاش رقمي</t>
+          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
         </is>
       </c>
       <c r="D33" s="54" t="inlineStr">
@@ -7964,168 +7993,6 @@
         </is>
       </c>
       <c r="E33" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="54" t="inlineStr">
-        <is>
-          <t>V-007</t>
-        </is>
-      </c>
-      <c r="B34" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C34" s="54" t="inlineStr">
-        <is>
-          <t>V-07 — تنبيه انخفاض المواد</t>
-        </is>
-      </c>
-      <c r="D34" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E34" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="54" t="inlineStr">
-        <is>
-          <t>V-008</t>
-        </is>
-      </c>
-      <c r="B35" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C35" s="54" t="inlineStr">
-        <is>
-          <t>V-08 — مصروف اليوم على الرئيسية</t>
-        </is>
-      </c>
-      <c r="D35" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E35" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="54" t="inlineStr">
-        <is>
-          <t>V-009</t>
-        </is>
-      </c>
-      <c r="B36" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C36" s="54" t="inlineStr">
-        <is>
-          <t>V-09 — رقم السحب الآمن الموحد</t>
-        </is>
-      </c>
-      <c r="D36" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E36" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="54" t="inlineStr">
-        <is>
-          <t>V-010</t>
-        </is>
-      </c>
-      <c r="B37" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C37" s="54" t="inlineStr">
-        <is>
-          <t>V-10 — كثافة صفحة المالية</t>
-        </is>
-      </c>
-      <c r="D37" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E37" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="54" t="inlineStr">
-        <is>
-          <t>V-011</t>
-        </is>
-      </c>
-      <c r="B38" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C38" s="54" t="inlineStr">
-        <is>
-          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
-        </is>
-      </c>
-      <c r="D38" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E38" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="54" t="inlineStr">
-        <is>
-          <t>V-012</t>
-        </is>
-      </c>
-      <c r="B39" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C39" s="54" t="inlineStr">
-        <is>
-          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
-        </is>
-      </c>
-      <c r="D39" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E39" s="54" t="inlineStr">
         <is>
           <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
@@ -8325,7 +8192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8592,6 +8459,50 @@
       <c r="D14" s="54" t="inlineStr">
         <is>
           <t>https://github.com/Qays7753/Documents/tree/main/reports/2026/2026-09-19/layered-financial-management-audit-001</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PRE-PILOT-SAFETY-A</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>pre-pilot safety package A (G-001/G-002/G-003/G-006)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>OPEN_PR_190_IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-20_pre-pilot-safety-package-a/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PRE-PILOT-SAFETY-B</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>pre-pilot safety package B (G-004/G-005)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>OPEN_PR_191_IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-20_pre-pilot-safety-package-b/report.md</t>
         </is>
       </c>
     </row>
@@ -8750,7 +8661,7 @@
       </c>
       <c r="B7" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C7" s="54" t="inlineStr">
@@ -8782,7 +8693,7 @@
       </c>
       <c r="B8" s="53" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C8" s="53" t="inlineStr">
@@ -8814,7 +8725,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
@@ -8846,7 +8757,7 @@
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
@@ -8878,7 +8789,7 @@
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
@@ -8910,7 +8821,7 @@
       </c>
       <c r="B12" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C12" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): record merged safety packages pending CI
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2560,7 +2560,7 @@
       </c>
       <c r="D29" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="E29" s="54" t="inlineStr">
@@ -2602,7 +2602,7 @@
       <c r="M29" s="54" t="inlineStr"/>
       <c r="N29" s="54" t="inlineStr">
         <is>
-          <t>مراجعة المالك لـPR #190 (الحزمة أ) ثم الدمج والتحقق على main.</t>
+          <t>انتظار نجاح CI على main عند f6879fbc8c15 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
         </is>
       </c>
       <c r="O29" s="54" t="inlineStr"/>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="D31" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="E31" s="54" t="inlineStr">
@@ -2756,7 +2756,7 @@
       <c r="M31" s="54" t="inlineStr"/>
       <c r="N31" s="54" t="inlineStr">
         <is>
-          <t>مراجعة المالك لـPR #190 (الحزمة أ) ثم الدمج والتحقق على main.</t>
+          <t>انتظار نجاح CI على main عند f6879fbc8c15 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
         </is>
       </c>
       <c r="O31" s="54" t="inlineStr"/>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="D32" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="E32" s="54" t="inlineStr">
@@ -2831,7 +2831,7 @@
       <c r="M32" s="54" t="inlineStr"/>
       <c r="N32" s="54" t="inlineStr">
         <is>
-          <t>مراجعة المالك لـPR #190 (الحزمة أ) ثم الدمج والتحقق على main.</t>
+          <t>انتظار نجاح CI على main عند f6879fbc8c15 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
         </is>
       </c>
       <c r="O32" s="54" t="inlineStr"/>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="D33" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="E33" s="54" t="inlineStr">
@@ -2906,7 +2906,7 @@
       <c r="M33" s="54" t="inlineStr"/>
       <c r="N33" s="54" t="inlineStr">
         <is>
-          <t>مراجعة المالك لـPR #191 (الحزمة ب) ثم الدمج والتحقق على main بعد دمج الحزمة أ (PR #190).</t>
+          <t>انتظار نجاح CI على main عند a054139b4340 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
         </is>
       </c>
       <c r="O33" s="54" t="inlineStr"/>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="D34" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="E34" s="54" t="inlineStr">
@@ -2981,7 +2981,7 @@
       <c r="M34" s="54" t="inlineStr"/>
       <c r="N34" s="54" t="inlineStr">
         <is>
-          <t>مراجعة المالك لـPR #191 (الحزمة ب) ثم الدمج والتحقق على main بعد دمج الحزمة أ (PR #190).</t>
+          <t>انتظار نجاح CI على main عند a054139b4340 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
         </is>
       </c>
       <c r="O34" s="54" t="inlineStr"/>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="D35" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="E35" s="54" t="inlineStr">
@@ -3056,7 +3056,7 @@
       <c r="M35" s="54" t="inlineStr"/>
       <c r="N35" s="54" t="inlineStr">
         <is>
-          <t>مراجعة المالك لـPR #190 (الحزمة أ) ثم الدمج والتحقق على main.</t>
+          <t>انتظار نجاح CI على main عند f6879fbc8c15 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
         </is>
       </c>
       <c r="O35" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6184,6 +6184,23 @@
       <c r="C12" t="inlineStr">
         <is>
           <t>WS-163 / PR #191</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>دمج Package A وPackage B؛ تحديث البنود إلى MERGED_UNVERIFIED حتى نجاح CI على main</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PR #190 f6879fbc / PR #191 a054139b</t>
         </is>
       </c>
     </row>
@@ -6276,7 +6293,7 @@
     <row r="7">
       <c r="A7" s="54" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED / IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED / REVIEW_REQUIRED / IN_REVIEW</t>
         </is>
       </c>
       <c r="B7" s="54" t="n">
@@ -6284,7 +6301,7 @@
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
-          <t>يحتاج مراجعة أو قرارًا</t>
+          <t>يحتاج تحقق CI أو مراجعة/قرارًا</t>
         </is>
       </c>
     </row>
@@ -6311,7 +6328,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>3702c90131472c7ebb117dc0d7d67cd96a47cfc6</t>
+          <t>a054139b43400b9909a10ac6c9187f1eebccda6b</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
@@ -6753,7 +6770,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -6771,7 +6788,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>تنفيذ إصلاحات الحزمة أ مع الاختبارات المركزة ثم فتح PR للحزمة أ على الفرع fix/pre-pilot-safety-a-b.</t>
+          <t>الحزمة أ مدموجة؛ انتظار CI النهائي على main ثم إغلاق التحقق.</t>
         </is>
       </c>
     </row>
@@ -6783,7 +6800,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>REVIEW_REQUIRED</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -6801,7 +6818,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>مراجعة المالك لـPR #191 ثم الدمج والتحقق على main بعد دمج الحزمة أ (PR #190).</t>
+          <t>الحزمة ب مدموجة؛ انتظار CI النهائي على main ثم إغلاق التحقق.</t>
         </is>
       </c>
     </row>
@@ -8661,7 +8678,7 @@
       </c>
       <c r="B7" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="C7" s="54" t="inlineStr">
@@ -8693,7 +8710,7 @@
       </c>
       <c r="B8" s="53" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="C8" s="53" t="inlineStr">
@@ -8725,7 +8742,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
@@ -8757,7 +8774,7 @@
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
@@ -8789,7 +8806,7 @@
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
@@ -8821,7 +8838,7 @@
       </c>
       <c r="B12" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>MERGED_UNVERIFIED</t>
         </is>
       </c>
       <c r="C12" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): verify safety packages on main after CI
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2560,7 +2560,7 @@
       </c>
       <c r="D29" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E29" s="54" t="inlineStr">
@@ -2602,7 +2602,7 @@
       <c r="M29" s="54" t="inlineStr"/>
       <c r="N29" s="54" t="inlineStr">
         <is>
-          <t>انتظار نجاح CI على main عند f6879fbc8c15 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
+          <t>لا إجراء تنفيذي إضافي لهذا Finding؛ تبقى بوابة PRE-PILOT محجوبة حتى إغلاق بقية المتطلبات وقرار المالك.</t>
         </is>
       </c>
       <c r="O29" s="54" t="inlineStr"/>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="D31" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E31" s="54" t="inlineStr">
@@ -2756,7 +2756,7 @@
       <c r="M31" s="54" t="inlineStr"/>
       <c r="N31" s="54" t="inlineStr">
         <is>
-          <t>انتظار نجاح CI على main عند f6879fbc8c15 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
+          <t>لا إجراء تنفيذي إضافي لهذا Finding؛ تبقى بوابة PRE-PILOT محجوبة حتى إغلاق بقية المتطلبات وقرار المالك.</t>
         </is>
       </c>
       <c r="O31" s="54" t="inlineStr"/>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="D32" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E32" s="54" t="inlineStr">
@@ -2831,7 +2831,7 @@
       <c r="M32" s="54" t="inlineStr"/>
       <c r="N32" s="54" t="inlineStr">
         <is>
-          <t>انتظار نجاح CI على main عند f6879fbc8c15 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
+          <t>لا إجراء تنفيذي إضافي لهذا Finding؛ تبقى بوابة PRE-PILOT محجوبة حتى إغلاق بقية المتطلبات وقرار المالك.</t>
         </is>
       </c>
       <c r="O32" s="54" t="inlineStr"/>
@@ -2864,7 +2864,7 @@
       </c>
       <c r="D33" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E33" s="54" t="inlineStr">
@@ -2906,7 +2906,7 @@
       <c r="M33" s="54" t="inlineStr"/>
       <c r="N33" s="54" t="inlineStr">
         <is>
-          <t>انتظار نجاح CI على main عند a054139b4340 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
+          <t>لا إجراء تنفيذي إضافي لهذا Finding؛ تبقى بوابة PRE-PILOT محجوبة حتى إغلاق بقية المتطلبات وقرار المالك.</t>
         </is>
       </c>
       <c r="O33" s="54" t="inlineStr"/>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="D34" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E34" s="54" t="inlineStr">
@@ -2981,7 +2981,7 @@
       <c r="M34" s="54" t="inlineStr"/>
       <c r="N34" s="54" t="inlineStr">
         <is>
-          <t>انتظار نجاح CI على main عند a054139b4340 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
+          <t>لا إجراء تنفيذي إضافي لهذا Finding؛ تبقى بوابة PRE-PILOT محجوبة حتى إغلاق بقية المتطلبات وقرار المالك.</t>
         </is>
       </c>
       <c r="O34" s="54" t="inlineStr"/>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="D35" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E35" s="54" t="inlineStr">
@@ -3056,7 +3056,7 @@
       <c r="M35" s="54" t="inlineStr"/>
       <c r="N35" s="54" t="inlineStr">
         <is>
-          <t>انتظار نجاح CI على main عند f6879fbc8c15 ثم تحديث VERIFIED مع verified_on_main_sha.</t>
+          <t>لا إجراء تنفيذي إضافي لهذا Finding؛ تبقى بوابة PRE-PILOT محجوبة حتى إغلاق بقية المتطلبات وقرار المالك.</t>
         </is>
       </c>
       <c r="O35" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6201,6 +6201,23 @@
       <c r="C13" t="inlineStr">
         <is>
           <t>PR #190 f6879fbc / PR #191 a054139b</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>نجاح CI على main وتثبيت G-001..G-006 وWS-162/WS-163 كـVERIFIED؛ PRE-PILOT وPilot ما زالا محجوبين</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>main 0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
         </is>
       </c>
     </row>
@@ -6282,7 +6299,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6293,15 +6310,15 @@
     <row r="7">
       <c r="A7" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED / REVIEW_REQUIRED / IN_REVIEW</t>
+          <t>REVIEW_REQUIRED / IN_REVIEW</t>
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
-          <t>يحتاج تحقق CI أو مراجعة/قرارًا</t>
+          <t>يحتاج مراجعة أو قرارًا</t>
         </is>
       </c>
     </row>
@@ -6328,7 +6345,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>a054139b43400b9909a10ac6c9187f1eebccda6b</t>
+          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
@@ -6770,7 +6787,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -6788,7 +6805,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>الحزمة أ مدموجة؛ انتظار CI النهائي على main ثم إغلاق التحقق.</t>
+          <t>لا إجراء إضافي؛ الحزمة مدموجة ومتحقق منها على main. لا يبدأ Pilot أو المرحلة التالية من هذا السجل.</t>
         </is>
       </c>
     </row>
@@ -6800,7 +6817,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>REVIEW_REQUIRED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -6818,7 +6835,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>الحزمة ب مدموجة؛ انتظار CI النهائي على main ثم إغلاق التحقق.</t>
+          <t>لا إجراء إضافي؛ الحزمة مدموجة ومتحقق منها على main. لا يبدأ Pilot أو المرحلة التالية من هذا السجل.</t>
         </is>
       </c>
     </row>
@@ -6836,7 +6853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6887,22 +6904,22 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="53" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>CTRL-001</t>
         </is>
       </c>
-      <c r="B5" s="53" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>اعتماد Operations Control v2</t>
         </is>
       </c>
-      <c r="C5" s="53" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>e75419504d61a60141c1776a5bfa69ed1faeb529</t>
         </is>
       </c>
-      <c r="D5" s="53" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>docs/operations/control/README.md
 https://github.com/Qays7753/Micro/pull/188
@@ -6912,22 +6929,22 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="54" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>CTRL-002</t>
         </is>
       </c>
-      <c r="B6" s="54" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>مصالحة القدرات والتقارير ومصادر الحقيقة</t>
         </is>
       </c>
-      <c r="C6" s="54" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>e75419504d61a60141c1776a5bfa69ed1faeb529</t>
         </is>
       </c>
-      <c r="D6" s="54" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>docs/operations/control/migration-map.md
 docs/operations/control/evidence/capability-reconciliation.md
@@ -6937,225 +6954,363 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="54" t="inlineStr">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>G-001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>فخ الاستهلاك المزدوج عند التسليم</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>f6879fbc8c152c4b630671b347b737112e065a19</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/gap-register.md
+https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/scenario-results.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>G-002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ذرية تخصيص دفعة المورد للمحفظة</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>f6879fbc8c152c4b630671b347b737112e065a19</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/gap-register.md
+https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/scenario-results.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>G-003</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>حرس القراءة القديمة عند حفظ الطلب</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>f6879fbc8c152c4b630671b347b737112e065a19</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/gap-register.md
+https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/scenario-results.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>G-004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>مطابقة تعطيل القدرات للوعد المرئي</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>a054139b43400b9909a10ac6c9187f1eebccda6b</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/gap-register.md
+https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/scenario-results.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>G-005</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>عزل فشل قراءات صفحة المالية</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>a054139b43400b9909a10ac6c9187f1eebccda6b</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/gap-register.md
+https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/scenario-results.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>G-006</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>توحيد حرس السحب بين مساري مال المالك</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>f6879fbc8c152c4b630671b347b737112e065a19</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/gap-register.md
+https://github.com/Qays7753/Documents/blob/main/reports/2026/2026-09-19/layered-financial-management-audit-001/scenario-results.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>HARD-009</t>
         </is>
       </c>
-      <c r="B7" s="54" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 9</t>
         </is>
       </c>
-      <c r="C7" s="54" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>255974a8cf66674e0a3dba477da9d9400cb28306</t>
         </is>
       </c>
-      <c r="D7" s="54" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="53" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>HARD-010</t>
         </is>
       </c>
-      <c r="B8" s="53" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 10</t>
         </is>
       </c>
-      <c r="C8" s="53" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>dcf60dbed79c09a06a46fcbad07e104277cb17de</t>
         </is>
       </c>
-      <c r="D8" s="53" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>HARD-011</t>
         </is>
       </c>
-      <c r="B9" s="54" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>إثبات إغلاق مجموعة المعالجة 11</t>
         </is>
       </c>
-      <c r="C9" s="54" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>79dac8e726b3cf5e682cb912b90d7c3757636f71</t>
         </is>
       </c>
-      <c r="D9" s="54" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>docs/operations/control/evidence/hardening-main-verification.md
 docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="54" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>HIST-001</t>
         </is>
       </c>
-      <c r="B10" s="54" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>الموجة الأولى: إصلاحات حرجة محددة</t>
         </is>
       </c>
-      <c r="C10" s="54" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>5c54d8a</t>
         </is>
       </c>
-      <c r="D10" s="54" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="54" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>HIST-002</t>
         </is>
       </c>
-      <c r="B11" s="54" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>الموجة الثانية: الأساسات المالية والبيانية</t>
         </is>
       </c>
-      <c r="C11" s="54" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>81d8d253984dee410c7fd6c3e461fcd0e76f327e</t>
         </is>
       </c>
-      <c r="D11" s="54" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-17_wave-2-financial-data-foundations/report.md</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="54" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>HIST-003</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>الموجة الثالثة: العقود والملكية التقنية</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>f8b37062c14aecf85abf5f64e11a191b00eb3c0d</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>docs/operations/current-state.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HIST-004</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>الموجة 4.1: مخطط تجربة المنتج</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>281a2878b61870792f76d651d0d822c7f0a5c0e1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>HIST-005</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>الموجة 4.2: الهيكل والتنقل والتسمية</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>9179ea785d7c35790c422a997fa210aaf7e875a6</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-17_wave-4-2-structure-navigation-naming/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>HIST-006</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>الموجة 4.3: إعادة بناء أسطح المنتج</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>e8a7b5a5f6678a4a93e3ab4c21814764f5895335</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>docs/operations/current-state.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>HIST-007</t>
         </is>
       </c>
-      <c r="B12" s="54" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>الموجة 4.4: الجودة النظامية والقبول المحلي</t>
         </is>
       </c>
-      <c r="C12" s="54" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>87ebcf2ffa74752bf385eff3a10962454b45d33e</t>
         </is>
       </c>
-      <c r="D12" s="54" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-18_wave-4-4-system-quality-final-qa/report.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="54" t="inlineStr">
-        <is>
-          <t>HIST-003</t>
-        </is>
-      </c>
-      <c r="B13" s="54" t="inlineStr">
-        <is>
-          <t>الموجة الثالثة: العقود والملكية التقنية</t>
-        </is>
-      </c>
-      <c r="C13" s="54" t="inlineStr">
-        <is>
-          <t>f8b37062c14aecf85abf5f64e11a191b00eb3c0d</t>
-        </is>
-      </c>
-      <c r="D13" s="54" t="inlineStr">
-        <is>
-          <t>docs/operations/current-state.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="54" t="inlineStr">
-        <is>
-          <t>HIST-004</t>
-        </is>
-      </c>
-      <c r="B14" s="54" t="inlineStr">
-        <is>
-          <t>الموجة 4.1: مخطط تجربة المنتج</t>
-        </is>
-      </c>
-      <c r="C14" s="54" t="inlineStr">
-        <is>
-          <t>281a2878b61870792f76d651d0d822c7f0a5c0e1</t>
-        </is>
-      </c>
-      <c r="D14" s="54" t="inlineStr">
-        <is>
-          <t>reports/agent-report/2026-09-17_wave-4-1-product-ux-blueprint/report.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="54" t="inlineStr">
-        <is>
-          <t>HIST-005</t>
-        </is>
-      </c>
-      <c r="B15" s="54" t="inlineStr">
-        <is>
-          <t>الموجة 4.2: الهيكل والتنقل والتسمية</t>
-        </is>
-      </c>
-      <c r="C15" s="54" t="inlineStr">
-        <is>
-          <t>9179ea785d7c35790c422a997fa210aaf7e875a6</t>
-        </is>
-      </c>
-      <c r="D15" s="54" t="inlineStr">
-        <is>
-          <t>reports/agent-report/2026-09-17_wave-4-2-structure-navigation-naming/report.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="54" t="inlineStr">
-        <is>
-          <t>HIST-006</t>
-        </is>
-      </c>
-      <c r="B16" s="54" t="inlineStr">
-        <is>
-          <t>الموجة 4.3: إعادة بناء أسطح المنتج</t>
-        </is>
-      </c>
-      <c r="C16" s="54" t="inlineStr">
-        <is>
-          <t>e8a7b5a5f6678a4a93e3ab4c21814764f5895335</t>
-        </is>
-      </c>
-      <c r="D16" s="54" t="inlineStr">
-        <is>
-          <t>docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
@@ -7173,7 +7328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7233,785 +7388,29 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="53" t="inlineStr">
-        <is>
-          <t>DEVICE-001</t>
-        </is>
-      </c>
-      <c r="B5" s="53" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="C5" s="53" t="inlineStr">
-        <is>
-          <t>QA على أجهزة فعلية وWebKit وPWA</t>
-        </is>
-      </c>
-      <c r="D5" s="53" t="inlineStr">
-        <is>
-          <t>الاعتماديات أو البيئة المطلوبة لم تكتمل: UX-001, REL-001</t>
-        </is>
-      </c>
-      <c r="E5" s="53" t="inlineStr">
-        <is>
-          <t>أغلق سبب الحجب قبل بدء العمل؛ الاعتماديات الحالية: UX-001, REL-001.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="54" t="inlineStr">
-        <is>
-          <t>LEGAL-001</t>
-        </is>
-      </c>
-      <c r="B6" s="54" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="C6" s="54" t="inlineStr">
-        <is>
-          <t>مراجعة أردنية مالية وقانونية</t>
-        </is>
-      </c>
-      <c r="D6" s="54" t="inlineStr">
-        <is>
-          <t>الاعتماديات أو البيئة المطلوبة لم تكتمل: FIN-007</t>
-        </is>
-      </c>
-      <c r="E6" s="54" t="inlineStr">
-        <is>
-          <t>أغلق سبب الحجب قبل بدء العمل؛ الاعتماديات الحالية: FIN-007.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="54" t="inlineStr">
-        <is>
-          <t>PILOT-001</t>
-        </is>
-      </c>
-      <c r="B7" s="54" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="C7" s="54" t="inlineStr">
-        <is>
-          <t>قرار بدء Pilot</t>
-        </is>
-      </c>
-      <c r="D7" s="54" t="inlineStr">
-        <is>
-          <t>المراحل 0–9 وبوابات المنتج والجهاز والقانون وUAT والتدقيق لم تثبت كلها VERIFIED على main.</t>
-        </is>
-      </c>
-      <c r="E7" s="54" t="inlineStr">
-        <is>
-          <t>لا يصبح Ready ولا يبدأ قبل VERIFIED لكل required_items في PRE-PILOT، ثم قرار المالك؛ لا يبدأ تلقائيًا بنجاح CI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="54" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>GOV-001</t>
         </is>
       </c>
-      <c r="B8" s="54" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>REVIEW_REQUIRED</t>
         </is>
       </c>
-      <c r="C8" s="54" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>مصالحة G10-A مع تعارض عقد C1</t>
         </is>
       </c>
-      <c r="D8" s="54" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>هل يوحّد G10-A عقد C1 أم يبقى مؤجلًا؟</t>
         </is>
       </c>
-      <c r="E8" s="54" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>يُراجع التعارض مع المالك ثم يثبت القرار كعقد أو تأجيل؛ لا يبدأ تنفيذًا صامتًا.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
-        <is>
-          <t>SCOPE-001</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>بوابة POS وCRM وWhatsApp والمزامنة وAuth والصلاحيات وCloud</t>
-        </is>
-      </c>
-      <c r="D9" s="54" t="inlineStr">
-        <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
-        </is>
-      </c>
-      <c r="E9" s="54" t="inlineStr">
-        <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="54" t="inlineStr">
-        <is>
-          <t>UX-001</t>
-        </is>
-      </c>
-      <c r="B10" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C10" s="54" t="inlineStr">
-        <is>
-          <t>إعادة تصميم UI وUX جذرية</t>
-        </is>
-      </c>
-      <c r="D10" s="54" t="inlineStr">
-        <is>
-          <t>تنفيذ مؤجل حتى استقرار الوظائف واعتماد الاتجاه وBenchmark، لكنه متطلب Gate قبل Pilot؛ لا يتجاوز بوابة الإصدار.</t>
-        </is>
-      </c>
-      <c r="E10" s="54" t="inlineStr">
-        <is>
-          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="54" t="inlineStr">
-        <is>
-          <t>BE-001</t>
-        </is>
-      </c>
-      <c r="B11" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C11" s="54" t="inlineStr">
-        <is>
-          <t>مصاريف متكررة محلية</t>
-        </is>
-      </c>
-      <c r="D11" s="54" t="inlineStr">
-        <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
-        </is>
-      </c>
-      <c r="E11" s="54" t="inlineStr">
-        <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'OPS-003') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="54" t="inlineStr">
-        <is>
-          <t>BE-002</t>
-        </is>
-      </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
-        <is>
-          <t>ميزانيات وأهداف بسيطة</t>
-        </is>
-      </c>
-      <c r="D12" s="54" t="inlineStr">
-        <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
-        </is>
-      </c>
-      <c r="E12" s="54" t="inlineStr">
-        <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-002') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="54" t="inlineStr">
-        <is>
-          <t>BE-003</t>
-        </is>
-      </c>
-      <c r="B13" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C13" s="54" t="inlineStr">
-        <is>
-          <t>ربحية المنتج عبر الفترات بمعرف كتالوج ثابت</t>
-        </is>
-      </c>
-      <c r="D13" s="54" t="inlineStr">
-        <is>
-          <t>DUPLICATE_HISTORICAL؛ محفوظ للتتبع ولا يتجاوز البوابة ولا يفتح تنفيذًا موازيًا.</t>
-        </is>
-      </c>
-      <c r="E13" s="54" t="inlineStr">
-        <is>
-          <t>لا تنشئ Claim مستقلًا؛ تابع ('DUPLICATE_HISTORICAL', 'FIN-006') بوصفه المالك الحي للقدرة، وأبقِ هذا السجل مرجعًا تاريخيًا.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="54" t="inlineStr">
-        <is>
-          <t>BE-004</t>
-        </is>
-      </c>
-      <c r="B14" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C14" s="54" t="inlineStr">
-        <is>
-          <t>إغلاق فترة رسمي</t>
-        </is>
-      </c>
-      <c r="D14" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
-        </is>
-      </c>
-      <c r="E14" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="54" t="inlineStr">
-        <is>
-          <t>BE-005</t>
-        </is>
-      </c>
-      <c r="B15" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C15" s="54" t="inlineStr">
-        <is>
-          <t>تقادم الديون بشرائح 30/60/90</t>
-        </is>
-      </c>
-      <c r="D15" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ لا يبدأ قبل دليل Pilot وقرار مالك، ولا يمثل متطلبًا مستقلًا قبل Pilot.</t>
-        </is>
-      </c>
-      <c r="E15" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="54" t="inlineStr">
-        <is>
-          <t>FIN-002</t>
-        </is>
-      </c>
-      <c r="B16" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C16" s="54" t="inlineStr">
-        <is>
-          <t>ميزانيات وأهداف بسيطة</t>
-        </is>
-      </c>
-      <c r="D16" s="54" t="inlineStr">
-        <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ الميزانيات والأهداف المبسطة مطلوبة ضمن المرحلة 3.</t>
-        </is>
-      </c>
-      <c r="E16" s="54" t="inlineStr">
-        <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ أبسط ميزانية/هدف مع اختبارات عدم خلط الخطة بالحدث المالي.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="54" t="inlineStr">
-        <is>
-          <t>FIN-006</t>
-        </is>
-      </c>
-      <c r="B17" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C17" s="54" t="inlineStr">
-        <is>
-          <t>ربحية المنتج بمعرف كتالوج ثابت</t>
-        </is>
-      </c>
-      <c r="D17" s="54" t="inlineStr">
-        <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ ربحية المنتجات/الخدمات بمعرف ثابت مطلوبة ضمن المرحلة 3.</t>
-        </is>
-      </c>
-      <c r="E17" s="54" t="inlineStr">
-        <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ ربحية بمعرف كتالوج ثابت واختبارات Snapshot/الفترات.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="54" t="inlineStr">
-        <is>
-          <t>FIN-008</t>
-        </is>
-      </c>
-      <c r="B18" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C18" s="54" t="inlineStr">
-        <is>
-          <t>تحقق الإهلاك بعد مرور الزمن</t>
-        </is>
-      </c>
-      <c r="D18" s="54" t="inlineStr">
-        <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ اختبار الإهلاك يستخدم Clock قابلًا للحقن ولا ينتظر شهرًا حقيقيًا.</t>
-        </is>
-      </c>
-      <c r="E18" s="54" t="inlineStr">
-        <is>
-          <t>صمّم/نفّذ اختبارًا باستخدام Clock قابل للحقن مع وقتين اصطناعيين على الأقل، ثم افتح Claim؛ لا تستخدم انتظارًا زمنيًا حقيقيًا.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="54" t="inlineStr">
-        <is>
-          <t>OPS-003</t>
-        </is>
-      </c>
-      <c r="B19" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C19" s="54" t="inlineStr">
-        <is>
-          <t>المصروفات المتكررة المحلية</t>
-        </is>
-      </c>
-      <c r="D19" s="54" t="inlineStr">
-        <is>
-          <t>تنفيذ مؤجل حتى اعتماد/إكمال الاعتماديات، لكنه متطلب Gate قبل Pilot؛ التذكير لا ينشئ حدثًا ماليًا تلقائيًا ويحتاج تأكيد المستخدم.</t>
-        </is>
-      </c>
-      <c r="E19" s="54" t="inlineStr">
-        <is>
-          <t>أكمل الاعتماديات، ثم افتح Claim لتنفيذ تذكير متكرر يحتاج تأكيد المستخدم؛ لا يكتب حدثًا ماليًا تلقائيًا.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="54" t="inlineStr">
-        <is>
-          <t>SCOPE-002</t>
-        </is>
-      </c>
-      <c r="B20" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C20" s="54" t="inlineStr">
-        <is>
-          <t>الموارد وقدرة المواد والتوسع التشغيلي</t>
-        </is>
-      </c>
-      <c r="D20" s="54" t="inlineStr">
-        <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
-        </is>
-      </c>
-      <c r="E20" s="54" t="inlineStr">
-        <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="54" t="inlineStr">
-        <is>
-          <t>UX-002</t>
-        </is>
-      </c>
-      <c r="B21" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C21" s="54" t="inlineStr">
-        <is>
-          <t>Backlog الموجة الرابعة في عقد الملكية</t>
-        </is>
-      </c>
-      <c r="D21" s="54" t="inlineStr">
-        <is>
-          <t>OUT_OF_SCOPE؛ لا يدخل PRE-PILOT ولا يتحول إلى Feature قبل نطاق وعقد وقرار مستقل.</t>
-        </is>
-      </c>
-      <c r="E21" s="54" t="inlineStr">
-        <is>
-          <t>لا تبدأ؛ أعد الفتح فقط بعد دليل، عقد، وقرار مالك مستقل خارج نطاق Pilot الحالي.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="54" t="inlineStr">
-        <is>
-          <t>V-001</t>
-        </is>
-      </c>
-      <c r="B22" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C22" s="54" t="inlineStr">
-        <is>
-          <t>V-01 — التقاط تواريخ استحقاق المشتريات</t>
-        </is>
-      </c>
-      <c r="D22" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E22" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="54" t="inlineStr">
-        <is>
-          <t>V-002</t>
-        </is>
-      </c>
-      <c r="B23" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C23" s="54" t="inlineStr">
-        <is>
-          <t>V-02 — متوقعات الكاش القصيرة</t>
-        </is>
-      </c>
-      <c r="D23" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E23" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="54" t="inlineStr">
-        <is>
-          <t>V-003</t>
-        </is>
-      </c>
-      <c r="B24" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C24" s="54" t="inlineStr">
-        <is>
-          <t>V-03 — أجندة القادم المجمعة بالتاريخ</t>
-        </is>
-      </c>
-      <c r="D24" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E24" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="54" t="inlineStr">
-        <is>
-          <t>V-004</t>
-        </is>
-      </c>
-      <c r="B25" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C25" s="54" t="inlineStr">
-        <is>
-          <t>V-04 — عرض التغطية عند قرار السحب</t>
-        </is>
-      </c>
-      <c r="D25" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E25" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="54" t="inlineStr">
-        <is>
-          <t>V-005</t>
-        </is>
-      </c>
-      <c r="B26" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C26" s="54" t="inlineStr">
-        <is>
-          <t>V-05 — مقارنة فترتين بسيطة</t>
-        </is>
-      </c>
-      <c r="D26" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E26" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="54" t="inlineStr">
-        <is>
-          <t>V-006</t>
-        </is>
-      </c>
-      <c r="B27" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C27" s="54" t="inlineStr">
-        <is>
-          <t>V-06 — جسر ربح إلى كاش رقمي</t>
-        </is>
-      </c>
-      <c r="D27" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E27" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="54" t="inlineStr">
-        <is>
-          <t>V-007</t>
-        </is>
-      </c>
-      <c r="B28" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C28" s="54" t="inlineStr">
-        <is>
-          <t>V-07 — تنبيه انخفاض المواد</t>
-        </is>
-      </c>
-      <c r="D28" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E28" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="54" t="inlineStr">
-        <is>
-          <t>V-008</t>
-        </is>
-      </c>
-      <c r="B29" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C29" s="54" t="inlineStr">
-        <is>
-          <t>V-08 — مصروف اليوم على الرئيسية</t>
-        </is>
-      </c>
-      <c r="D29" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E29" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="54" t="inlineStr">
-        <is>
-          <t>V-009</t>
-        </is>
-      </c>
-      <c r="B30" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C30" s="54" t="inlineStr">
-        <is>
-          <t>V-09 — رقم السحب الآمن الموحد</t>
-        </is>
-      </c>
-      <c r="D30" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E30" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="54" t="inlineStr">
-        <is>
-          <t>V-010</t>
-        </is>
-      </c>
-      <c r="B31" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C31" s="54" t="inlineStr">
-        <is>
-          <t>V-10 — كثافة صفحة المالية</t>
-        </is>
-      </c>
-      <c r="D31" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E31" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="54" t="inlineStr">
-        <is>
-          <t>V-011</t>
-        </is>
-      </c>
-      <c r="B32" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C32" s="54" t="inlineStr">
-        <is>
-          <t>V-11 — فهم نموذج التوزيع الصريح للكاش</t>
-        </is>
-      </c>
-      <c r="D32" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E32" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="54" t="inlineStr">
-        <is>
-          <t>V-012</t>
-        </is>
-      </c>
-      <c r="B33" s="54" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="C33" s="54" t="inlineStr">
-        <is>
-          <t>V-12 — تسجيل الإهلاك بعد شهر استخدام</t>
-        </is>
-      </c>
-      <c r="D33" s="54" t="inlineStr">
-        <is>
-          <t>PILOT_EVIDENCE_REQUIRED؛ فرضية تحقق أثناء Pilot وليست Feature قبل دليل وقرار.</t>
-        </is>
-      </c>
-      <c r="E33" s="54" t="inlineStr">
-        <is>
-          <t>أضف السؤال إلى بروتوكول Pilot، ثم سجّل النتيجة والقرار قبل فتح أي تنفيذ.</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8077,7 @@
       </c>
       <c r="B7" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C7" s="54" t="inlineStr">
@@ -8710,7 +8109,7 @@
       </c>
       <c r="B8" s="53" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C8" s="53" t="inlineStr">
@@ -8742,7 +8141,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
@@ -8774,7 +8173,7 @@
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
@@ -8806,7 +8205,7 @@
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
@@ -8838,7 +8237,7 @@
       </c>
       <c r="B12" s="54" t="inlineStr">
         <is>
-          <t>MERGED_UNVERIFIED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C12" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): claim WS-164 for Stage 2 Wave 1 (OPS-001)
OPS-001 moves READY -> CLAIMED -> IN_PROGRESS per the Operations Control v2 cycle.
Base SHA 7189df66 (origin/main, CI green). Branch stage-2/ops-001-due-dates.
Scope: due dates + basic aging read/classification layer only; no schema/export
change (35/27); no financial Writer change; no refactoring.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1533,7 +1533,7 @@
       </c>
       <c r="D16" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E16" s="54" t="inlineStr">
@@ -1579,7 +1579,7 @@
       <c r="M16" s="54" t="inlineStr"/>
       <c r="N16" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تنفيذ الموجة 1 قيد التنفيذ داخل WS-164 على فرع stage-2/ops-001-due-dates؛ بعد اكتمال الاختبارات وPR تنتقل إلى IN_REVIEW.</t>
         </is>
       </c>
       <c r="O16" s="54" t="inlineStr"/>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="Q16" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6218,6 +6218,23 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>main 0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>فتح Claim الموجة 1 من Stage 2 (WS-164) — OPS-001 إلى IN_PROGRESS على فرع stage-2/ops-001-due-dates من خط أساس 7189df66</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>WS-164 / stage-2/ops-001-due-dates</t>
         </is>
       </c>
     </row>
@@ -6235,7 +6252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6323,66 +6340,81 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="53" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>قيد التنفيذ الآن في Claim نشط</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="53" t="inlineStr">
         <is>
           <t>BLOCKED / DEFERRED</t>
         </is>
       </c>
-      <c r="B8" s="53" t="n">
+      <c r="B9" s="53" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="53" t="inlineStr">
+      <c r="C9" s="53" t="inlineStr">
         <is>
           <t>بوابة أو دليل مؤجل</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
-        <is>
-          <t>main SHA</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
-        </is>
-      </c>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>PRE-PILOT</t>
+          <t>main SHA</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
+          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
+          <t>PRE-PILOT</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
           <t>السياق الدائم</t>
         </is>
       </c>
-      <c r="B11" s="54" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>docs/operations/control/context.md</t>
         </is>
       </c>
-      <c r="C11" s="54" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>الخطة والأدوار ومصادر السلطة</t>
         </is>
@@ -6623,7 +6655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6836,6 +6868,33 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>لا إجراء إضافي؛ الحزمة مدموجة ومتحقق منها على main. لا يبدأ Pilot أو المرحلة التالية من هذا السجل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WS-164</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CLAIMED</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>stage-2/ops-001-due-dates</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OPS-001</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>تنفيذ طبقة قراءة/تصنيف التقادم الأساسي مع اختبارات مركزة ثم PR للموجة 1.</t>
         </is>
       </c>
     </row>
@@ -8269,7 +8328,7 @@
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): Stage 2 Wave 1 IN_REVIEW — PR #196, execution report, QA record, current-state §48
OPS-001 and WS-164 move to IN_REVIEW (actor pr:196). Report + test-results
under reports/agent-report/2026-09-20_stage-2-ops-001-due-dates/. QA record
under docs/quality/stage-2-ops-001-qa-2026-09-20.md. Reports index + README
runs row. Views/Excel/meta regenerated and validated.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1533,7 +1533,7 @@
       </c>
       <c r="D16" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E16" s="54" t="inlineStr">
@@ -1579,7 +1579,7 @@
       <c r="M16" s="54" t="inlineStr"/>
       <c r="N16" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ الموجة 1 قيد التنفيذ داخل WS-164 على فرع stage-2/ops-001-due-dates؛ بعد اكتمال الاختبارات وPR تنتقل إلى IN_REVIEW.</t>
+          <t>PR #196 مفتوح للموجة 1؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
         </is>
       </c>
       <c r="O16" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6235,6 +6235,23 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>WS-164 / stage-2/ops-001-due-dates</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>اكتمال الموجة 1 من Stage 2 (OPS-001) وفتح PR #196 — OPS-001 وWS-164 إلى IN_REVIEW مع Views/Excel محدثة</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>WS-164 / PR #196</t>
         </is>
       </c>
     </row>
@@ -6252,7 +6269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6331,7 +6348,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6340,81 +6357,66 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>قيد التنفيذ الآن في Claim نشط</t>
+      <c r="A8" s="53" t="inlineStr">
+        <is>
+          <t>BLOCKED / DEFERRED</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>بوابة أو دليل مؤجل</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="53" t="inlineStr">
-        <is>
-          <t>BLOCKED / DEFERRED</t>
-        </is>
-      </c>
-      <c r="B9" s="53" t="n">
-        <v>28</v>
-      </c>
-      <c r="C9" s="53" t="inlineStr">
-        <is>
-          <t>بوابة أو دليل مؤجل</t>
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>main SHA</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>main SHA</t>
+          <t>PRE-PILOT</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>يجب تثبيته قبل أي تنفيذ</t>
+          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>PRE-PILOT</t>
+          <t>السياق الدائم</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>docs/operations/control/context.md</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
-        <is>
-          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="54" t="inlineStr">
-        <is>
-          <t>السياق الدائم</t>
-        </is>
-      </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>docs/operations/control/context.md</t>
-        </is>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>الخطة والأدوار ومصادر السلطة</t>
         </is>
@@ -6879,7 +6881,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -6887,6 +6889,9 @@
           <t>stage-2/ops-001-due-dates</t>
         </is>
       </c>
+      <c r="D10" t="n">
+        <v>196</v>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>OPS-001</t>
@@ -6894,7 +6899,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>تنفيذ طبقة قراءة/تصنيف التقادم الأساسي مع اختبارات مركزة ثم PR للموجة 1.</t>
+          <t>انتظار CI على PR #196 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
         </is>
       </c>
     </row>
@@ -7667,7 +7672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7978,6 +7983,28 @@
       <c r="D16" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-20_pre-pilot-safety-package-b/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>STAGE-2-OPS-001</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>stage 2 wave 1 (OPS-001 due dates and basic aging)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>OPEN_PR_196_IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-20_stage-2-ops-001-due-dates/report.md</t>
         </is>
       </c>
     </row>
@@ -8328,7 +8355,7 @@
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): close Wave 1 verified on main + claim WS-165 for Wave 2 (OPS-005/OPS-006)
OPS-001 and WS-164 -> VERIFIED: PR #196 merged at bf24bdb (merge commit),
CI green on that exact main SHA (checks + Cloudflare Pages), evidence
reachable from main. OPS-005/OPS-006 -> IN_PROGRESS inside new claim WS-165
(branch stage-2/ops-005-006-upcoming-aging, base bf24bdb). Single
closure+claim commit avoids the transient active-overlap error (owner
#192/#193 mechanism). Views/Excel/meta regenerated and validated.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1533,7 +1533,7 @@
       </c>
       <c r="D16" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E16" s="54" t="inlineStr">
@@ -1579,7 +1579,7 @@
       <c r="M16" s="54" t="inlineStr"/>
       <c r="N16" s="54" t="inlineStr">
         <is>
-          <t>PR #196 مفتوح للموجة 1؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
+          <t>لا إجراء؛ OPS-001 منفذ ومتحقق على main عند bf24bdbfe653e9f7cf8f14f93af9fe6019bd1cb6 (CI أخضر على SHA نفسه). الموجة 2 (OPS-005+OPS-006) تفتح Claim مستقلًا WS-165.</t>
         </is>
       </c>
       <c r="O16" s="54" t="inlineStr"/>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D17" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E17" s="54" t="inlineStr">
@@ -1658,7 +1658,7 @@
       <c r="M17" s="54" t="inlineStr"/>
       <c r="N17" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>تنفيذ الموجة 2 قيد التنفيذ داخل WS-165 على فرع stage-2/ops-005-006-upcoming-aging؛ بعد اكتمال الاختبارات وPR تنتقل إلى IN_REVIEW.</t>
         </is>
       </c>
       <c r="O17" s="54" t="inlineStr"/>
@@ -1669,7 +1669,7 @@
       </c>
       <c r="Q17" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="D24" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E24" s="54" t="inlineStr">
@@ -2211,7 +2211,7 @@
       <c r="M24" s="54" t="inlineStr"/>
       <c r="N24" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>تنفيذ الموجة 2 قيد التنفيذ داخل WS-165 على فرع stage-2/ops-005-006-upcoming-aging؛ بعد اكتمال الاختبارات وPR تنتقل إلى IN_REVIEW.</t>
         </is>
       </c>
       <c r="O24" s="54" t="inlineStr"/>
@@ -2222,7 +2222,7 @@
       </c>
       <c r="Q24" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6252,6 +6252,23 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>WS-164 / PR #196</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>إغلاق الموجة 1 كـVERIFIED على main (bf24bdb) وفتح Claim الموجة 2 WS-165 — OPS-005/OPS-006 إلى IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>WS-164→VERIFIED / WS-165 CLAIMED</t>
         </is>
       </c>
     </row>
@@ -6269,7 +6286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6333,7 +6350,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6348,75 +6365,90 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>يحتاج مراجعة أو قرارًا</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="54" t="inlineStr">
-        <is>
-          <t>يحتاج مراجعة أو قرارًا</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="53" t="inlineStr">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>قيد التنفيذ الآن في Claim نشط</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="53" t="inlineStr">
         <is>
           <t>BLOCKED / DEFERRED</t>
         </is>
       </c>
-      <c r="B8" s="53" t="n">
+      <c r="B9" s="53" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="53" t="inlineStr">
+      <c r="C9" s="53" t="inlineStr">
         <is>
           <t>بوابة أو دليل مؤجل</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
-        <is>
-          <t>main SHA</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
-        </is>
-      </c>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>PRE-PILOT</t>
+          <t>main SHA</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
+          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
+          <t>PRE-PILOT</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
           <t>السياق الدائم</t>
         </is>
       </c>
-      <c r="B11" s="54" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>docs/operations/control/context.md</t>
         </is>
       </c>
-      <c r="C11" s="54" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>الخطة والأدوار ومصادر السلطة</t>
         </is>
@@ -6657,7 +6689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6881,7 +6913,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -6899,7 +6931,34 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>انتظار CI على PR #196 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
+          <t>لا إجراء إضافي؛ الموجة 1 مدموجة ومتحققة على main. الموجة 2 في WS-165 من رأس main المتحقق نفسه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WS-165</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CLAIMED</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>stage-2/ops-005-006-upcoming-aging</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OPS-005, OPS-006</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>تنفيذ قارئ القادم/المتأخر الموحد (قراءة فقط، فشل معزول لكل كتلة) وسطح عرضه ثم اختبارات مركزة وPR.</t>
         </is>
       </c>
     </row>
@@ -6917,7 +6976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7375,6 +7434,30 @@
       <c r="D22" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-18_wave-4-4-system-quality-final-qa/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>OPS-001</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>المواعيد والاستحقاقات وتقادم الذمم الأساسي</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>bf24bdbfe653e9f7cf8f14f93af9fe6019bd1cb6</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Micro/pull/196
+reports/agent-report/2026-09-20_stage-2-ops-001-due-dates/report.md
+https://github.com/Qays7753/Micro/commit/bf24bdbfe653e9f7cf8f14f93af9fe6019bd1cb6</t>
         </is>
       </c>
     </row>
@@ -8355,7 +8438,7 @@
       </c>
       <c r="B13" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C13" s="54" t="inlineStr">
@@ -8483,7 +8566,7 @@
       </c>
       <c r="B17" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="C17" s="54" t="inlineStr">
@@ -8515,7 +8598,7 @@
       </c>
       <c r="B18" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="C18" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): Stage 2 Wave 2 IN_REVIEW — PR #197, execution report, QA record, current-state §49
OPS-005/OPS-006 and WS-165 move to IN_REVIEW (actor pr:197). Report +
test-results under reports/agent-report/2026-09-20_stage-2-ops-005-006-upcoming-aging/.
QA record under docs/quality/stage-2-ops-005-006-qa-2026-09-20.md. Reports
index + README runs row. Views/Excel/meta regenerated and validated.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D17" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E17" s="54" t="inlineStr">
@@ -1658,7 +1658,7 @@
       <c r="M17" s="54" t="inlineStr"/>
       <c r="N17" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ الموجة 2 قيد التنفيذ داخل WS-165 على فرع stage-2/ops-005-006-upcoming-aging؛ بعد اكتمال الاختبارات وPR تنتقل إلى IN_REVIEW.</t>
+          <t>PR #197 مفتوح للموجة 2؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
         </is>
       </c>
       <c r="O17" s="54" t="inlineStr"/>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="D24" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E24" s="54" t="inlineStr">
@@ -2211,7 +2211,7 @@
       <c r="M24" s="54" t="inlineStr"/>
       <c r="N24" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ الموجة 2 قيد التنفيذ داخل WS-165 على فرع stage-2/ops-005-006-upcoming-aging؛ بعد اكتمال الاختبارات وPR تنتقل إلى IN_REVIEW.</t>
+          <t>PR #197 مفتوح للموجة 2؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
         </is>
       </c>
       <c r="O24" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6269,6 +6269,23 @@
       <c r="C17" t="inlineStr">
         <is>
           <t>WS-164→VERIFIED / WS-165 CLAIMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>اكتمال الموجة 2 من Stage 2 (OPS-005+OPS-006) وفتح PR #197 — البندان وWS-165 إلى IN_REVIEW مع Views/Excel محدثة</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>WS-165 / PR #197</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6365,7 +6382,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6374,81 +6391,66 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>قيد التنفيذ الآن في Claim نشط</t>
+      <c r="A8" s="53" t="inlineStr">
+        <is>
+          <t>BLOCKED / DEFERRED</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>بوابة أو دليل مؤجل</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="53" t="inlineStr">
-        <is>
-          <t>BLOCKED / DEFERRED</t>
-        </is>
-      </c>
-      <c r="B9" s="53" t="n">
-        <v>28</v>
-      </c>
-      <c r="C9" s="53" t="inlineStr">
-        <is>
-          <t>بوابة أو دليل مؤجل</t>
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>main SHA</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>main SHA</t>
+          <t>PRE-PILOT</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>يجب تثبيته قبل أي تنفيذ</t>
+          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>PRE-PILOT</t>
+          <t>السياق الدائم</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>docs/operations/control/context.md</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
-        <is>
-          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="54" t="inlineStr">
-        <is>
-          <t>السياق الدائم</t>
-        </is>
-      </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>docs/operations/control/context.md</t>
-        </is>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>الخطة والأدوار ومصادر السلطة</t>
         </is>
@@ -6943,7 +6945,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -6951,6 +6953,9 @@
           <t>stage-2/ops-005-006-upcoming-aging</t>
         </is>
       </c>
+      <c r="D11" t="n">
+        <v>197</v>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>OPS-005, OPS-006</t>
@@ -6958,7 +6963,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>تنفيذ قارئ القادم/المتأخر الموحد (قراءة فقط، فشل معزول لكل كتلة) وسطح عرضه ثم اختبارات مركزة وPR.</t>
+          <t>انتظار CI على PR #197 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
         </is>
       </c>
     </row>
@@ -7755,7 +7760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8088,6 +8093,28 @@
       <c r="D17" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-20_stage-2-ops-001-due-dates/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>STAGE-2-OPS-005-006</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>stage 2 wave 2 (OPS-005 unified upcoming/overdue surface + OPS-006 simple debt aging)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>OPEN_PR_197_IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-20_stage-2-ops-005-006-upcoming-aging/report.md</t>
         </is>
       </c>
     </row>
@@ -8566,7 +8593,7 @@
       </c>
       <c r="B17" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C17" s="54" t="inlineStr">
@@ -8598,7 +8625,7 @@
       </c>
       <c r="B18" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C18" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): close Wave 2 verified on main + claim WS-166 for Wave 3 (OPS-004)
OPS-005/OPS-006 and WS-165 -> VERIFIED: PR #197 merged at 1836855 (merge
commit), CI green on that exact main SHA, evidence reachable from main.
OPS-004 -> IN_PROGRESS inside new claim WS-166 (branch
stage-2/ops-004-planned-cost, base 1836855). Single closure+claim commit
avoids the transient active-overlap error. Views/Excel/meta regenerated
and validated.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1612,7 +1612,7 @@
       </c>
       <c r="D17" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E17" s="54" t="inlineStr">
@@ -1658,7 +1658,7 @@
       <c r="M17" s="54" t="inlineStr"/>
       <c r="N17" s="54" t="inlineStr">
         <is>
-          <t>PR #197 مفتوح للموجة 2؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
+          <t>لا إجراء؛ OPS-005 منفذ ومتحقق على main عند 18368558b6df0dfbc1b1910e961d1504e9e460fb (CI أخضر على SHA نفسه).</t>
         </is>
       </c>
       <c r="O17" s="54" t="inlineStr"/>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="D23" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E23" s="54" t="inlineStr">
@@ -2132,7 +2132,7 @@
       <c r="M23" s="54" t="inlineStr"/>
       <c r="N23" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>تنفيذ الموجة 3 قيد التنفيذ داخل WS-166 على فرع stage-2/ops-004-planned-cost؛ بعد اكتمال الاختبارات وPR تنتقل إلى IN_REVIEW.</t>
         </is>
       </c>
       <c r="O23" s="54" t="inlineStr"/>
@@ -2143,7 +2143,7 @@
       </c>
       <c r="Q23" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
     </row>
@@ -2165,7 +2165,7 @@
       </c>
       <c r="D24" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E24" s="54" t="inlineStr">
@@ -2211,7 +2211,7 @@
       <c r="M24" s="54" t="inlineStr"/>
       <c r="N24" s="54" t="inlineStr">
         <is>
-          <t>PR #197 مفتوح للموجة 2؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
+          <t>لا إجراء؛ OPS-006 منفذ ومتحقق على main عند 18368558b6df0dfbc1b1910e961d1504e9e460fb (CI أخضر على SHA نفسه).</t>
         </is>
       </c>
       <c r="O24" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6286,6 +6286,23 @@
       <c r="C18" t="inlineStr">
         <is>
           <t>WS-165 / PR #197</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>إغلاق الموجة 2 كـVERIFIED على main (1836855) وفتح Claim الموجة 3 WS-166 — OPS-004 إلى IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>WS-165→VERIFIED / WS-166 CLAIMED</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6367,7 +6384,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6382,7 +6399,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6391,66 +6408,81 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="53" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>قيد التنفيذ الآن في Claim نشط</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="53" t="inlineStr">
         <is>
           <t>BLOCKED / DEFERRED</t>
         </is>
       </c>
-      <c r="B8" s="53" t="n">
+      <c r="B9" s="53" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="53" t="inlineStr">
+      <c r="C9" s="53" t="inlineStr">
         <is>
           <t>بوابة أو دليل مؤجل</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="54" t="inlineStr">
-        <is>
-          <t>main SHA</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
-        </is>
-      </c>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>PRE-PILOT</t>
+          <t>main SHA</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
+          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
+          <t>PRE-PILOT</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="54" t="inlineStr">
+        <is>
           <t>السياق الدائم</t>
         </is>
       </c>
-      <c r="B11" s="54" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>docs/operations/control/context.md</t>
         </is>
       </c>
-      <c r="C11" s="54" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>الخطة والأدوار ومصادر السلطة</t>
         </is>
@@ -6691,7 +6723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6945,7 +6977,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -6963,7 +6995,34 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>انتظار CI على PR #197 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
+          <t>لا إجراء إضافي؛ الموجة 2 مدموجة ومتحققة على main. الموجة 3 في WS-166 من رأس main المتحقق نفسه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WS-166</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CLAIMED</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>stage-2/ops-004-planned-cost</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>OPS-004</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>تنفيذ قارئ التكلفة/الكمية المخططتين للقوالب (بلا أي كتابة) مع اختبارات مركزة ثم PR.</t>
         </is>
       </c>
     </row>
@@ -6981,7 +7040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7463,6 +7522,54 @@
           <t>https://github.com/Qays7753/Micro/pull/196
 reports/agent-report/2026-09-20_stage-2-ops-001-due-dates/report.md
 https://github.com/Qays7753/Micro/commit/bf24bdbfe653e9f7cf8f14f93af9fe6019bd1cb6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>OPS-005</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>سطح قادم موحد للدفعات والتحصيلات والطلبات والالتزامات</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>18368558b6df0dfbc1b1910e961d1504e9e460fb</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Micro/pull/197
+reports/agent-report/2026-09-20_stage-2-ops-005-006-upcoming-aging/report.md
+https://github.com/Qays7753/Micro/commit/18368558b6df0dfbc1b1910e961d1504e9e460fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>OPS-006</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>تقادم ديون مبسط قبل الشرائح المتقدمة</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>18368558b6df0dfbc1b1910e961d1504e9e460fb</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Micro/pull/197
+reports/agent-report/2026-09-20_stage-2-ops-005-006-upcoming-aging/report.md
+https://github.com/Qays7753/Micro/commit/18368558b6df0dfbc1b1910e961d1504e9e460fb</t>
         </is>
       </c>
     </row>
@@ -8561,7 +8668,7 @@
       </c>
       <c r="B16" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="C16" s="54" t="inlineStr">
@@ -8593,7 +8700,7 @@
       </c>
       <c r="B17" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C17" s="54" t="inlineStr">
@@ -8625,7 +8732,7 @@
       </c>
       <c r="B18" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C18" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): Stage 2 Wave 3 IN_REVIEW — PR #198, execution report, QA record, current-state §50
OPS-004 and WS-166 move to IN_REVIEW (actor pr:198). Report + test-results
under reports/agent-report/2026-09-20_stage-2-ops-004-planned-cost/. QA
record under docs/quality/stage-2-ops-004-qa-2026-09-20.md. Reports index +
README runs row. Views/Excel/meta regenerated and validated.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2086,7 +2086,7 @@
       </c>
       <c r="D23" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E23" s="54" t="inlineStr">
@@ -2132,7 +2132,7 @@
       <c r="M23" s="54" t="inlineStr"/>
       <c r="N23" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ الموجة 3 قيد التنفيذ داخل WS-166 على فرع stage-2/ops-004-planned-cost؛ بعد اكتمال الاختبارات وPR تنتقل إلى IN_REVIEW.</t>
+          <t>PR #198 مفتوح للموجة 3؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
         </is>
       </c>
       <c r="O23" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6303,6 +6303,23 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>WS-165→VERIFIED / WS-166 CLAIMED</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>اكتمال الموجة 3 من Stage 2 (OPS-004) وفتح PR #198 — البند وWS-166 إلى IN_REVIEW مع Views/Excel محدثة</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>WS-166 / PR #198</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6399,7 +6416,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -6408,81 +6425,66 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>قيد التنفيذ الآن في Claim نشط</t>
+      <c r="A8" s="53" t="inlineStr">
+        <is>
+          <t>BLOCKED / DEFERRED</t>
+        </is>
+      </c>
+      <c r="B8" s="53" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" s="53" t="inlineStr">
+        <is>
+          <t>بوابة أو دليل مؤجل</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="53" t="inlineStr">
-        <is>
-          <t>BLOCKED / DEFERRED</t>
-        </is>
-      </c>
-      <c r="B9" s="53" t="n">
-        <v>28</v>
-      </c>
-      <c r="C9" s="53" t="inlineStr">
-        <is>
-          <t>بوابة أو دليل مؤجل</t>
+      <c r="A9" s="54" t="inlineStr">
+        <is>
+          <t>main SHA</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>يجب تثبيته قبل أي تنفيذ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="54" t="inlineStr">
         <is>
-          <t>main SHA</t>
+          <t>PRE-PILOT</t>
         </is>
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>يجب تثبيته قبل أي تنفيذ</t>
+          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="54" t="inlineStr">
         <is>
-          <t>PRE-PILOT</t>
+          <t>السياق الدائم</t>
         </is>
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>docs/operations/control/context.md</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
-        <is>
-          <t>لا Pilot قبل تحقق required_items وقرار المالك</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="54" t="inlineStr">
-        <is>
-          <t>السياق الدائم</t>
-        </is>
-      </c>
-      <c r="B12" s="54" t="inlineStr">
-        <is>
-          <t>docs/operations/control/context.md</t>
-        </is>
-      </c>
-      <c r="C12" s="54" t="inlineStr">
         <is>
           <t>الخطة والأدوار ومصادر السلطة</t>
         </is>
@@ -7007,7 +7009,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -7015,6 +7017,9 @@
           <t>stage-2/ops-004-planned-cost</t>
         </is>
       </c>
+      <c r="D12" t="n">
+        <v>198</v>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>OPS-004</t>
@@ -7022,7 +7027,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>تنفيذ قارئ التكلفة/الكمية المخططتين للقوالب (بلا أي كتابة) مع اختبارات مركزة ثم PR.</t>
+          <t>انتظار CI على PR #198 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
         </is>
       </c>
     </row>
@@ -7867,7 +7872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8222,6 +8227,28 @@
       <c r="D18" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-20_stage-2-ops-005-006-upcoming-aging/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>STAGE-2-OPS-004</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>stage 2 wave 3 (OPS-004 template planned cost/quantity read layer)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>OPEN_PR_198_IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-20_stage-2-ops-004-planned-cost/report.md</t>
         </is>
       </c>
     </row>
@@ -8668,7 +8695,7 @@
       </c>
       <c r="B16" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C16" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): close Wave 3 verified on main — Phase 0 tracker reconciliation (OPS-004/WS-166)
OPS-004 IN_REVIEW -> MERGED_UNVERIFIED -> VERIFIED and WS-166
IN_REVIEW -> REVIEW_REQUIRED -> VERIFIED (legal workstream path per
WS-164/WS-165 precedent): PR #198 merged at 0660fdcc510642831419f3cfe8b5b560773e8773
(merge commit), CI green on that exact main SHA (checks + Cloudflare Pages),
evidence reachable from main. current-state §50 now describes Wave 3 as
merged and verified; reports index entry updated; views + Excel meta
regenerated and validated. Documentation-only: no application code, no
schema/export change (35/27), no branch cleanup. Wave 4 (OPS-007+OPS-009)
will open an independent claim from the verified main head only.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2086,7 +2086,7 @@
       </c>
       <c r="D23" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E23" s="54" t="inlineStr">
@@ -2132,7 +2132,7 @@
       <c r="M23" s="54" t="inlineStr"/>
       <c r="N23" s="54" t="inlineStr">
         <is>
-          <t>PR #198 مفتوح للموجة 3؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
+          <t>لا إجراء؛ OPS-004 منفذ ومتحقق على main عند 0660fdcc510642831419f3cfe8b5b560773e8773 (CI أخضر على SHA نفسه). الموجة 4 (OPS-007+OPS-009) تفتح Claim مستقلًا من رأس main المتحقق فقط.</t>
         </is>
       </c>
       <c r="O23" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6320,6 +6320,23 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>WS-166 / PR #198</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>إغلاق Phase 0: دمج PR #198 عند 0660fdcc ونجاح CI عليه؛ OPS-004 وWS-166 -&gt; VERIFIED (مصالحة ما بعد الدمج بلا تغيير كود)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>OPS-004→VERIFIED / WS-166→VERIFIED / PR #198 0660fdcc</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6418,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6416,7 +6433,7 @@
         </is>
       </c>
       <c r="B7" s="54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="54" t="inlineStr">
         <is>
@@ -7009,7 +7026,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -7027,7 +7044,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>انتظار CI على PR #198 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
+          <t>لا إجراء إضافي؛ الموجة 3 مدموجة ومتحققة على main. الموجة 4 (OPS-007+OPS-009) تفتح Claim مستقلًا من رأس main المتحقق نفسه.</t>
         </is>
       </c>
     </row>
@@ -7045,7 +7062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7575,6 +7592,30 @@
           <t>https://github.com/Qays7753/Micro/pull/197
 reports/agent-report/2026-09-20_stage-2-ops-005-006-upcoming-aging/report.md
 https://github.com/Qays7753/Micro/commit/18368558b6df0dfbc1b1910e961d1504e9e460fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>OPS-004</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ربط القوالب بالتكلفة المخططة دون استهلاك فعلي</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>0660fdcc510642831419f3cfe8b5b560773e8773</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Micro/pull/198
+reports/agent-report/2026-09-20_stage-2-ops-004-planned-cost/report.md
+https://github.com/Qays7753/Micro/commit/0660fdcc510642831419f3cfe8b5b560773e8773</t>
         </is>
       </c>
     </row>
@@ -8243,7 +8284,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OPEN_PR_198_IN_REVIEW</t>
+          <t>MERGED_VERIFIED_MAIN_0660FDCC</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): Stage 2 Wave 4 IN_REVIEW — PR #200, execution report, QA record, current-state §51
OPS-007/OPS-009 and WS-167 -> IN_REVIEW (pr:200) with full history;
reports index + agent-report README row; QA record
docs/quality/stage-2-ops-007-009-qa-2026-09-21.md; current-state §51.
Views/Excel/meta regenerated and validated; full pnpm check re-run after
guarded-file changes: EXIT 0 (404+1674 tests, budget 615,929/146,588).
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1691,7 +1691,7 @@
       </c>
       <c r="D18" s="54" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E18" s="54" t="inlineStr">
@@ -1737,7 +1737,7 @@
       <c r="M18" s="54" t="inlineStr"/>
       <c r="N18" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ ضمن WS-167: إغلاق فجوات صدق المقارنة وإثبات حتمية اللقطة، ثم PR.</t>
+          <t>PR #200 مفتوح للموجة 4؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
         </is>
       </c>
       <c r="O18" s="54" t="inlineStr"/>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="D25" s="54" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E25" s="54" t="inlineStr">
@@ -2290,7 +2290,7 @@
       <c r="M25" s="54" t="inlineStr"/>
       <c r="N25" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ ضمن WS-167: إغلاق فجوات صدق المقارنة وإثبات حتمية اللقطة، ثم PR.</t>
+          <t>PR #200 مفتوح للموجة 4؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
         </is>
       </c>
       <c r="O25" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6354,6 +6354,23 @@
       <c r="C22" t="inlineStr">
         <is>
           <t>WS-167 CLAIM / PR #199 da958893</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>اكتمال الموجة 4 من Stage 2 (OPS-007+OPS-009): إعلان سبب المراجعة ودليل حتمية اللقطة؛ فتح PR #200</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>WS-167 / PR #200</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7090,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -7081,10 +7098,8 @@
           <t>stage-2/completion-remaining</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D13" t="n">
+        <v>200</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -7093,7 +7108,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>تنفيذ ضمن WS-167: إغلاق فجوات صدق المقارنة وإثبات حتمية اللقطة، ثم PR.</t>
+          <t>انتظار CI على PR #200 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
         </is>
       </c>
     </row>
@@ -7962,7 +7977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8339,6 +8354,28 @@
       <c r="D19" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-20_stage-2-ops-004-planned-cost/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>STAGE-2-OPS-007-009</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>stage 2 wave 4 (OPS-007 comparison review-reason honesty + OPS-009 Cost Snapshot immutability evidence)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>OPEN_PR_200_IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-21_stage-2-ops-007-009-comparison-honesty/report.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(operations): close Wave 4 verified on main + claim WS-168 for Wave 5 (OPS-008)
OPS-007/OPS-009 and WS-167 -> VERIFIED: PR #200 merged at 8986385 (merge
commit), CI green on that exact main SHA (checks + Cloudflare Pages),
evidence reachable from main. OPS-008 -> IN_PROGRESS inside new claim
WS-168 (branch stage-2/completion-remaining, base 8986385). Single
closure+claim commit avoids the transient active-overlap error.
Views/Excel/meta regenerated and validated.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -1691,7 +1691,7 @@
       </c>
       <c r="D18" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E18" s="54" t="inlineStr">
@@ -1737,7 +1737,7 @@
       <c r="M18" s="54" t="inlineStr"/>
       <c r="N18" s="54" t="inlineStr">
         <is>
-          <t>PR #200 مفتوح للموجة 4؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
+          <t>لا إجراء؛ منفذ ومتحقق على main عند 8986385 (CI أخضر على SHA نفسه). الموجة 5 (OPS-008) تفتح Claim مستقلًا.</t>
         </is>
       </c>
       <c r="O18" s="54" t="inlineStr"/>
@@ -2244,7 +2244,7 @@
       </c>
       <c r="D25" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E25" s="54" t="inlineStr">
@@ -2290,7 +2290,7 @@
       <c r="M25" s="54" t="inlineStr"/>
       <c r="N25" s="54" t="inlineStr">
         <is>
-          <t>PR #200 مفتوح للموجة 4؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
+          <t>لا إجراء؛ منفذ ومتحقق على main عند 8986385 (CI أخضر على SHA نفسه). الموجة 5 (OPS-008) تفتح Claim مستقلًا.</t>
         </is>
       </c>
       <c r="O25" s="54" t="inlineStr"/>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="D26" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>CLAIMED</t>
         </is>
       </c>
       <c r="E26" s="54" t="inlineStr">
@@ -2369,7 +2369,7 @@
       <c r="M26" s="54" t="inlineStr"/>
       <c r="N26" s="54" t="inlineStr">
         <is>
-          <t>انتظر اعتماد CTRL-001 وCTRL-002 ثم أنشئ Workstream claim مستقلًا عند تحقق الاعتماديات.</t>
+          <t>تنفيذ ضمن WS-168: إغلاق فجوات صدق مقارنة الوقت، ثم PR.</t>
         </is>
       </c>
       <c r="O26" s="54" t="inlineStr"/>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="Q26" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6371,6 +6371,40 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>WS-167 / PR #200</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>دمج الموجة 4 (PR #200) عند 8986385 ونجاح CI عليه؛ OPS-007/OPS-009/WS-167 -&gt; VERIFIED</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>WS-167→VERIFIED / PR #200 8986385</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>فتح Claim الموجة 5 (OPS-008 — صدق مقارنة الوقت) ضمن WS-168 من رأس main المتحقق</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>WS-168 CLAIM</t>
         </is>
       </c>
     </row>
@@ -6452,7 +6486,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6776,7 +6810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7090,7 +7124,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -7108,7 +7142,39 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>انتظار CI على PR #200 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
+          <t>لا إجراء إضافي؛ الموجة 4 مدموجة ومتحققة على main. الموجة 5 (OPS-008) تفتح Claim مستقلًا.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WS-168</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CLAIMED</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>stage-2/completion-remaining</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>OPS-008</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>تنفيذ إغلاق فجوات صدق مقارنة الوقت ثم PR.</t>
         </is>
       </c>
     </row>
@@ -7126,7 +7192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7680,6 +7746,54 @@
           <t>https://github.com/Qays7753/Micro/pull/198
 reports/agent-report/2026-09-20_stage-2-ops-004-planned-cost/report.md
 https://github.com/Qays7753/Micro/commit/0660fdcc510642831419f3cfe8b5b560773e8773</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>OPS-007</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>مقارنة التكلفة المخططة بالمستهلكة والفرق</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>8986385fcab1e1ee38c376d938f2475b6ab1c86c</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Micro/pull/200
+reports/agent-report/2026-09-21_stage-2-ops-007-009-comparison-honesty/report.md
+https://github.com/Qays7753/Micro/commit/8986385fcab1e1ee38c376d938f2475b6ab1c86c</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>OPS-009</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>حماية Cost Snapshot وإعلان النتيجة النهائية أو التقديرية</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>8986385fcab1e1ee38c376d938f2475b6ab1c86c</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Micro/pull/200
+reports/agent-report/2026-09-21_stage-2-ops-007-009-comparison-honesty/report.md
+https://github.com/Qays7753/Micro/commit/8986385fcab1e1ee38c376d938f2475b6ab1c86c</t>
         </is>
       </c>
     </row>
@@ -8370,7 +8484,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>OPEN_PR_200_IN_REVIEW</t>
+          <t>MERGED_VERIFIED_MAIN_8986385</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): Stage 2 Wave 5 IN_REVIEW — PR #201, execution report, QA record, current-state §52
OPS-008 and WS-168 -> IN_REVIEW (pr:201) with full history; reports
index + agent-report README row; QA record
docs/quality/stage-2-ops-008-qa-2026-09-21.md; current-state §52.
Views/Excel/meta regenerated and validated; full pnpm check re-run after
guarded-file changes: EXIT 0.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2323,7 +2323,7 @@
       </c>
       <c r="D26" s="54" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E26" s="54" t="inlineStr">
@@ -2369,7 +2369,7 @@
       <c r="M26" s="54" t="inlineStr"/>
       <c r="N26" s="54" t="inlineStr">
         <is>
-          <t>تنفيذ ضمن WS-168: إغلاق فجوات صدق مقارنة الوقت، ثم PR.</t>
+          <t>PR #201 مفتوح للموجة 5؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
         </is>
       </c>
       <c r="O26" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6405,6 +6405,23 @@
       <c r="C25" t="inlineStr">
         <is>
           <t>WS-168 CLAIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>اكتمال الموجة 5 من Stage 2 (OPS-008): السبب الصادق من مصدر الوقت؛ فتح PR #201</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>WS-168 / PR #201</t>
         </is>
       </c>
     </row>
@@ -7154,7 +7171,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CLAIMED</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -7162,10 +7179,8 @@
           <t>stage-2/completion-remaining</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="D14" t="n">
+        <v>201</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -7174,7 +7189,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>تنفيذ إغلاق فجوات صدق مقارنة الوقت ثم PR.</t>
+          <t>انتظار CI على PR #201 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
         </is>
       </c>
     </row>
@@ -8091,7 +8106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8490,6 +8505,28 @@
       <c r="D20" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-21_stage-2-ops-007-009-comparison-honesty/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>STAGE-2-OPS-008</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>stage 2 wave 5 (OPS-008 honest time-comparison cause from its time source)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>OPEN_PR_201_IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-21_stage-2-ops-008-time-honesty/report.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(operations): Stage 2 Wave 6 IN_REVIEW — PR #202, execution report, QA record, current-state §53
Wave 5 closed VERIFIED on main (OPS-008/WS-168 at 771db4e, CI green on the
exact merge SHA). WS-169 claim recorded with the wave documentation (no
other active claims existed during execution on the dedicated branch).
OPS-002 -> IN_REVIEW (pr:202). Views/Excel/meta regenerated and validated;
full pnpm check re-run after guarded-file changes: EXIT 0.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -2007,7 +2007,7 @@
       </c>
       <c r="D22" s="54" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="E22" s="54" t="inlineStr">
@@ -2053,7 +2053,7 @@
       <c r="M22" s="54" t="inlineStr"/>
       <c r="N22" s="54" t="inlineStr">
         <is>
-          <t>تحقق من الاعتماديات (CTRL-001) ثم أنشئ Workstream claim قبل التنفيذ.</t>
+          <t>PR #202 مفتوح للموجة 6؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED.</t>
         </is>
       </c>
       <c r="O22" s="54" t="inlineStr"/>
@@ -2064,7 +2064,7 @@
       </c>
       <c r="Q22" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="D26" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E26" s="54" t="inlineStr">
@@ -2369,7 +2369,7 @@
       <c r="M26" s="54" t="inlineStr"/>
       <c r="N26" s="54" t="inlineStr">
         <is>
-          <t>PR #201 مفتوح للموجة 5؛ بعد نجاح CI والدمج تنتقل إلى MERGED_UNVERIFIED ثم VERIFIED بتحقق SHA الدمج نفسه على origin/main.</t>
+          <t>لا إجراء؛ منفذ ومتحقق على main عند 771db4e (CI أخضر على SHA نفسه).</t>
         </is>
       </c>
       <c r="O26" s="54" t="inlineStr"/>
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6422,6 +6422,23 @@
       <c r="C26" t="inlineStr">
         <is>
           <t>WS-168 / PR #201</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>دمج الموجة 5 (PR #201) عند 771db4e ونجاح CI؛ OPS-008/WS-168 -&gt; VERIFIED؛ Claim الموجة 6 (OPS-002) ضمن WS-169 وفتح PR #202</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>WS-168→VERIFIED / WS-169 / PR #202</t>
         </is>
       </c>
     </row>
@@ -6503,7 +6520,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6827,7 +6844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7171,7 +7188,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -7189,7 +7206,37 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>انتظار CI على PR #201 ثم الدمج (مصرّح به لهذه الموجة) والتحقق على main قبل إغلاق الموجة.</t>
+          <t>لا إجراء إضافي؛ الموجة 5 مدموجة ومتحققة على main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WS-169</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>stage-2/completion-remaining</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>202</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>OPS-002</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>انتظار CI على PR #202 ثم الدمج (مصرّح به) والتحقق على main.</t>
         </is>
       </c>
     </row>
@@ -7207,7 +7254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -7809,6 +7856,30 @@
           <t>https://github.com/Qays7753/Micro/pull/200
 reports/agent-report/2026-09-21_stage-2-ops-007-009-comparison-honesty/report.md
 https://github.com/Qays7753/Micro/commit/8986385fcab1e1ee38c376d938f2475b6ab1c86c</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>OPS-008</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>الوقت الفعلي مقابل المخطط</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>771db4e75b90ab0806b72efd39742e6d2516c94e</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://github.com/Qays7753/Micro/pull/201
+reports/agent-report/2026-09-21_stage-2-ops-008-time-honesty/report.md
+https://github.com/Qays7753/Micro/commit/771db4e75b90ab0806b72efd39742e6d2516c94e</t>
         </is>
       </c>
     </row>
@@ -8106,7 +8177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8521,12 +8592,34 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>OPEN_PR_201_IN_REVIEW</t>
+          <t>MERGED_VERIFIED_MAIN_771DB4E</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-21_stage-2-ops-008-time-honesty/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>STAGE-2-OPS-002</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>stage 2 wave 6 (OPS-002 honest low-stock alerts on optional per-material thresholds)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>OPEN_PR_202_IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-21_stage-2-ops-002-low-stock-alerts/report.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(operations): Stage 2 final closure — unified execution report + reports-index reconciliation
Unified execution report for the whole session (baseline 0660fdc -> final
head e493122 across five merged+verified PRs #199-#203): per-phase shared-
agent usage, exact commands/exit codes, CI conclusions on every merge SHA,
rollback boundaries, schema/export impact (35/27 unchanged throughout),
forbidden operations not performed, and the single open item — OPS-003
DEFERRED with owner decisions D1-D6. Reports-index reconciliation (stale
pre-session entries -> merged/verified statuses); current-state §55;
views/Excel/meta regenerated; full pnpm check re-run after guarded-file
changes: EXIT 0.
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -6009,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6456,6 +6456,23 @@
       <c r="C28" t="inlineStr">
         <is>
           <t>WS-169→VERIFIED / WS-170 DEFERRED / OPS-003 قرارات د١–د٦</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>إغلاق جلسة استكمال Stage 2: التقرير الموحد + مصالحة فهرس التقارير + بقاء OPS-003 (د١–د٦) البند الوحيد المفتوح</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>STAGE-2-FINAL-EXECUTION / OPS-003 D1-D6</t>
         </is>
       </c>
     </row>
@@ -8250,7 +8267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8533,7 +8550,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>OPEN_PR_190_IN_REVIEW</t>
+          <t>MERGED</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8555,7 +8572,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>OPEN_PR_191_IN_REVIEW</t>
+          <t>MERGED</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -8577,7 +8594,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>OPEN_PR_196_IN_REVIEW</t>
+          <t>MERGED_VERIFIED_MAIN_BF24BDB</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -8599,7 +8616,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>OPEN_PR_197_IN_REVIEW</t>
+          <t>MERGED_VERIFIED_MAIN_1836855</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -8709,12 +8726,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DOC_ONLY_PR_PENDING</t>
+          <t>MERGED_DOC_ONLY_E493122</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-21_stage-2-ops-003-deferral-decision/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>STAGE-2-FINAL-EXECUTION</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Stage 2 completion session — unified execution report (Phase 0 + Waves 4-7)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>OPEN_PR_PENDING</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-21_stage-2-final-execution-report/report.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(operations): OPS-003/WS-171 IN_REVIEW — implementation report, test results, QA record, current-state §56, PR #205 evidence
- reports/agent-report/2026-09-21_ops-003-recurring-expense-system/{report,test-results}.md:
  full waves A–E record (baseline 16b4c8af, five-agent review + 8 design adjustments, per-wave
  files/decisions, acceptance-risk coverage matrix, rollback boundary, executed/forbidden writes)
- docs/quality/ops-003-recurring-expense-qa-2026-09-21.md: live browser QA NOT_EXECUTED (no
  browser in environment); automated DOM coverage 18 tests; required live-QA checklist for review
- current-state §56: honest branch state — IN_REVIEW at PR #205, no VERIFIED before merge+verify
- tracker: OPS-003 + WS-171 IN_PROGRESS → IN_REVIEW (legal), evidence appended, views/xlsx/meta
  regenerated, validate.py valid, operations-control tests 8/8
- next: owner merge decision on PR #205, then post-merge verification on main
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -3903,13 +3903,11 @@
       </c>
       <c r="D46" s="54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="E46" s="54" t="inlineStr">
-        <is>
-          <t>FIX_BEFORE_PILOT</t>
-        </is>
+          <t>IN_REVIEW</t>
+        </is>
+      </c>
+      <c r="E46" s="54" t="n">
+        <v>205</v>
       </c>
       <c r="F46" s="54" t="inlineStr">
         <is>
@@ -3953,7 +3951,7 @@
       </c>
       <c r="N46" s="54" t="inlineStr">
         <is>
-          <t>إكمال موجات D (واجهة عربية RTL) وE (تحقق كامل + PR) على الفرع المخصص ثم قرار دمج المالك.</t>
+          <t>قرار دمج المالك لـPR #205 ثم التحقق على main وإغلاق VERIFIED بأدلة ما بعد الدمج.</t>
         </is>
       </c>
       <c r="O46" s="54" t="inlineStr">
@@ -6009,7 +6007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6490,6 +6488,23 @@
       <c r="C30" t="inlineStr">
         <is>
           <t>WS-171 IN_PROGRESS (waves A–C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>OPS-003/WS-171 IN_PROGRESS → IN_REVIEW: الموجات A–E منفذة على الفرع المخصص (عقد ٤١ + دومين + تخزين ٣٦/٢٨ + خدمة التأكيد الحتمي + واجهة RTL)؛ pnpm check EXIT 0؛ PR #205 مفتوح</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>WS-171 IN_REVIEW / PR #205</t>
         </is>
       </c>
     </row>
@@ -7331,7 +7346,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>IN_REVIEW</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -7341,7 +7356,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>205</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -7351,7 +7366,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>الموجة D (واجهة عربية RTL للقائمة/التفصيل/المراجعة/التأكيد) ثم الموجة E (pnpm check كاملًا + Tracker IN_REVIEW + تقرير + PR) والتوقف عند PR-ready لقرار دمج المالك.</t>
+          <t>انتظار CI على رأس PR #205 ثم قرار دمج المالك ثم إغلاق VERIFIED بأدلة ما بعد الدمج.</t>
         </is>
       </c>
     </row>
@@ -8316,7 +8331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8803,6 +8818,28 @@
       <c r="D24" t="inlineStr">
         <is>
           <t>reports/agent-report/2026-09-21_stage-2-final-execution-report/report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>OPS-003 Complete Controlled Implementation (waves A–E)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-21_ops-003-recurring-expense-system/report.md</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PR #205 open — awaiting owner merge decision</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(operations): close OPS-003 after main verification
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -3903,7 +3903,7 @@
       </c>
       <c r="D46" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E46" s="54" t="n">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="N46" s="54" t="inlineStr">
         <is>
-          <t>قرار دمج المالك لـPR #205 ثم التحقق على main وإغلاق VERIFIED بأدلة ما بعد الدمج.</t>
+          <t>لا إجراء تنفيذي إضافي لهذا البند؛ تبقى PRE-PILOT محجوبة حتى تحقق بقية المتطلبات وقرار المالك، ولا يبدأ Pilot من هذا السجل.</t>
         </is>
       </c>
       <c r="O46" s="54" t="inlineStr">
@@ -6007,7 +6007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6505,6 +6505,23 @@
       <c r="C31" t="inlineStr">
         <is>
           <t>WS-171 IN_REVIEW / PR #205</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>دمج PR #205 وتحقق CI وCloudflare على main؛ إغلاق OPS-003 وWS-171 إلى VERIFIED مع إبقاء PRE-PILOT وPilot محجوبين</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>OPS-003 / WS-171 / PR #205</t>
         </is>
       </c>
     </row>
@@ -6586,7 +6603,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6616,7 +6633,7 @@
         </is>
       </c>
       <c r="B8" s="53" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" s="53" t="inlineStr">
         <is>
@@ -6632,7 +6649,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+          <t>4b374edb325f6331864a5f10111ec620f7a2aee0</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
@@ -7346,7 +7363,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -7354,10 +7371,8 @@
           <t>ops-003/recurring-expense-system</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>205</t>
-        </is>
+      <c r="D17" t="n">
+        <v>205</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -7366,7 +7381,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>انتظار CI على رأس PR #205 ثم قرار دمج المالك ثم إغلاق VERIFIED بأدلة ما بعد الدمج.</t>
+          <t>لا إجراء تنفيذي إضافي؛ OPS-003 مدموج ومتحقق على main. تبقى PRE-PILOT محجوبة ببقية المتطلبات، ولا يبدأ Pilot من هذا السجل.</t>
         </is>
       </c>
     </row>
@@ -7384,7 +7399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8034,6 +8049,41 @@
           <t>https://github.com/Qays7753/Micro/pull/202
 reports/agent-report/2026-09-21_stage-2-ops-002-low-stock-alerts/report.md
 https://github.com/Qays7753/Micro/commit/ee0bcee7b2490a5977171de919496cea26252970</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>OPS-003</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>المصروفات المتكررة المحلية</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>4b374edb325f6331864a5f10111ec620f7a2aee0</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-21_stage-2-ops-003-deferral-decision/report.md
+docs/contracts/05-financial-p0-policies.md
+docs/contracts/06-financial-event-prototype-contract.md
+src/domain/financial-event/policies.ts
+src/domain/shared/businessTime.ts
+docs/contracts/41-recurring-expense-reminders-contract.md
+reports/agent-report/2026-09-21_ops-003-recurring-expense-system/report.md
+reports/agent-report/2026-09-21_ops-003-recurring-expense-system/test-results.md
+docs/quality/ops-003-recurring-expense-qa-2026-09-21.md
+https://github.com/Qays7753/Micro/pull/205
+https://github.com/Qays7753/Micro/commit/4b374edb325f6331864a5f10111ec620f7a2aee0
+https://github.com/Qays7753/Micro/actions/runs/35600599024/job/106335505937
+https://dash.cloudflare.com/?to=/663413a9a3389b95eb5d970c6a7ef9d5/pages/view/micro-prototype/16b28a47-f030-4ee1-9e01-4d59b7292f5f
+docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
@@ -9254,7 +9304,7 @@
       </c>
       <c r="B15" s="54" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C15" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs(operations): close OPS-003 after main verification (#206)
Co-authored-by: Qays7753 <2.14180459e+08+Qays7753@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -3903,7 +3903,7 @@
       </c>
       <c r="D46" s="54" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="E46" s="54" t="n">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="N46" s="54" t="inlineStr">
         <is>
-          <t>قرار دمج المالك لـPR #205 ثم التحقق على main وإغلاق VERIFIED بأدلة ما بعد الدمج.</t>
+          <t>لا إجراء تنفيذي إضافي لهذا البند؛ تبقى PRE-PILOT محجوبة حتى تحقق بقية المتطلبات وقرار المالك، ولا يبدأ Pilot من هذا السجل.</t>
         </is>
       </c>
       <c r="O46" s="54" t="inlineStr">
@@ -6007,7 +6007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6505,6 +6505,23 @@
       <c r="C31" t="inlineStr">
         <is>
           <t>WS-171 IN_REVIEW / PR #205</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>دمج PR #205 وتحقق CI وCloudflare على main؛ إغلاق OPS-003 وWS-171 إلى VERIFIED مع إبقاء PRE-PILOT وPilot محجوبين</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>OPS-003 / WS-171 / PR #205</t>
         </is>
       </c>
     </row>
@@ -6586,7 +6603,7 @@
         </is>
       </c>
       <c r="B6" s="54" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" s="54" t="inlineStr">
         <is>
@@ -6616,7 +6633,7 @@
         </is>
       </c>
       <c r="B8" s="53" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C8" s="53" t="inlineStr">
         <is>
@@ -6632,7 +6649,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>0187f475d6bb0cda54d33fee9cc3c0faeb2784f8</t>
+          <t>4b374edb325f6331864a5f10111ec620f7a2aee0</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
@@ -7346,7 +7363,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IN_REVIEW</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -7354,10 +7371,8 @@
           <t>ops-003/recurring-expense-system</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>205</t>
-        </is>
+      <c r="D17" t="n">
+        <v>205</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -7366,7 +7381,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>انتظار CI على رأس PR #205 ثم قرار دمج المالك ثم إغلاق VERIFIED بأدلة ما بعد الدمج.</t>
+          <t>لا إجراء تنفيذي إضافي؛ OPS-003 مدموج ومتحقق على main. تبقى PRE-PILOT محجوبة ببقية المتطلبات، ولا يبدأ Pilot من هذا السجل.</t>
         </is>
       </c>
     </row>
@@ -7384,7 +7399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8034,6 +8049,41 @@
           <t>https://github.com/Qays7753/Micro/pull/202
 reports/agent-report/2026-09-21_stage-2-ops-002-low-stock-alerts/report.md
 https://github.com/Qays7753/Micro/commit/ee0bcee7b2490a5977171de919496cea26252970</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>OPS-003</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>المصروفات المتكررة المحلية</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>4b374edb325f6331864a5f10111ec620f7a2aee0</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>reports/agent-report/2026-09-21_stage-2-ops-003-deferral-decision/report.md
+docs/contracts/05-financial-p0-policies.md
+docs/contracts/06-financial-event-prototype-contract.md
+src/domain/financial-event/policies.ts
+src/domain/shared/businessTime.ts
+docs/contracts/41-recurring-expense-reminders-contract.md
+reports/agent-report/2026-09-21_ops-003-recurring-expense-system/report.md
+reports/agent-report/2026-09-21_ops-003-recurring-expense-system/test-results.md
+docs/quality/ops-003-recurring-expense-qa-2026-09-21.md
+https://github.com/Qays7753/Micro/pull/205
+https://github.com/Qays7753/Micro/commit/4b374edb325f6331864a5f10111ec620f7a2aee0
+https://github.com/Qays7753/Micro/actions/runs/35600599024/job/106335505937
+https://dash.cloudflare.com/?to=/663413a9a3389b95eb5d970c6a7ef9d5/pages/view/micro-prototype/16b28a47-f030-4ee1-9e01-4d59b7292f5f
+docs/operations/current-state.md</t>
         </is>
       </c>
     </row>
@@ -9254,7 +9304,7 @@
       </c>
       <c r="B15" s="54" t="inlineStr">
         <is>
-          <t>DEFERRED</t>
+          <t>VERIFIED</t>
         </is>
       </c>
       <c r="C15" s="54" t="inlineStr">

</xml_diff>

<commit_message>
docs: close UI V2 Phase 1 mapping gate
</commit_message>
<xml_diff>
--- a/docs/operations/control/generated/MASTER-TRACKER.xlsx
+++ b/docs/operations/control/generated/MASTER-TRACKER.xlsx
@@ -3217,12 +3217,12 @@
       </c>
       <c r="M37" s="54" t="inlineStr">
         <is>
-          <t>اعتماد الاتجاه البصري النهائي ونتائج Benchmark قبل التنفيذ.</t>
+          <t>Phase 0/1 owner direction: Bold Modular V2 owns visual direction; Micro owns functionality, data, financial contracts, and operational behavior; Documents is reviewed by topic/revision. #D97757 remains identity; #A94630 is a future solid-action direction only. Preserve Micro state semantics, vocabulary, two-decimal money contract, due-today neutrality, and numeric IBM Plex Mono until verified. V2 Shell, عرض الكل, and OVR-SNAPSHOT-ALL are later waves. No cap raise, runtime/token/Documents write, bulk move, or broad refactor in closeout.</t>
         </is>
       </c>
       <c r="N37" s="54" t="inlineStr">
         <is>
-          <t>اعتمد الاتجاه وBenchmark بعد استقرار الوظائف، ثم افتح Claim UI/UX؛ يبقى مطلوبًا قبل Pilot.</t>
+          <t>Phase 2: create a Claim from current origin/main; inventory consumers, then implement only the approved foundations/first-screen slice. No bulk move, competing token source, financial/wording change, or VERIFIED before merge and main evidence.</t>
         </is>
       </c>
       <c r="O37" s="54" t="inlineStr">
@@ -3237,7 +3237,7 @@
       </c>
       <c r="Q37" s="54" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -6007,7 +6007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6522,6 +6522,23 @@
       <c r="C32" t="inlineStr">
         <is>
           <t>OPS-003 / WS-171 / PR #205</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>إغلاق خريطة V2-to-Micro وقرارات OD-01..OD-12؛ إبقاء UX-001 مؤجلًا وتحديد Phase 2 كالتالي</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>D-039 / UX-001 / Phase 1</t>
         </is>
       </c>
     </row>
@@ -6649,7 +6666,7 @@
       </c>
       <c r="B9" s="54" t="inlineStr">
         <is>
-          <t>4b374edb325f6331864a5f10111ec620f7a2aee0</t>
+          <t>4e1bab9198023cf76bf1ebd5e9481d898a95700e</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
@@ -6829,12 +6846,12 @@
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>إعادة تصميم UI/UX النهائية</t>
+          <t>UI/UX V2 Phase 1 ثم التنفيذ المرحلي</t>
         </is>
       </c>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>UX-001؛ اتجاه معتمد ورحلات RTL ووصول</t>
+          <t>Phase 1 mapping وOD-01..OD-12 مغلقة؛ Phase 2 تبدأ من main بعد Claim وأثر مستهلكين؛ UX-001 يبقى Gate قبل Pilot</t>
         </is>
       </c>
     </row>
@@ -8101,7 +8118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8187,6 +8204,33 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>UX-001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>إعادة تصميم UI وUX جذرية</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Phase 0/1 owner direction: Bold Modular V2 owns visual direction; Micro owns functionality, data, financial contracts, and operational behavior; Documents is reviewed by topic/revision. #D97757 remains identity; #A94630 is a future solid-action direction only. Preserve Micro state semantics, vocabulary, two-decimal money contract, due-today neutrality, and numeric IBM Plex Mono until verified. V2 Shell, عرض الكل, and OVR-SNAPSHOT-ALL are later waves. No cap raise, runtime/token/Documents write, bulk move, or broad refactor in closeout.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Phase 2: create a Claim from current origin/main; inventory consumers, then implement only the approved foundations/first-screen slice. No bulk move, competing token source, financial/wording change, or VERIFIED before merge and main evidence.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:D2"/>
@@ -8201,7 +8245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8364,6 +8408,18 @@
       <c r="B15" s="54" t="inlineStr">
         <is>
           <t>مصفوفة أدلة 49/46 ومصالحة عقد الزمن القديم مع تنفيذ Wave 4.4؛ CTRL-002</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="54" t="inlineStr">
+        <is>
+          <t>UI/UX V2 Phase 1</t>
+        </is>
+      </c>
+      <c r="B16" s="54" t="inlineStr">
+        <is>
+          <t>Phase 0/1 owner direction: Bold Modular V2 owns visual direction; Micro owns functionality, data, financial contracts, and operational behavior; Documents is reviewed by topic/revision. #D97757 remains identity; #A94630 is a future solid-action direction only. Preserve Micro state semantics, vocabulary, two-decimal money contract, due-today neutrality, and numeric IBM Plex Mono until verified. V2 Shell, عرض الكل, and OVR-SNAPSHOT-ALL are later waves. No cap raise, runtime/token/Documents write, bulk move, or broad refactor in closeout.</t>
         </is>
       </c>
     </row>

</xml_diff>